<commit_message>
split particiapnts for analysis
</commit_message>
<xml_diff>
--- a/ParticipantData and Labelling.xlsx
+++ b/ParticipantData and Labelling.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Basilio\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Basilio\Documents\Thesis Gigler\squatting_fais\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B9514FD7-D749-463E-8CD7-3AAD0FC77A5D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{77A23979-F699-483B-8DA6-A0AD391786AE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="14020" tabRatio="798" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="10" yWindow="0" windowWidth="25580" windowHeight="13800" tabRatio="798" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Demographics" sheetId="1" r:id="rId1"/>
@@ -643,7 +643,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2888" uniqueCount="576">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2900" uniqueCount="576">
   <si>
     <t>Subject</t>
   </si>
@@ -2467,10 +2467,10 @@
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="3">
     <numFmt numFmtId="164" formatCode="0.0"/>
-    <numFmt numFmtId="166" formatCode="dd/mm/yyyy;@"/>
-    <numFmt numFmtId="167" formatCode="yyyy\-mm\-dd\ h:mm:ss"/>
+    <numFmt numFmtId="165" formatCode="dd/mm/yyyy;@"/>
+    <numFmt numFmtId="166" formatCode="yyyy\-mm\-dd\ h:mm:ss"/>
   </numFmts>
-  <fonts count="13" x14ac:knownFonts="1">
+  <fonts count="15">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -2560,8 +2560,22 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFC00000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="17">
+  <fills count="18">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -2655,6 +2669,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -2917,7 +2937,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="99">
+  <cellXfs count="104">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -3077,22 +3097,22 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="166" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
     <xf numFmtId="14" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="right" vertical="top"/>
     </xf>
-    <xf numFmtId="166" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="right" vertical="top"/>
     </xf>
-    <xf numFmtId="166" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="right" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -3100,18 +3120,27 @@
     </xf>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="17" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="17" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="17" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="123">
-    <dxf>
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="bottom"/>
-    </dxf>
     <dxf>
       <fill>
         <patternFill patternType="solid">
@@ -3631,11 +3660,11 @@
       <alignment horizontal="general" vertical="bottom"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="165" formatCode="m/d/yyyy"/>
+      <numFmt numFmtId="167" formatCode="m/d/yyyy"/>
       <alignment horizontal="general" vertical="bottom"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="165" formatCode="m/d/yyyy"/>
+      <numFmt numFmtId="167" formatCode="m/d/yyyy"/>
     </dxf>
     <dxf>
       <alignment horizontal="general" vertical="bottom"/>
@@ -3684,6 +3713,12 @@
     </dxf>
     <dxf>
       <alignment horizontal="general" vertical="bottom"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="bottom"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <alignment horizontal="general" vertical="bottom"/>
@@ -3754,50 +3789,50 @@
     <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="Sex" totalsRowDxfId="118"/>
     <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="Measured Leg" dataDxfId="117" totalsRowDxfId="116"/>
     <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000005000000}" name="Dominant Leg " totalsRowDxfId="115"/>
-    <tableColumn id="13" xr3:uid="{C9829FE8-EED4-4D6D-A3F4-FE8FBD360404}" name="Squat_used" dataDxfId="0" totalsRowDxfId="1"/>
-    <tableColumn id="30" xr3:uid="{00000000-0010-0000-0000-00001E000000}" name="StrengthData" totalsRowDxfId="114"/>
-    <tableColumn id="27" xr3:uid="{00000000-0010-0000-0000-00001B000000}" name="Alpha angle" totalsRowDxfId="113"/>
-    <tableColumn id="45" xr3:uid="{00000000-0010-0000-0000-00002D000000}" name="Centre edge angle" dataDxfId="112" totalsRowDxfId="111"/>
-    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0000-000006000000}" name="Group" totalsRowDxfId="110"/>
-    <tableColumn id="28" xr3:uid="{00000000-0010-0000-0000-00001C000000}" name="Intramuscular" totalsRowDxfId="109"/>
-    <tableColumn id="25" xr3:uid="{00000000-0010-0000-0000-000019000000}" name="FADIR" totalsRowDxfId="108"/>
-    <tableColumn id="26" xr3:uid="{00000000-0010-0000-0000-00001A000000}" name="FABER" totalsRowDxfId="107"/>
-    <tableColumn id="29" xr3:uid="{00000000-0010-0000-0000-00001D000000}" name="Pain" totalsRowDxfId="106"/>
-    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0000-000007000000}" name="Symptomatic side" totalsRowDxfId="105"/>
-    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0000-000008000000}" name="Duration of Symptoms" totalsRowDxfId="104"/>
-    <tableColumn id="24" xr3:uid="{00000000-0010-0000-0000-000018000000}" name="Birth Date" totalsRowDxfId="103"/>
-    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0000-000009000000}" name="Date" dataDxfId="102" totalsRowDxfId="101"/>
-    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0000-00000A000000}" name="Date_num" totalsRowDxfId="100"/>
-    <tableColumn id="11" xr3:uid="{00000000-0010-0000-0000-00000B000000}" name="Weight" totalsRowDxfId="99"/>
-    <tableColumn id="12" xr3:uid="{00000000-0010-0000-0000-00000C000000}" name="Height" totalsRowDxfId="98"/>
-    <tableColumn id="47" xr3:uid="{00000000-0010-0000-0000-00002F000000}" name="BMI" dataDxfId="97" totalsRowDxfId="96">
+    <tableColumn id="13" xr3:uid="{C9829FE8-EED4-4D6D-A3F4-FE8FBD360404}" name="Squat_used" dataDxfId="114" totalsRowDxfId="113"/>
+    <tableColumn id="30" xr3:uid="{00000000-0010-0000-0000-00001E000000}" name="StrengthData" totalsRowDxfId="112"/>
+    <tableColumn id="27" xr3:uid="{00000000-0010-0000-0000-00001B000000}" name="Alpha angle" totalsRowDxfId="111"/>
+    <tableColumn id="45" xr3:uid="{00000000-0010-0000-0000-00002D000000}" name="Centre edge angle" dataDxfId="110" totalsRowDxfId="109"/>
+    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0000-000006000000}" name="Group" totalsRowDxfId="108"/>
+    <tableColumn id="28" xr3:uid="{00000000-0010-0000-0000-00001C000000}" name="Intramuscular" totalsRowDxfId="107"/>
+    <tableColumn id="25" xr3:uid="{00000000-0010-0000-0000-000019000000}" name="FADIR" totalsRowDxfId="106"/>
+    <tableColumn id="26" xr3:uid="{00000000-0010-0000-0000-00001A000000}" name="FABER" totalsRowDxfId="105"/>
+    <tableColumn id="29" xr3:uid="{00000000-0010-0000-0000-00001D000000}" name="Pain" totalsRowDxfId="104"/>
+    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0000-000007000000}" name="Symptomatic side" totalsRowDxfId="103"/>
+    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0000-000008000000}" name="Duration of Symptoms" totalsRowDxfId="102"/>
+    <tableColumn id="24" xr3:uid="{00000000-0010-0000-0000-000018000000}" name="Birth Date" totalsRowDxfId="101"/>
+    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0000-000009000000}" name="Date" dataDxfId="100" totalsRowDxfId="99"/>
+    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0000-00000A000000}" name="Date_num" totalsRowDxfId="98"/>
+    <tableColumn id="11" xr3:uid="{00000000-0010-0000-0000-00000B000000}" name="Weight" totalsRowDxfId="97"/>
+    <tableColumn id="12" xr3:uid="{00000000-0010-0000-0000-00000C000000}" name="Height" totalsRowDxfId="96"/>
+    <tableColumn id="47" xr3:uid="{00000000-0010-0000-0000-00002F000000}" name="BMI" dataDxfId="95" totalsRowDxfId="94">
       <calculatedColumnFormula>Table1[[#This Row],[Weight]]/((Table1[[#This Row],[Height]]/100)^2)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="31" xr3:uid="{00000000-0010-0000-0000-00001F000000}" name="Current level" dataDxfId="95" totalsRowDxfId="94"/>
-    <tableColumn id="32" xr3:uid="{00000000-0010-0000-0000-000020000000}" name="If you are no longer exercising at the same level, please indicate the reasons" dataDxfId="93" totalsRowDxfId="92"/>
-    <tableColumn id="33" xr3:uid="{00000000-0010-0000-0000-000021000000}" name="Total hours exercise per week" dataDxfId="91" totalsRowDxfId="90"/>
-    <tableColumn id="46" xr3:uid="{00000000-0010-0000-0000-00002E000000}" name="Total min exer per week " dataDxfId="89" totalsRowDxfId="88">
+    <tableColumn id="31" xr3:uid="{00000000-0010-0000-0000-00001F000000}" name="Current level" dataDxfId="93" totalsRowDxfId="92"/>
+    <tableColumn id="32" xr3:uid="{00000000-0010-0000-0000-000020000000}" name="If you are no longer exercising at the same level, please indicate the reasons" dataDxfId="91" totalsRowDxfId="90"/>
+    <tableColumn id="33" xr3:uid="{00000000-0010-0000-0000-000021000000}" name="Total hours exercise per week" dataDxfId="89" totalsRowDxfId="88"/>
+    <tableColumn id="46" xr3:uid="{00000000-0010-0000-0000-00002E000000}" name="Total min exer per week " dataDxfId="87" totalsRowDxfId="86">
       <calculatedColumnFormula>Table1[[#This Row],[Total hours exercise per week]]*60</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="43" xr3:uid="{00000000-0010-0000-0000-00002B000000}" name="Sports" dataDxfId="87" totalsRowDxfId="86"/>
-    <tableColumn id="34" xr3:uid="{00000000-0010-0000-0000-000022000000}" name="Sports Category (based on Nawabi et al. 2014)" dataDxfId="85" totalsRowDxfId="84"/>
-    <tableColumn id="40" xr3:uid="{00000000-0010-0000-0000-000028000000}" name="Total Hours Competetive sport per week" dataDxfId="83" totalsRowDxfId="82"/>
-    <tableColumn id="39" xr3:uid="{00000000-0010-0000-0000-000027000000}" name="Competetive Sport" dataDxfId="81" totalsRowDxfId="80"/>
-    <tableColumn id="35" xr3:uid="{00000000-0010-0000-0000-000023000000}" name="Highest level of competition" dataDxfId="79" totalsRowDxfId="78"/>
-    <tableColumn id="36" xr3:uid="{00000000-0010-0000-0000-000024000000}" name="Sport" dataDxfId="77" totalsRowDxfId="76"/>
-    <tableColumn id="37" xr3:uid="{00000000-0010-0000-0000-000025000000}" name="SumYears" dataDxfId="75" totalsRowDxfId="74"/>
-    <tableColumn id="42" xr3:uid="{00000000-0010-0000-0000-00002A000000}" name="Modified Tagner BEFORE" dataDxfId="73" totalsRowDxfId="72"/>
-    <tableColumn id="41" xr3:uid="{00000000-0010-0000-0000-000029000000}" name="Modified Tagner CURRENT" dataDxfId="71" totalsRowDxfId="70"/>
+    <tableColumn id="43" xr3:uid="{00000000-0010-0000-0000-00002B000000}" name="Sports" dataDxfId="85" totalsRowDxfId="84"/>
+    <tableColumn id="34" xr3:uid="{00000000-0010-0000-0000-000022000000}" name="Sports Category (based on Nawabi et al. 2014)" dataDxfId="83" totalsRowDxfId="82"/>
+    <tableColumn id="40" xr3:uid="{00000000-0010-0000-0000-000028000000}" name="Total Hours Competetive sport per week" dataDxfId="81" totalsRowDxfId="80"/>
+    <tableColumn id="39" xr3:uid="{00000000-0010-0000-0000-000027000000}" name="Competetive Sport" dataDxfId="79" totalsRowDxfId="78"/>
+    <tableColumn id="35" xr3:uid="{00000000-0010-0000-0000-000023000000}" name="Highest level of competition" dataDxfId="77" totalsRowDxfId="76"/>
+    <tableColumn id="36" xr3:uid="{00000000-0010-0000-0000-000024000000}" name="Sport" dataDxfId="75" totalsRowDxfId="74"/>
+    <tableColumn id="37" xr3:uid="{00000000-0010-0000-0000-000025000000}" name="SumYears" dataDxfId="73" totalsRowDxfId="72"/>
+    <tableColumn id="42" xr3:uid="{00000000-0010-0000-0000-00002A000000}" name="Modified Tagner BEFORE" dataDxfId="71" totalsRowDxfId="70"/>
+    <tableColumn id="41" xr3:uid="{00000000-0010-0000-0000-000029000000}" name="Modified Tagner CURRENT" dataDxfId="69" totalsRowDxfId="68"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{00000000-000C-0000-FFFF-FFFF01000000}" name="Table5" displayName="Table5" ref="A1:O23" totalsRowShown="0" headerRowDxfId="69">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{00000000-000C-0000-FFFF-FFFF01000000}" name="Table5" displayName="Table5" ref="A1:O23" totalsRowShown="0" headerRowDxfId="67">
   <autoFilter ref="A1:O23" xr:uid="{00000000-0009-0000-0100-000002000000}"/>
   <tableColumns count="15">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0100-000001000000}" name="Subject" dataDxfId="68"/>
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0100-000001000000}" name="Subject" dataDxfId="66"/>
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0100-000002000000}" name="Joint mobilisation/manipulation"/>
     <tableColumn id="3" xr3:uid="{00000000-0010-0000-0100-000003000000}" name="Stretching"/>
     <tableColumn id="4" xr3:uid="{00000000-0010-0000-0100-000004000000}" name="Strengtheneing"/>
@@ -3818,50 +3853,50 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{00000000-000C-0000-FFFF-FFFF02000000}" name="Table7" displayName="Table7" ref="A2:AJ17" totalsRowShown="0" headerRowDxfId="67" dataDxfId="66">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{00000000-000C-0000-FFFF-FFFF02000000}" name="Table7" displayName="Table7" ref="A2:AJ17" totalsRowShown="0" headerRowDxfId="65" dataDxfId="64">
   <autoFilter ref="A2:AJ17" xr:uid="{00000000-0009-0000-0100-000003000000}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A3:AJ22">
     <sortCondition ref="A2:A22"/>
   </sortState>
   <tableColumns count="36">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0200-000001000000}" name="Subject"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0200-000002000000}" name="Q01 How often does your hip/groin ache?" dataDxfId="65"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0200-000003000000}" name="Q02 How stiff is your hip as a result of sitting/resting during the day?" dataDxfId="64"/>
-    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0200-000004000000}" name="Q03 How difficult is it for you to walk long distances?" dataDxfId="63"/>
-    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0200-000005000000}" name="Q04 How much pain do you have in your hip while sitting?" dataDxfId="62"/>
-    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0200-000006000000}" name="Q05 How much trouble do you have standing on your feet for long periods of time?" dataDxfId="61"/>
-    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0200-000007000000}" name="Q06 How difficult is it for you to get up and down off the floor/ground?" dataDxfId="60"/>
-    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0200-000008000000}" name="Q07 How difficult is it for you to walk on uneven surfaces?" dataDxfId="59"/>
-    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0200-000009000000}" name="Q08 How difficult is it for you to lie on your affected hip side?" dataDxfId="58"/>
-    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0200-00000A000000}" name="Q09 How much trouble do you have with stepping over obstacles?" dataDxfId="57"/>
-    <tableColumn id="11" xr3:uid="{00000000-0010-0000-0200-00000B000000}" name="Q10 How much trouble do you have with climbing up/down stairs?" dataDxfId="56"/>
-    <tableColumn id="12" xr3:uid="{00000000-0010-0000-0200-00000C000000}" name="Q11 How much trouble do you have with rising from a sitting position?" dataDxfId="55"/>
-    <tableColumn id="13" xr3:uid="{00000000-0010-0000-0200-00000D000000}" name="Q12 How much discomfort do you have with taking long strides?" dataDxfId="54"/>
-    <tableColumn id="14" xr3:uid="{00000000-0010-0000-0200-00000E000000}" name="Q13 How much difficulty do you have with getting into and/or out of a car?_x000a_" dataDxfId="53"/>
-    <tableColumn id="15" xr3:uid="{00000000-0010-0000-0200-00000F000000}" name="Q14 How much trouble do you have with grinding, catching or clicking in your hip?" dataDxfId="52"/>
-    <tableColumn id="16" xr3:uid="{00000000-0010-0000-0200-000010000000}" name="Q15 How much difficulty do you have with putting on/taking off socks, stockings or shoes?" dataDxfId="51"/>
-    <tableColumn id="17" xr3:uid="{00000000-0010-0000-0200-000011000000}" name="Q16 Overall, how much pain do you have in your hip/groin?" dataDxfId="50"/>
-    <tableColumn id="18" xr3:uid="{00000000-0010-0000-0200-000012000000}" name="Q17 How concerned are you about your ability to maintain your desired fitness level?" dataDxfId="49"/>
-    <tableColumn id="19" xr3:uid="{00000000-0010-0000-0200-000013000000}" name="Q18 How much pain do you experience in your hip after activity?" dataDxfId="48"/>
-    <tableColumn id="20" xr3:uid="{00000000-0010-0000-0200-000014000000}" name="Q19 How concerned are you that the pain in your hip will increase if you participate in sports or recreational activities?_x000a_" dataDxfId="47"/>
-    <tableColumn id="21" xr3:uid="{00000000-0010-0000-0200-000015000000}" name="Q20 How much has your quality of life deteriorated because you cannot participate in sport/recreational activities?" dataDxfId="46"/>
-    <tableColumn id="22" xr3:uid="{00000000-0010-0000-0200-000016000000}" name="Q21 How concerned are you about cutting/changing direction during your sport or recreational activities?" dataDxfId="45"/>
-    <tableColumn id="23" xr3:uid="{00000000-0010-0000-0200-000017000000}" name="Q22 How much has your performance level decreased in your sport or recreational activities?" dataDxfId="44"/>
-    <tableColumn id="24" xr3:uid="{00000000-0010-0000-0200-000018000000}" name="Q23 How much trouble do you have pushing, pulling, lifting or carrying heavy objects at work?" dataDxfId="43"/>
-    <tableColumn id="25" xr3:uid="{00000000-0010-0000-0200-000019000000}" name="Q24 How much trouble do you have with crouching/squatting?_x000a_" dataDxfId="42"/>
-    <tableColumn id="26" xr3:uid="{00000000-0010-0000-0200-00001A000000}" name="Q25 How concerned are you that your job will make your hip worse?_x000a__x000a_" dataDxfId="41"/>
-    <tableColumn id="27" xr3:uid="{00000000-0010-0000-0200-00001B000000}" name="Q26 How much difficulty do you have at work because of reduced hip mobility?" dataDxfId="40"/>
-    <tableColumn id="28" xr3:uid="{00000000-0010-0000-0200-00001C000000}" name="Q27 How frustrated are you because of your hip problem?" dataDxfId="39"/>
-    <tableColumn id="29" xr3:uid="{00000000-0010-0000-0200-00001D000000}" name="Q28 How much trouble do you have with sexual activity because of your hip?" dataDxfId="38"/>
-    <tableColumn id="30" xr3:uid="{00000000-0010-0000-0200-00001E000000}" name="Q29 How much of a distraction is your hip problem?" dataDxfId="37"/>
-    <tableColumn id="31" xr3:uid="{00000000-0010-0000-0200-00001F000000}" name="Q30 How difficult is it for you to release tension and stress because of your hip problem?" dataDxfId="36"/>
-    <tableColumn id="32" xr3:uid="{00000000-0010-0000-0200-000020000000}" name="Q31 How discouraged are you because of your hip problem?" dataDxfId="35"/>
-    <tableColumn id="33" xr3:uid="{00000000-0010-0000-0200-000021000000}" name="Q32 How concerned are you about picking up or carrying children because of your hip?" dataDxfId="34"/>
-    <tableColumn id="34" xr3:uid="{00000000-0010-0000-0200-000022000000}" name="Q33 How much of the time are you aware of the disability in your hip?" dataDxfId="33"/>
-    <tableColumn id="35" xr3:uid="{00000000-0010-0000-0200-000023000000}" name="Sum" dataDxfId="32">
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0200-000002000000}" name="Q01 How often does your hip/groin ache?" dataDxfId="63"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0200-000003000000}" name="Q02 How stiff is your hip as a result of sitting/resting during the day?" dataDxfId="62"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0200-000004000000}" name="Q03 How difficult is it for you to walk long distances?" dataDxfId="61"/>
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0200-000005000000}" name="Q04 How much pain do you have in your hip while sitting?" dataDxfId="60"/>
+    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0200-000006000000}" name="Q05 How much trouble do you have standing on your feet for long periods of time?" dataDxfId="59"/>
+    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0200-000007000000}" name="Q06 How difficult is it for you to get up and down off the floor/ground?" dataDxfId="58"/>
+    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0200-000008000000}" name="Q07 How difficult is it for you to walk on uneven surfaces?" dataDxfId="57"/>
+    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0200-000009000000}" name="Q08 How difficult is it for you to lie on your affected hip side?" dataDxfId="56"/>
+    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0200-00000A000000}" name="Q09 How much trouble do you have with stepping over obstacles?" dataDxfId="55"/>
+    <tableColumn id="11" xr3:uid="{00000000-0010-0000-0200-00000B000000}" name="Q10 How much trouble do you have with climbing up/down stairs?" dataDxfId="54"/>
+    <tableColumn id="12" xr3:uid="{00000000-0010-0000-0200-00000C000000}" name="Q11 How much trouble do you have with rising from a sitting position?" dataDxfId="53"/>
+    <tableColumn id="13" xr3:uid="{00000000-0010-0000-0200-00000D000000}" name="Q12 How much discomfort do you have with taking long strides?" dataDxfId="52"/>
+    <tableColumn id="14" xr3:uid="{00000000-0010-0000-0200-00000E000000}" name="Q13 How much difficulty do you have with getting into and/or out of a car?_x000a_" dataDxfId="51"/>
+    <tableColumn id="15" xr3:uid="{00000000-0010-0000-0200-00000F000000}" name="Q14 How much trouble do you have with grinding, catching or clicking in your hip?" dataDxfId="50"/>
+    <tableColumn id="16" xr3:uid="{00000000-0010-0000-0200-000010000000}" name="Q15 How much difficulty do you have with putting on/taking off socks, stockings or shoes?" dataDxfId="49"/>
+    <tableColumn id="17" xr3:uid="{00000000-0010-0000-0200-000011000000}" name="Q16 Overall, how much pain do you have in your hip/groin?" dataDxfId="48"/>
+    <tableColumn id="18" xr3:uid="{00000000-0010-0000-0200-000012000000}" name="Q17 How concerned are you about your ability to maintain your desired fitness level?" dataDxfId="47"/>
+    <tableColumn id="19" xr3:uid="{00000000-0010-0000-0200-000013000000}" name="Q18 How much pain do you experience in your hip after activity?" dataDxfId="46"/>
+    <tableColumn id="20" xr3:uid="{00000000-0010-0000-0200-000014000000}" name="Q19 How concerned are you that the pain in your hip will increase if you participate in sports or recreational activities?_x000a_" dataDxfId="45"/>
+    <tableColumn id="21" xr3:uid="{00000000-0010-0000-0200-000015000000}" name="Q20 How much has your quality of life deteriorated because you cannot participate in sport/recreational activities?" dataDxfId="44"/>
+    <tableColumn id="22" xr3:uid="{00000000-0010-0000-0200-000016000000}" name="Q21 How concerned are you about cutting/changing direction during your sport or recreational activities?" dataDxfId="43"/>
+    <tableColumn id="23" xr3:uid="{00000000-0010-0000-0200-000017000000}" name="Q22 How much has your performance level decreased in your sport or recreational activities?" dataDxfId="42"/>
+    <tableColumn id="24" xr3:uid="{00000000-0010-0000-0200-000018000000}" name="Q23 How much trouble do you have pushing, pulling, lifting or carrying heavy objects at work?" dataDxfId="41"/>
+    <tableColumn id="25" xr3:uid="{00000000-0010-0000-0200-000019000000}" name="Q24 How much trouble do you have with crouching/squatting?_x000a_" dataDxfId="40"/>
+    <tableColumn id="26" xr3:uid="{00000000-0010-0000-0200-00001A000000}" name="Q25 How concerned are you that your job will make your hip worse?_x000a__x000a_" dataDxfId="39"/>
+    <tableColumn id="27" xr3:uid="{00000000-0010-0000-0200-00001B000000}" name="Q26 How much difficulty do you have at work because of reduced hip mobility?" dataDxfId="38"/>
+    <tableColumn id="28" xr3:uid="{00000000-0010-0000-0200-00001C000000}" name="Q27 How frustrated are you because of your hip problem?" dataDxfId="37"/>
+    <tableColumn id="29" xr3:uid="{00000000-0010-0000-0200-00001D000000}" name="Q28 How much trouble do you have with sexual activity because of your hip?" dataDxfId="36"/>
+    <tableColumn id="30" xr3:uid="{00000000-0010-0000-0200-00001E000000}" name="Q29 How much of a distraction is your hip problem?" dataDxfId="35"/>
+    <tableColumn id="31" xr3:uid="{00000000-0010-0000-0200-00001F000000}" name="Q30 How difficult is it for you to release tension and stress because of your hip problem?" dataDxfId="34"/>
+    <tableColumn id="32" xr3:uid="{00000000-0010-0000-0200-000020000000}" name="Q31 How discouraged are you because of your hip problem?" dataDxfId="33"/>
+    <tableColumn id="33" xr3:uid="{00000000-0010-0000-0200-000021000000}" name="Q32 How concerned are you about picking up or carrying children because of your hip?" dataDxfId="32"/>
+    <tableColumn id="34" xr3:uid="{00000000-0010-0000-0200-000022000000}" name="Q33 How much of the time are you aware of the disability in your hip?" dataDxfId="31"/>
+    <tableColumn id="35" xr3:uid="{00000000-0010-0000-0200-000023000000}" name="Sum" dataDxfId="30">
       <calculatedColumnFormula>SUM(Table7[[#This Row],[Q01 How often does your hip/groin ache?]:[Q33 How much of the time are you aware of the disability in your hip?]])/AJ3</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="36" xr3:uid="{00000000-0010-0000-0200-000024000000}" name="Column1" dataDxfId="31">
+    <tableColumn id="36" xr3:uid="{00000000-0010-0000-0200-000024000000}" name="Column1" dataDxfId="29">
       <calculatedColumnFormula>COUNTA(B3:AH3)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -3870,13 +3905,13 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{00000000-000C-0000-FFFF-FFFF03000000}" name="Table4" displayName="Table4" ref="A1:AR16" totalsRowShown="0" headerRowDxfId="30">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{00000000-000C-0000-FFFF-FFFF03000000}" name="Table4" displayName="Table4" ref="A1:AR16" totalsRowShown="0" headerRowDxfId="28">
   <autoFilter ref="A1:AR16" xr:uid="{00000000-0009-0000-0100-000004000000}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:AR21">
     <sortCondition ref="A1:A21"/>
   </sortState>
   <tableColumns count="44">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0300-000001000000}" name="Scoringleft to right (0-4)" dataDxfId="29"/>
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0300-000001000000}" name="Scoringleft to right (0-4)" dataDxfId="27"/>
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0300-000002000000}" name="S1. Do you feel discomfort in your hip and/or groin?"/>
     <tableColumn id="3" xr3:uid="{00000000-0010-0000-0300-000003000000}" name="S2. Do you hear clicking or any other type of noise from your hip and/or groin?"/>
     <tableColumn id="4" xr3:uid="{00000000-0010-0000-0300-000004000000}" name="S3. Do you have any difficulties stretching your legs far out to the side?"/>
@@ -3884,10 +3919,10 @@
     <tableColumn id="6" xr3:uid="{00000000-0010-0000-0300-000006000000}" name="S5. Do you experience sudden twinging/ stabbing sensations in your hip and/or groin?"/>
     <tableColumn id="7" xr3:uid="{00000000-0010-0000-0300-000007000000}" name="S6. How severe is your hip and/or groin after first awakening in the morning?"/>
     <tableColumn id="39" xr3:uid="{00000000-0010-0000-0300-000027000000}" name="S7. How severe is your hip and/or groin stiffness after sitting, lying or resting later in the day?"/>
-    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0300-000008000000}" name="Sum_S" dataDxfId="28">
+    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0300-000008000000}" name="Sum_S" dataDxfId="26">
       <calculatedColumnFormula>100-(SUM(B2:H2)*100)/28</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0300-000009000000}" name="P1. How often is your hip and/or groin painful?" dataDxfId="27"/>
+    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0300-000009000000}" name="P1. How often is your hip and/or groin painful?" dataDxfId="25"/>
     <tableColumn id="10" xr3:uid="{00000000-0010-0000-0300-00000A000000}" name="P2. How often do you have pain in areas other than your hip and/or groin that you think may be related to your hip and/or groin problem?"/>
     <tableColumn id="11" xr3:uid="{00000000-0010-0000-0300-00000B000000}" name="P3. Straightening your hip fully"/>
     <tableColumn id="12" xr3:uid="{00000000-0010-0000-0300-00000C000000}" name="P4. Bending your hip fully"/>
@@ -3897,15 +3932,15 @@
     <tableColumn id="16" xr3:uid="{00000000-0010-0000-0300-000010000000}" name="P8. Standing upright"/>
     <tableColumn id="17" xr3:uid="{00000000-0010-0000-0300-000011000000}" name="P9. Walking on a hard surface (asphalt, concrete, etc.)"/>
     <tableColumn id="40" xr3:uid="{00000000-0010-0000-0300-000028000000}" name="P10. Walking on an uneven surface"/>
-    <tableColumn id="18" xr3:uid="{00000000-0010-0000-0300-000012000000}" name="Sum_P" dataDxfId="26">
+    <tableColumn id="18" xr3:uid="{00000000-0010-0000-0300-000012000000}" name="Sum_P" dataDxfId="24">
       <calculatedColumnFormula>100-(SUM(J2:S2)*100)/40</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="19" xr3:uid="{00000000-0010-0000-0300-000013000000}" name="A1. Walking up stairs" dataDxfId="25"/>
+    <tableColumn id="19" xr3:uid="{00000000-0010-0000-0300-000013000000}" name="A1. Walking up stairs" dataDxfId="23"/>
     <tableColumn id="20" xr3:uid="{00000000-0010-0000-0300-000014000000}" name="A2. Bending down, e.g. to pick something up from the floor"/>
     <tableColumn id="21" xr3:uid="{00000000-0010-0000-0300-000015000000}" name="A3. Getting in/out of car"/>
     <tableColumn id="22" xr3:uid="{00000000-0010-0000-0300-000016000000}" name="A4. Lying in bed (turning over or maintaining the same hip position for a long time)"/>
     <tableColumn id="41" xr3:uid="{00000000-0010-0000-0300-000029000000}" name="A5. Heavy domestic duties (scrubbing floors, vacuuming, moving heavy boxes etc.)"/>
-    <tableColumn id="23" xr3:uid="{00000000-0010-0000-0300-000017000000}" name="Sum_A" dataDxfId="24">
+    <tableColumn id="23" xr3:uid="{00000000-0010-0000-0300-000017000000}" name="Sum_A" dataDxfId="22">
       <calculatedColumnFormula>100-(SUM(U2:Y2)*100)/20</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="24" xr3:uid="{00000000-0010-0000-0300-000018000000}" name="SP1. Squatting"/>
@@ -3916,12 +3951,12 @@
     <tableColumn id="29" xr3:uid="{00000000-0010-0000-0300-00001D000000}" name="SP6. Bringing the leg forcefully forward and/or out to the side, such as in kicking, skating etc."/>
     <tableColumn id="30" xr3:uid="{00000000-0010-0000-0300-00001E000000}" name="SP7. Sudden explosive movements that involve quick footwork, such as accelerations, decelerations, change of direction etc."/>
     <tableColumn id="42" xr3:uid="{00000000-0010-0000-0300-00002A000000}" name="SP8. Situations where the leg is stretched into an outer position (such as when the leg is placed as far away from the body as possible)"/>
-    <tableColumn id="31" xr3:uid="{00000000-0010-0000-0300-00001F000000}" name="Sum_SP" dataDxfId="23">
+    <tableColumn id="31" xr3:uid="{00000000-0010-0000-0300-00001F000000}" name="Sum_SP" dataDxfId="21">
       <calculatedColumnFormula>100-(SUM(AA2:AH2)*100)/32</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="32" xr3:uid="{00000000-0010-0000-0300-000020000000}" name="PA1. Are you able to participate in your preferred physical activities for as long as you would like?"/>
     <tableColumn id="43" xr3:uid="{00000000-0010-0000-0300-00002B000000}" name="PA2. Are you able to participate in your preferred physical activities at your normal performance level?"/>
-    <tableColumn id="33" xr3:uid="{00000000-0010-0000-0300-000021000000}" name="Sum_PA" dataDxfId="22">
+    <tableColumn id="33" xr3:uid="{00000000-0010-0000-0300-000021000000}" name="Sum_PA" dataDxfId="20">
       <calculatedColumnFormula>100-(SUM(AJ2:AK2)*100)/8</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="34" xr3:uid="{00000000-0010-0000-0300-000022000000}" name="Q1. How often are you aware of your hip and/or groin problem?"/>
@@ -3929,7 +3964,7 @@
     <tableColumn id="36" xr3:uid="{00000000-0010-0000-0300-000024000000}" name="Q3. In general, how much difficulty do you have with your hip and/or groin?"/>
     <tableColumn id="37" xr3:uid="{00000000-0010-0000-0300-000025000000}" name="Q4. Does your hip and/or groin problem affect your mood in a negative way?"/>
     <tableColumn id="38" xr3:uid="{00000000-0010-0000-0300-000026000000}" name="Q5. Do you feel restricted due to your hip and/or groin problem?"/>
-    <tableColumn id="44" xr3:uid="{00000000-0010-0000-0300-00002C000000}" name="Sum_Q" dataDxfId="21">
+    <tableColumn id="44" xr3:uid="{00000000-0010-0000-0300-00002C000000}" name="Sum_Q" dataDxfId="19">
       <calculatedColumnFormula>100-(SUM(AM2:AQ2)*100)/20</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -3947,8 +3982,8 @@
     </filterColumn>
   </autoFilter>
   <tableColumns count="33">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0400-000001000000}" name="Subject" dataDxfId="20"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0400-000002000000}" name="Group " dataDxfId="19"/>
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0400-000001000000}" name="Subject" dataDxfId="18"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0400-000002000000}" name="Group " dataDxfId="17"/>
     <tableColumn id="3" xr3:uid="{00000000-0010-0000-0400-000003000000}" name="HE"/>
     <tableColumn id="4" xr3:uid="{00000000-0010-0000-0400-000004000000}" name="HEAB"/>
     <tableColumn id="5" xr3:uid="{00000000-0010-0000-0400-000005000000}" name="HEER"/>
@@ -3996,32 +4031,32 @@
     <tableColumn id="5" xr3:uid="{00000000-0010-0000-0500-000005000000}" name="s004"/>
     <tableColumn id="6" xr3:uid="{00000000-0010-0000-0500-000006000000}" name="s005"/>
     <tableColumn id="7" xr3:uid="{00000000-0010-0000-0500-000007000000}" name="s006"/>
-    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0500-000008000000}" name="s007" dataDxfId="18"/>
-    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0500-000009000000}" name="s008" dataDxfId="17"/>
+    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0500-000008000000}" name="s007" dataDxfId="16"/>
+    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0500-000009000000}" name="s008" dataDxfId="15"/>
     <tableColumn id="10" xr3:uid="{00000000-0010-0000-0500-00000A000000}" name="s009"/>
-    <tableColumn id="11" xr3:uid="{00000000-0010-0000-0500-00000B000000}" name="s010" dataDxfId="16"/>
-    <tableColumn id="12" xr3:uid="{00000000-0010-0000-0500-00000C000000}" name="s011" dataDxfId="15"/>
+    <tableColumn id="11" xr3:uid="{00000000-0010-0000-0500-00000B000000}" name="s010" dataDxfId="14"/>
+    <tableColumn id="12" xr3:uid="{00000000-0010-0000-0500-00000C000000}" name="s011" dataDxfId="13"/>
     <tableColumn id="13" xr3:uid="{00000000-0010-0000-0500-00000D000000}" name="s012"/>
     <tableColumn id="14" xr3:uid="{00000000-0010-0000-0500-00000E000000}" name="s013"/>
-    <tableColumn id="15" xr3:uid="{00000000-0010-0000-0500-00000F000000}" name="s014" dataDxfId="14"/>
+    <tableColumn id="15" xr3:uid="{00000000-0010-0000-0500-00000F000000}" name="s014" dataDxfId="12"/>
     <tableColumn id="16" xr3:uid="{00000000-0010-0000-0500-000010000000}" name="s015"/>
-    <tableColumn id="17" xr3:uid="{00000000-0010-0000-0500-000011000000}" name="s016" dataDxfId="13"/>
-    <tableColumn id="18" xr3:uid="{00000000-0010-0000-0500-000012000000}" name="s017" dataDxfId="12"/>
+    <tableColumn id="17" xr3:uid="{00000000-0010-0000-0500-000011000000}" name="s016" dataDxfId="11"/>
+    <tableColumn id="18" xr3:uid="{00000000-0010-0000-0500-000012000000}" name="s017" dataDxfId="10"/>
     <tableColumn id="19" xr3:uid="{00000000-0010-0000-0500-000013000000}" name="s018"/>
     <tableColumn id="20" xr3:uid="{00000000-0010-0000-0500-000014000000}" name="s019"/>
-    <tableColumn id="21" xr3:uid="{00000000-0010-0000-0500-000015000000}" name="s020" dataDxfId="11"/>
+    <tableColumn id="21" xr3:uid="{00000000-0010-0000-0500-000015000000}" name="s020" dataDxfId="9"/>
     <tableColumn id="22" xr3:uid="{00000000-0010-0000-0500-000016000000}" name="s021"/>
     <tableColumn id="23" xr3:uid="{00000000-0010-0000-0500-000017000000}" name="s022"/>
-    <tableColumn id="24" xr3:uid="{00000000-0010-0000-0500-000018000000}" name="s023" dataDxfId="10"/>
+    <tableColumn id="24" xr3:uid="{00000000-0010-0000-0500-000018000000}" name="s023" dataDxfId="8"/>
     <tableColumn id="25" xr3:uid="{00000000-0010-0000-0500-000019000000}" name="s024"/>
     <tableColumn id="26" xr3:uid="{00000000-0010-0000-0500-00001A000000}" name="s025"/>
     <tableColumn id="27" xr3:uid="{00000000-0010-0000-0500-00001B000000}" name="s026"/>
-    <tableColumn id="28" xr3:uid="{00000000-0010-0000-0500-00001C000000}" name="s027" dataDxfId="9"/>
+    <tableColumn id="28" xr3:uid="{00000000-0010-0000-0500-00001C000000}" name="s027" dataDxfId="7"/>
     <tableColumn id="29" xr3:uid="{00000000-0010-0000-0500-00001D000000}" name="s028"/>
     <tableColumn id="30" xr3:uid="{00000000-0010-0000-0500-00001E000000}" name="s029"/>
     <tableColumn id="31" xr3:uid="{00000000-0010-0000-0500-00001F000000}" name="s030"/>
     <tableColumn id="32" xr3:uid="{00000000-0010-0000-0500-000020000000}" name="s031"/>
-    <tableColumn id="33" xr3:uid="{00000000-0010-0000-0500-000021000000}" name="s032" dataDxfId="8"/>
+    <tableColumn id="33" xr3:uid="{00000000-0010-0000-0500-000021000000}" name="s032" dataDxfId="6"/>
     <tableColumn id="34" xr3:uid="{00000000-0010-0000-0500-000022000000}" name="s033"/>
     <tableColumn id="35" xr3:uid="{00000000-0010-0000-0500-000023000000}" name="s034"/>
     <tableColumn id="36" xr3:uid="{00000000-0010-0000-0500-000024000000}" name="s035"/>
@@ -4031,11 +4066,11 @@
     <tableColumn id="40" xr3:uid="{00000000-0010-0000-0500-000028000000}" name="s039"/>
     <tableColumn id="41" xr3:uid="{00000000-0010-0000-0500-000029000000}" name="s040"/>
     <tableColumn id="42" xr3:uid="{00000000-0010-0000-0500-00002A000000}" name="s041"/>
-    <tableColumn id="43" xr3:uid="{00000000-0010-0000-0500-00002B000000}" name="s042" dataDxfId="7"/>
+    <tableColumn id="43" xr3:uid="{00000000-0010-0000-0500-00002B000000}" name="s042" dataDxfId="5"/>
     <tableColumn id="44" xr3:uid="{00000000-0010-0000-0500-00002C000000}" name="s043"/>
     <tableColumn id="45" xr3:uid="{00000000-0010-0000-0500-00002D000000}" name="s044"/>
     <tableColumn id="46" xr3:uid="{00000000-0010-0000-0500-00002E000000}" name="s045"/>
-    <tableColumn id="47" xr3:uid="{00000000-0010-0000-0500-00002F000000}" name="s046" dataDxfId="6"/>
+    <tableColumn id="47" xr3:uid="{00000000-0010-0000-0500-00002F000000}" name="s046" dataDxfId="4"/>
     <tableColumn id="48" xr3:uid="{00000000-0010-0000-0500-000030000000}" name="s047"/>
     <tableColumn id="49" xr3:uid="{00000000-0010-0000-0500-000031000000}" name="s048"/>
     <tableColumn id="50" xr3:uid="{00000000-0010-0000-0500-000032000000}" name="s049"/>
@@ -4043,10 +4078,10 @@
     <tableColumn id="53" xr3:uid="{00000000-0010-0000-0500-000035000000}" name="s052"/>
     <tableColumn id="54" xr3:uid="{00000000-0010-0000-0500-000036000000}" name="s053"/>
     <tableColumn id="55" xr3:uid="{00000000-0010-0000-0500-000037000000}" name="s054"/>
-    <tableColumn id="56" xr3:uid="{00000000-0010-0000-0500-000038000000}" name="s055" dataDxfId="5"/>
+    <tableColumn id="56" xr3:uid="{00000000-0010-0000-0500-000038000000}" name="s055" dataDxfId="3"/>
     <tableColumn id="57" xr3:uid="{00000000-0010-0000-0500-000039000000}" name="s056"/>
     <tableColumn id="58" xr3:uid="{00000000-0010-0000-0500-00003A000000}" name="s057"/>
-    <tableColumn id="59" xr3:uid="{00000000-0010-0000-0500-00003B000000}" name="s058" dataDxfId="4"/>
+    <tableColumn id="59" xr3:uid="{00000000-0010-0000-0500-00003B000000}" name="s058" dataDxfId="2"/>
     <tableColumn id="60" xr3:uid="{00000000-0010-0000-0500-00003C000000}" name="s059"/>
     <tableColumn id="61" xr3:uid="{00000000-0010-0000-0500-00003D000000}" name="s060"/>
     <tableColumn id="62" xr3:uid="{00000000-0010-0000-0500-00003E000000}" name="s061"/>
@@ -4055,12 +4090,12 @@
     <tableColumn id="65" xr3:uid="{00000000-0010-0000-0500-000041000000}" name="s064"/>
     <tableColumn id="66" xr3:uid="{00000000-0010-0000-0500-000042000000}" name="s065"/>
     <tableColumn id="67" xr3:uid="{00000000-0010-0000-0500-000043000000}" name="s066"/>
-    <tableColumn id="68" xr3:uid="{00000000-0010-0000-0500-000044000000}" name="s067" dataDxfId="3"/>
+    <tableColumn id="68" xr3:uid="{00000000-0010-0000-0500-000044000000}" name="s067" dataDxfId="1"/>
     <tableColumn id="69" xr3:uid="{00000000-0010-0000-0500-000045000000}" name="s068"/>
     <tableColumn id="70" xr3:uid="{00000000-0010-0000-0500-000046000000}" name="s069"/>
     <tableColumn id="71" xr3:uid="{00000000-0010-0000-0500-000047000000}" name="s070"/>
     <tableColumn id="72" xr3:uid="{00000000-0010-0000-0500-000048000000}" name="s071"/>
-    <tableColumn id="73" xr3:uid="{00000000-0010-0000-0500-000049000000}" name="s072" dataDxfId="2"/>
+    <tableColumn id="73" xr3:uid="{00000000-0010-0000-0500-000049000000}" name="s072" dataDxfId="0"/>
     <tableColumn id="74" xr3:uid="{00000000-0010-0000-0500-00004A000000}" name="s073"/>
     <tableColumn id="75" xr3:uid="{00000000-0010-0000-0500-00004B000000}" name="s074"/>
     <tableColumn id="76" xr3:uid="{00000000-0010-0000-0500-00004C000000}" name="s075"/>
@@ -4380,11 +4415,13 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:AI74"/>
-  <sheetFormatPr defaultColWidth="9.1796875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultColWidth="9.1796875" defaultRowHeight="14.5"/>
   <cols>
     <col min="1" max="1" width="10" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="7.81640625" customWidth="1"/>
-    <col min="4" max="20" width="7.54296875" customWidth="1"/>
+    <col min="4" max="5" width="7.54296875" customWidth="1"/>
+    <col min="6" max="6" width="12.90625" bestFit="1" customWidth="1"/>
+    <col min="7" max="20" width="7.54296875" customWidth="1"/>
     <col min="21" max="21" width="10" bestFit="1" customWidth="1"/>
     <col min="22" max="22" width="9.26953125" bestFit="1" customWidth="1"/>
     <col min="23" max="23" width="22.26953125" customWidth="1"/>
@@ -4396,7 +4433,7 @@
     <col min="36" max="36" width="15.7265625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:35" ht="45" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:35" ht="45" customHeight="1">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -4503,7 +4540,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="2" spans="1:35" s="41" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:35" s="41" customFormat="1">
       <c r="A2" s="56" t="s">
         <v>59</v>
       </c>
@@ -4592,7 +4629,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="3" spans="1:35" s="41" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:35" s="41" customFormat="1">
       <c r="A3" s="56" t="s">
         <v>62</v>
       </c>
@@ -4680,7 +4717,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="4" spans="1:35" s="41" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:35" s="41" customFormat="1">
       <c r="A4" s="56" t="s">
         <v>64</v>
       </c>
@@ -4696,6 +4733,7 @@
       <c r="E4" s="41" t="s">
         <v>35</v>
       </c>
+      <c r="F4" s="99"/>
       <c r="G4" s="41" t="s">
         <v>36</v>
       </c>
@@ -4743,7 +4781,7 @@
       <c r="AG4"/>
       <c r="AH4"/>
     </row>
-    <row r="5" spans="1:35" s="41" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:35" s="41" customFormat="1">
       <c r="A5" s="56" t="s">
         <v>65</v>
       </c>
@@ -4827,7 +4865,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="6" spans="1:35" s="41" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:35" s="41" customFormat="1">
       <c r="A6" s="56" t="s">
         <v>67</v>
       </c>
@@ -4914,7 +4952,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="7" spans="1:35" s="41" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:35" s="41" customFormat="1">
       <c r="A7" s="56" t="s">
         <v>69</v>
       </c>
@@ -4997,7 +5035,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="8" spans="1:35" s="41" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:35" s="41" customFormat="1">
       <c r="A8" s="56" t="s">
         <v>71</v>
       </c>
@@ -5082,7 +5120,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="9" spans="1:35" s="41" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:35" s="41" customFormat="1">
       <c r="A9" s="56" t="s">
         <v>73</v>
       </c>
@@ -5169,7 +5207,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="10" spans="1:35" s="41" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:35" s="41" customFormat="1">
       <c r="A10" s="56" t="s">
         <v>75</v>
       </c>
@@ -5256,7 +5294,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="11" spans="1:35" s="41" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:35" s="41" customFormat="1">
       <c r="A11" s="56" t="s">
         <v>78</v>
       </c>
@@ -5272,16 +5310,19 @@
       <c r="E11" s="41" t="s">
         <v>35</v>
       </c>
-      <c r="G11" s="41" t="s">
+      <c r="F11" s="102" t="s">
+        <v>38</v>
+      </c>
+      <c r="G11" s="101" t="s">
         <v>56</v>
       </c>
-      <c r="H11" s="41">
+      <c r="H11" s="101">
         <v>61</v>
       </c>
-      <c r="I11" s="41">
+      <c r="I11" s="101">
         <v>16.2</v>
       </c>
-      <c r="J11" s="41" t="s">
+      <c r="J11" s="102" t="s">
         <v>52</v>
       </c>
       <c r="K11" s="41" t="s">
@@ -5346,7 +5387,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="12" spans="1:35" s="41" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:35" s="41" customFormat="1">
       <c r="A12" s="61" t="s">
         <v>81</v>
       </c>
@@ -5362,6 +5403,7 @@
       <c r="E12" s="41" t="s">
         <v>41</v>
       </c>
+      <c r="F12" s="100"/>
       <c r="G12" s="41" t="s">
         <v>36</v>
       </c>
@@ -5369,7 +5411,7 @@
         <v>48.4</v>
       </c>
       <c r="I12"/>
-      <c r="J12" s="41" t="s">
+      <c r="J12" s="100" t="s">
         <v>42</v>
       </c>
       <c r="K12" s="41" t="s">
@@ -5434,7 +5476,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="13" spans="1:35" s="41" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:35" s="41" customFormat="1">
       <c r="A13" s="61" t="s">
         <v>85</v>
       </c>
@@ -5518,7 +5560,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="14" spans="1:35" s="41" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:35" s="41" customFormat="1">
       <c r="A14" s="61" t="s">
         <v>87</v>
       </c>
@@ -5608,7 +5650,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="15" spans="1:35" s="41" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:35" s="41" customFormat="1">
       <c r="A15" s="61" t="s">
         <v>89</v>
       </c>
@@ -5696,7 +5738,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="16" spans="1:35" s="41" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:35" s="41" customFormat="1">
       <c r="A16" s="61" t="s">
         <v>91</v>
       </c>
@@ -5783,7 +5825,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="17" spans="1:35" s="41" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:35" s="41" customFormat="1">
       <c r="A17" s="61" t="s">
         <v>94</v>
       </c>
@@ -5867,7 +5909,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="18" spans="1:35" s="41" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:35" s="41" customFormat="1">
       <c r="A18" s="61" t="s">
         <v>96</v>
       </c>
@@ -5951,7 +5993,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="19" spans="1:35" s="41" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:35" s="41" customFormat="1">
       <c r="A19" s="61" t="s">
         <v>98</v>
       </c>
@@ -6032,7 +6074,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="20" spans="1:35" s="41" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:35" s="41" customFormat="1">
       <c r="A20" s="61" t="s">
         <v>100</v>
       </c>
@@ -6116,7 +6158,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="21" spans="1:35" s="41" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:35" s="41" customFormat="1">
       <c r="A21" s="61" t="s">
         <v>102</v>
       </c>
@@ -6201,7 +6243,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="22" spans="1:35" s="41" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:35" s="41" customFormat="1">
       <c r="A22" s="61" t="s">
         <v>104</v>
       </c>
@@ -6291,7 +6333,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="23" spans="1:35" s="41" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:35" s="41" customFormat="1">
       <c r="A23" s="61" t="s">
         <v>107</v>
       </c>
@@ -6381,7 +6423,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="24" spans="1:35" s="41" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:35" s="41" customFormat="1">
       <c r="A24" s="61" t="s">
         <v>109</v>
       </c>
@@ -6466,7 +6508,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="25" spans="1:35" s="41" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:35" s="41" customFormat="1">
       <c r="A25" s="61" t="s">
         <v>112</v>
       </c>
@@ -6560,7 +6602,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="26" spans="1:35" s="41" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:35" s="41" customFormat="1">
       <c r="A26" s="61" t="s">
         <v>116</v>
       </c>
@@ -6648,7 +6690,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="27" spans="1:35" s="41" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:35" s="41" customFormat="1">
       <c r="A27" s="61" t="s">
         <v>119</v>
       </c>
@@ -6718,7 +6760,7 @@
       <c r="AG27"/>
       <c r="AH27"/>
     </row>
-    <row r="28" spans="1:35" s="41" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:35" s="41" customFormat="1">
       <c r="A28" s="61" t="s">
         <v>122</v>
       </c>
@@ -6735,16 +6777,19 @@
       <c r="E28" s="41" t="s">
         <v>35</v>
       </c>
-      <c r="G28" s="41" t="s">
+      <c r="F28" s="102" t="s">
+        <v>38</v>
+      </c>
+      <c r="G28" s="101" t="s">
         <v>56</v>
       </c>
-      <c r="H28" s="41">
+      <c r="H28" s="101">
         <v>45.5</v>
       </c>
-      <c r="I28" s="41">
+      <c r="I28" s="101">
         <v>27.8</v>
       </c>
-      <c r="J28" s="41" t="s">
+      <c r="J28" s="102" t="s">
         <v>42</v>
       </c>
       <c r="K28" s="41" t="s">
@@ -6808,7 +6853,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="29" spans="1:35" s="41" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:35" s="41" customFormat="1">
       <c r="A29" s="61" t="s">
         <v>125</v>
       </c>
@@ -6898,7 +6943,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="30" spans="1:35" s="41" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:35" s="41" customFormat="1">
       <c r="A30" s="61" t="s">
         <v>127</v>
       </c>
@@ -6915,16 +6960,19 @@
       <c r="E30" s="41" t="s">
         <v>35</v>
       </c>
-      <c r="G30" s="41" t="s">
+      <c r="F30" s="102" t="s">
+        <v>38</v>
+      </c>
+      <c r="G30" s="101" t="s">
         <v>56</v>
       </c>
-      <c r="H30" s="41">
+      <c r="H30" s="101">
         <v>61.4</v>
       </c>
-      <c r="I30" s="41">
+      <c r="I30" s="101">
         <v>27.7</v>
       </c>
-      <c r="J30" s="41" t="s">
+      <c r="J30" s="102" t="s">
         <v>52</v>
       </c>
       <c r="K30" s="41" t="s">
@@ -6988,7 +7036,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="31" spans="1:35" s="41" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:35" s="41" customFormat="1">
       <c r="A31" s="61" t="s">
         <v>129</v>
       </c>
@@ -7005,16 +7053,19 @@
       <c r="E31" s="41" t="s">
         <v>35</v>
       </c>
-      <c r="G31" s="41" t="s">
+      <c r="F31" s="102" t="s">
+        <v>38</v>
+      </c>
+      <c r="G31" s="101" t="s">
         <v>56</v>
       </c>
-      <c r="H31" s="41">
+      <c r="H31" s="101">
         <v>48.3</v>
       </c>
-      <c r="I31" s="41">
+      <c r="I31" s="101">
         <v>22.6</v>
       </c>
-      <c r="J31" s="41" t="s">
+      <c r="J31" s="102" t="s">
         <v>42</v>
       </c>
       <c r="K31" s="41" t="s">
@@ -7078,7 +7129,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="32" spans="1:35" s="41" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:35" s="41" customFormat="1">
       <c r="A32" s="61" t="s">
         <v>131</v>
       </c>
@@ -7095,16 +7146,19 @@
       <c r="E32" s="41" t="s">
         <v>35</v>
       </c>
-      <c r="G32" s="41" t="s">
+      <c r="F32" s="102" t="s">
+        <v>38</v>
+      </c>
+      <c r="G32" s="101" t="s">
         <v>56</v>
       </c>
-      <c r="H32" s="41">
+      <c r="H32" s="101">
         <v>42.3</v>
       </c>
-      <c r="I32" s="41">
+      <c r="I32" s="101">
         <v>17.8</v>
       </c>
-      <c r="J32" s="41" t="s">
+      <c r="J32" s="102" t="s">
         <v>42</v>
       </c>
       <c r="K32" s="41" t="s">
@@ -7168,7 +7222,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="33" spans="1:35" s="41" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:35" s="41" customFormat="1">
       <c r="A33" s="61" t="s">
         <v>134</v>
       </c>
@@ -7185,16 +7239,19 @@
       <c r="E33" s="41" t="s">
         <v>35</v>
       </c>
-      <c r="G33" s="41" t="s">
+      <c r="F33" s="102" t="s">
+        <v>38</v>
+      </c>
+      <c r="G33" s="101" t="s">
         <v>56</v>
       </c>
-      <c r="H33" s="41">
+      <c r="H33" s="101">
         <v>49.4</v>
       </c>
-      <c r="I33" s="41">
+      <c r="I33" s="101">
         <v>22.5</v>
       </c>
-      <c r="J33" s="41" t="s">
+      <c r="J33" s="102" t="s">
         <v>42</v>
       </c>
       <c r="K33" s="41" t="s">
@@ -7258,7 +7315,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="34" spans="1:35" s="41" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:35" s="41" customFormat="1">
       <c r="A34" s="61" t="s">
         <v>136</v>
       </c>
@@ -7322,7 +7379,7 @@
       <c r="AG34"/>
       <c r="AH34"/>
     </row>
-    <row r="35" spans="1:35" s="41" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:35" s="41" customFormat="1">
       <c r="A35" s="61" t="s">
         <v>137</v>
       </c>
@@ -7339,16 +7396,17 @@
       <c r="E35" s="41" t="s">
         <v>35</v>
       </c>
-      <c r="G35" s="41" t="s">
+      <c r="F35" s="102"/>
+      <c r="G35" s="101" t="s">
         <v>56</v>
       </c>
-      <c r="H35" s="41">
+      <c r="H35" s="101">
         <v>52.4</v>
       </c>
-      <c r="I35" s="41">
+      <c r="I35" s="101">
         <v>23.2</v>
       </c>
-      <c r="J35" s="41" t="s">
+      <c r="J35" s="102" t="s">
         <v>42</v>
       </c>
       <c r="K35" s="41" t="s">
@@ -7412,7 +7470,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="36" spans="1:35" s="41" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:35" s="41" customFormat="1">
       <c r="A36" s="61" t="s">
         <v>140</v>
       </c>
@@ -7429,19 +7487,22 @@
       <c r="E36" s="41" t="s">
         <v>35</v>
       </c>
-      <c r="G36" s="41" t="s">
+      <c r="F36" s="102" t="s">
+        <v>38</v>
+      </c>
+      <c r="G36" s="101" t="s">
         <v>56</v>
       </c>
-      <c r="H36" s="41">
+      <c r="H36" s="101">
         <v>74</v>
       </c>
-      <c r="I36" s="41">
+      <c r="I36" s="101">
         <v>13.9</v>
       </c>
-      <c r="J36" s="41" t="s">
+      <c r="J36" s="102" t="s">
         <v>52</v>
       </c>
-      <c r="K36" s="41" t="s">
+      <c r="K36" s="102" t="s">
         <v>44</v>
       </c>
       <c r="L36" s="41" t="s">
@@ -7502,7 +7563,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="37" spans="1:35" s="41" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:35" s="41" customFormat="1">
       <c r="A37" s="61" t="s">
         <v>143</v>
       </c>
@@ -7584,7 +7645,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="38" spans="1:35" s="41" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:35" s="41" customFormat="1">
       <c r="A38" s="61" t="s">
         <v>145</v>
       </c>
@@ -7652,7 +7713,7 @@
       <c r="AG38"/>
       <c r="AH38"/>
     </row>
-    <row r="39" spans="1:35" s="41" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:35" s="41" customFormat="1">
       <c r="A39" s="61" t="s">
         <v>147</v>
       </c>
@@ -7669,16 +7730,17 @@
       <c r="E39" s="41" t="s">
         <v>35</v>
       </c>
-      <c r="G39" s="41" t="s">
+      <c r="F39" s="102"/>
+      <c r="G39" s="101" t="s">
         <v>56</v>
       </c>
-      <c r="H39" s="41">
+      <c r="H39" s="101">
         <v>39.6</v>
       </c>
-      <c r="I39" s="41">
+      <c r="I39" s="101">
         <v>23.6</v>
       </c>
-      <c r="J39" s="41" t="s">
+      <c r="J39" s="102" t="s">
         <v>42</v>
       </c>
       <c r="K39" s="41" t="s">
@@ -7744,7 +7806,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="40" spans="1:35" s="41" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:35" s="41" customFormat="1">
       <c r="A40" s="61" t="s">
         <v>150</v>
       </c>
@@ -7836,7 +7898,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="41" spans="1:35" s="41" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:35" s="41" customFormat="1">
       <c r="A41" s="61" t="s">
         <v>152</v>
       </c>
@@ -7909,7 +7971,7 @@
       <c r="AG41"/>
       <c r="AH41"/>
     </row>
-    <row r="42" spans="1:35" s="41" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:35" s="41" customFormat="1">
       <c r="A42" s="61" t="s">
         <v>153</v>
       </c>
@@ -8001,7 +8063,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="43" spans="1:35" s="41" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:35" s="41" customFormat="1">
       <c r="A43" s="61" t="s">
         <v>156</v>
       </c>
@@ -8101,7 +8163,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="44" spans="1:35" s="41" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:35" s="41" customFormat="1">
       <c r="A44" s="61" t="s">
         <v>159</v>
       </c>
@@ -8168,7 +8230,7 @@
       <c r="AG44"/>
       <c r="AH44"/>
     </row>
-    <row r="45" spans="1:35" s="41" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:35" s="41" customFormat="1">
       <c r="A45" s="61" t="s">
         <v>160</v>
       </c>
@@ -8185,19 +8247,22 @@
       <c r="E45" s="41" t="s">
         <v>35</v>
       </c>
-      <c r="G45" s="41" t="s">
+      <c r="F45" s="102" t="s">
+        <v>38</v>
+      </c>
+      <c r="G45" s="101" t="s">
         <v>56</v>
       </c>
-      <c r="H45" s="41">
+      <c r="H45" s="101">
         <v>66.900000000000006</v>
       </c>
-      <c r="I45" s="41">
+      <c r="I45" s="101">
         <v>14.2</v>
       </c>
-      <c r="J45" s="41" t="s">
+      <c r="J45" s="101" t="s">
         <v>52</v>
       </c>
-      <c r="K45" s="41" t="s">
+      <c r="K45" s="102" t="s">
         <v>44</v>
       </c>
       <c r="L45" s="41" t="s">
@@ -8258,7 +8323,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="46" spans="1:35" s="41" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:35" s="41" customFormat="1">
       <c r="A46" s="61" t="s">
         <v>162</v>
       </c>
@@ -8364,7 +8429,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="47" spans="1:35" s="41" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:35" s="41" customFormat="1">
       <c r="A47" s="61" t="s">
         <v>165</v>
       </c>
@@ -8454,7 +8519,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="48" spans="1:35" s="41" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:35" s="41" customFormat="1">
       <c r="A48" s="61" t="s">
         <v>168</v>
       </c>
@@ -8524,7 +8589,7 @@
       <c r="AG48"/>
       <c r="AH48"/>
     </row>
-    <row r="49" spans="1:35" s="41" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:35" s="41" customFormat="1">
       <c r="A49" s="61" t="s">
         <v>169</v>
       </c>
@@ -8633,7 +8698,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="50" spans="1:35" s="41" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:35" s="41" customFormat="1" ht="16.5" customHeight="1">
       <c r="A50" s="61" t="s">
         <v>172</v>
       </c>
@@ -8706,7 +8771,7 @@
       <c r="AG50"/>
       <c r="AH50"/>
     </row>
-    <row r="51" spans="1:35" s="41" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:35" s="41" customFormat="1">
       <c r="A51" s="61" t="s">
         <v>174</v>
       </c>
@@ -8815,7 +8880,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="52" spans="1:35" s="41" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:35" s="41" customFormat="1">
       <c r="A52" s="61" t="s">
         <v>177</v>
       </c>
@@ -8925,7 +8990,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="53" spans="1:35" s="41" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:35" s="41" customFormat="1">
       <c r="A53" s="61" t="s">
         <v>180</v>
       </c>
@@ -8999,7 +9064,7 @@
       <c r="AG53"/>
       <c r="AH53"/>
     </row>
-    <row r="54" spans="1:35" s="41" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:35" s="41" customFormat="1">
       <c r="A54" s="61" t="s">
         <v>181</v>
       </c>
@@ -9102,7 +9167,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="55" spans="1:35" s="41" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:35" s="41" customFormat="1">
       <c r="A55" s="61" t="s">
         <v>184</v>
       </c>
@@ -9175,7 +9240,7 @@
       <c r="AG55"/>
       <c r="AH55"/>
     </row>
-    <row r="56" spans="1:35" s="41" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:35" s="41" customFormat="1">
       <c r="A56" s="61" t="s">
         <v>185</v>
       </c>
@@ -9256,7 +9321,7 @@
       <c r="AG56"/>
       <c r="AH56"/>
     </row>
-    <row r="57" spans="1:35" s="41" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:35" s="41" customFormat="1">
       <c r="A57" s="61" t="s">
         <v>186</v>
       </c>
@@ -9329,7 +9394,7 @@
       <c r="AG57"/>
       <c r="AH57"/>
     </row>
-    <row r="58" spans="1:35" s="41" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:35" s="41" customFormat="1">
       <c r="A58" s="61" t="s">
         <v>187</v>
       </c>
@@ -9438,7 +9503,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="59" spans="1:35" s="41" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:35" s="41" customFormat="1">
       <c r="A59" s="61" t="s">
         <v>190</v>
       </c>
@@ -9545,7 +9610,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="60" spans="1:35" s="41" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:35" s="41" customFormat="1">
       <c r="A60" s="61" t="s">
         <v>194</v>
       </c>
@@ -9654,7 +9719,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="61" spans="1:35" s="41" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:35" s="41" customFormat="1">
       <c r="A61" s="61" t="s">
         <v>197</v>
       </c>
@@ -9763,7 +9828,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="62" spans="1:35" s="41" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:35" s="41" customFormat="1">
       <c r="A62" s="61" t="s">
         <v>200</v>
       </c>
@@ -9873,7 +9938,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="63" spans="1:35" s="41" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:35" s="41" customFormat="1">
       <c r="A63" s="61" t="s">
         <v>204</v>
       </c>
@@ -9890,16 +9955,19 @@
       <c r="E63" s="41" t="s">
         <v>35</v>
       </c>
-      <c r="G63" s="41" t="s">
+      <c r="F63" s="102" t="s">
+        <v>38</v>
+      </c>
+      <c r="G63" s="101" t="s">
         <v>56</v>
       </c>
-      <c r="H63" s="95">
+      <c r="H63" s="103">
         <v>74</v>
       </c>
-      <c r="I63" s="95">
+      <c r="I63" s="103">
         <v>11</v>
       </c>
-      <c r="J63" s="41" t="s">
+      <c r="J63" s="102" t="s">
         <v>157</v>
       </c>
       <c r="K63" s="41" t="s">
@@ -9982,7 +10050,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="64" spans="1:35" s="41" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:35" s="41" customFormat="1">
       <c r="A64" s="61" t="s">
         <v>206</v>
       </c>
@@ -9999,16 +10067,19 @@
       <c r="E64" s="41" t="s">
         <v>35</v>
       </c>
-      <c r="G64" s="41" t="s">
+      <c r="F64" s="102" t="s">
+        <v>38</v>
+      </c>
+      <c r="G64" s="101" t="s">
         <v>56</v>
       </c>
-      <c r="H64" s="41">
+      <c r="H64" s="101">
         <v>57.7</v>
       </c>
-      <c r="I64" s="41">
+      <c r="I64" s="101">
         <v>26.2</v>
       </c>
-      <c r="J64" s="41" t="s">
+      <c r="J64" s="102" t="s">
         <v>157</v>
       </c>
       <c r="K64" s="41" t="s">
@@ -10091,7 +10162,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="65" spans="1:35" s="41" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="65" spans="1:35" s="41" customFormat="1">
       <c r="A65" s="61" t="s">
         <v>209</v>
       </c>
@@ -10108,16 +10179,19 @@
       <c r="E65" s="41" t="s">
         <v>41</v>
       </c>
-      <c r="G65" s="41" t="s">
+      <c r="F65" s="102" t="s">
+        <v>38</v>
+      </c>
+      <c r="G65" s="101" t="s">
         <v>56</v>
       </c>
-      <c r="H65" s="41">
+      <c r="H65" s="101">
         <v>59.9</v>
       </c>
-      <c r="I65" s="41">
+      <c r="I65" s="101">
         <v>20.7</v>
       </c>
-      <c r="J65" s="41" t="s">
+      <c r="J65" s="102" t="s">
         <v>157</v>
       </c>
       <c r="K65" s="41" t="s">
@@ -10200,7 +10274,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="66" spans="1:35" s="41" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="66" spans="1:35" s="41" customFormat="1">
       <c r="A66" s="61" t="s">
         <v>212</v>
       </c>
@@ -10311,7 +10385,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="67" spans="1:35" s="41" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="67" spans="1:35" s="41" customFormat="1" ht="15.75" customHeight="1">
       <c r="A67" s="61" t="s">
         <v>215</v>
       </c>
@@ -10327,16 +10401,19 @@
       <c r="E67" s="41" t="s">
         <v>35</v>
       </c>
-      <c r="G67" s="41" t="s">
+      <c r="F67" s="102" t="s">
+        <v>38</v>
+      </c>
+      <c r="G67" s="101" t="s">
         <v>56</v>
       </c>
-      <c r="H67" s="41">
+      <c r="H67" s="101">
         <v>59.9</v>
       </c>
-      <c r="I67" s="41">
+      <c r="I67" s="101">
         <v>22.6</v>
       </c>
-      <c r="J67" s="41" t="s">
+      <c r="J67" s="102" t="s">
         <v>157</v>
       </c>
       <c r="K67" s="41" t="s">
@@ -10418,7 +10495,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="68" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="68" spans="1:35">
       <c r="A68" s="3"/>
       <c r="B68" s="66"/>
       <c r="Q68" s="96"/>
@@ -10436,7 +10513,7 @@
       <c r="AG68"/>
       <c r="AH68"/>
     </row>
-    <row r="69" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="69" spans="1:35">
       <c r="A69" s="98"/>
       <c r="B69" s="98"/>
       <c r="C69" s="98"/>
@@ -10473,7 +10550,7 @@
       <c r="AH69" s="98"/>
       <c r="AI69" s="98"/>
     </row>
-    <row r="70" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="70" spans="1:35">
       <c r="A70" s="98"/>
       <c r="B70" s="98"/>
       <c r="C70" s="98"/>
@@ -10510,7 +10587,7 @@
       <c r="AH70" s="98"/>
       <c r="AI70" s="98"/>
     </row>
-    <row r="71" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="71" spans="1:35">
       <c r="A71" s="98"/>
       <c r="B71" s="98"/>
       <c r="C71" s="98"/>
@@ -10547,7 +10624,7 @@
       <c r="AH71" s="98"/>
       <c r="AI71" s="98"/>
     </row>
-    <row r="72" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="72" spans="1:35">
       <c r="A72" s="98"/>
       <c r="B72" s="98"/>
       <c r="C72" s="98"/>
@@ -10584,22 +10661,30 @@
       <c r="AH72" s="98"/>
       <c r="AI72" s="98"/>
     </row>
-    <row r="73" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="73" spans="1:35">
+      <c r="B73" s="66">
+        <f>AVERAGE(B3,B11,B21,B23,B28,B30,B36,B45,B63,B64,B65,B67)</f>
+        <v>26.833333333333332</v>
+      </c>
+      <c r="D73">
+        <f>_xlfn.STDEV.P(B3,B11,B21,B23,B28,B30,B36,B45,B63,B64,B65,B67)</f>
+        <v>5.6984403324262525</v>
+      </c>
       <c r="R73" s="98"/>
       <c r="AG73"/>
       <c r="AH73"/>
     </row>
-    <row r="74" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="74" spans="1:35">
       <c r="R74" s="98"/>
       <c r="AG74"/>
       <c r="AH74"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait"/>
-  <legacyDrawing r:id="rId1"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
+  <legacyDrawing r:id="rId2"/>
   <tableParts count="1">
-    <tablePart r:id="rId2"/>
+    <tablePart r:id="rId3"/>
   </tableParts>
 </worksheet>
 </file>
@@ -10607,9 +10692,9 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:D3"/>
-  <sheetFormatPr defaultColWidth="8.7265625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultColWidth="8.7265625" defaultRowHeight="14.5"/>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:4">
       <c r="B1" t="s">
         <v>220</v>
       </c>
@@ -10620,7 +10705,7 @@
         <v>222</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:4">
       <c r="A2" t="s">
         <v>223</v>
       </c>
@@ -10634,7 +10719,7 @@
         <v>0.5</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:4">
       <c r="A3" t="s">
         <v>224</v>
       </c>
@@ -10647,12 +10732,12 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:O23"/>
-  <sheetFormatPr defaultColWidth="8.7265625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultColWidth="8.7265625" defaultRowHeight="14.5"/>
   <cols>
     <col min="1" max="15" width="14.26953125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" s="43" customFormat="1" ht="57" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:15" s="43" customFormat="1" ht="57" customHeight="1">
       <c r="A1" s="43" t="s">
         <v>0</v>
       </c>
@@ -10699,7 +10784,7 @@
         <v>238</v>
       </c>
     </row>
-    <row r="2" spans="1:15" s="43" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:15" s="43" customFormat="1">
       <c r="A2" s="48" t="s">
         <v>204</v>
       </c>
@@ -10746,7 +10831,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:15">
       <c r="A3" s="49" t="s">
         <v>206</v>
       </c>
@@ -10793,7 +10878,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:15">
       <c r="A4" s="49" t="s">
         <v>209</v>
       </c>
@@ -10840,7 +10925,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:15">
       <c r="A5" s="49" t="s">
         <v>200</v>
       </c>
@@ -10887,7 +10972,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:15">
       <c r="A6" s="49" t="s">
         <v>197</v>
       </c>
@@ -10934,7 +11019,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:15">
       <c r="A7" s="49" t="s">
         <v>194</v>
       </c>
@@ -10981,7 +11066,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="8" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:15">
       <c r="A8" s="49" t="s">
         <v>190</v>
       </c>
@@ -11028,7 +11113,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="9" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:15">
       <c r="A9" s="49" t="s">
         <v>187</v>
       </c>
@@ -11075,7 +11160,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="10" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:15">
       <c r="A10" s="49" t="s">
         <v>177</v>
       </c>
@@ -11122,7 +11207,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="11" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:15">
       <c r="A11" s="49" t="s">
         <v>174</v>
       </c>
@@ -11169,7 +11254,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="12" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:15">
       <c r="A12" s="49" t="s">
         <v>169</v>
       </c>
@@ -11216,7 +11301,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="13" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:15">
       <c r="A13" s="49" t="s">
         <v>162</v>
       </c>
@@ -11263,7 +11348,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="14" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:15">
       <c r="A14" s="49" t="s">
         <v>156</v>
       </c>
@@ -11310,7 +11395,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="15" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:15">
       <c r="A15" s="49" t="s">
         <v>212</v>
       </c>
@@ -11357,7 +11442,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="16" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:15">
       <c r="A16" s="49" t="s">
         <v>215</v>
       </c>
@@ -11404,31 +11489,31 @@
         <v>1</v>
       </c>
     </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:6">
       <c r="A17" s="49"/>
       <c r="F17" s="52"/>
     </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:6">
       <c r="A18" s="49"/>
       <c r="F18" s="52"/>
     </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:6">
       <c r="A19" s="49"/>
       <c r="F19" s="52"/>
     </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:6">
       <c r="A20" s="49"/>
       <c r="F20" s="52"/>
     </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:6">
       <c r="A21" s="49"/>
       <c r="F21" s="52"/>
     </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:6">
       <c r="A22" s="49"/>
       <c r="F22" s="52"/>
     </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:6">
       <c r="A23" s="49"/>
     </row>
   </sheetData>
@@ -11442,7 +11527,7 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:AJ23"/>
-  <sheetFormatPr defaultColWidth="14.453125" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultColWidth="14.453125" defaultRowHeight="14.5"/>
   <cols>
     <col min="1" max="16" width="25.453125" style="41" customWidth="1"/>
     <col min="17" max="17" width="25.453125" style="44" customWidth="1"/>
@@ -11455,7 +11540,7 @@
     <col min="36" max="16384" width="14.453125" style="41"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:36" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:36" ht="18" customHeight="1">
       <c r="B1" s="42" t="s">
         <v>239</v>
       </c>
@@ -11469,7 +11554,7 @@
         <v>242</v>
       </c>
     </row>
-    <row r="2" spans="1:36" s="43" customFormat="1" ht="90" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:36" s="43" customFormat="1" ht="90" customHeight="1">
       <c r="A2" s="43" t="s">
         <v>0</v>
       </c>
@@ -11579,7 +11664,7 @@
         <v>277</v>
       </c>
     </row>
-    <row r="3" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:36">
       <c r="A3" s="77" t="s">
         <v>156</v>
       </c>
@@ -11691,7 +11776,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="4" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:36">
       <c r="A4" s="77" t="s">
         <v>162</v>
       </c>
@@ -11800,7 +11885,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="5" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:36">
       <c r="A5" s="77" t="s">
         <v>169</v>
       </c>
@@ -11906,7 +11991,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="6" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:36">
       <c r="A6" s="79" t="s">
         <v>174</v>
       </c>
@@ -12015,7 +12100,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="7" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:36">
       <c r="A7" s="79" t="s">
         <v>177</v>
       </c>
@@ -12116,7 +12201,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="8" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:36">
       <c r="A8" s="81" t="s">
         <v>181</v>
       </c>
@@ -12124,7 +12209,7 @@
       <c r="W8" s="41"/>
       <c r="AA8" s="41"/>
     </row>
-    <row r="9" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:36">
       <c r="A9" s="41" t="s">
         <v>187</v>
       </c>
@@ -12222,7 +12307,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="10" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:36">
       <c r="A10" s="41" t="s">
         <v>194</v>
       </c>
@@ -12334,7 +12419,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="11" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:36">
       <c r="A11" s="78" t="s">
         <v>197</v>
       </c>
@@ -12446,7 +12531,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="12" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:36">
       <c r="A12" s="49" t="s">
         <v>200</v>
       </c>
@@ -12552,7 +12637,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="13" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:36">
       <c r="A13" s="78" t="s">
         <v>204</v>
       </c>
@@ -12664,7 +12749,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="14" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:36">
       <c r="A14" s="49" t="s">
         <v>206</v>
       </c>
@@ -12770,7 +12855,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="15" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:36">
       <c r="A15" s="78" t="s">
         <v>209</v>
       </c>
@@ -12876,7 +12961,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="16" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:36">
       <c r="A16" s="49" t="s">
         <v>212</v>
       </c>
@@ -12988,7 +13073,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="17" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:36">
       <c r="A17" s="78" t="s">
         <v>215</v>
       </c>
@@ -13096,7 +13181,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="19" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:36">
       <c r="AH19" s="41" t="s">
         <v>278</v>
       </c>
@@ -13109,7 +13194,7 @@
         <v>31.5</v>
       </c>
     </row>
-    <row r="20" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:36">
       <c r="AH20" s="41" t="s">
         <v>279</v>
       </c>
@@ -13122,7 +13207,7 @@
         <v>1.5566235649883124</v>
       </c>
     </row>
-    <row r="21" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:36">
       <c r="AH21" s="41" t="s">
         <v>280</v>
       </c>
@@ -13135,7 +13220,7 @@
         <v>31.5</v>
       </c>
     </row>
-    <row r="22" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:36">
       <c r="AH22" s="41" t="s">
         <v>281</v>
       </c>
@@ -13148,7 +13233,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="23" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:36">
       <c r="AH23" s="41" t="s">
         <v>282</v>
       </c>
@@ -13173,7 +13258,7 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A1:AR24"/>
-  <sheetFormatPr defaultColWidth="8.7265625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultColWidth="8.7265625" defaultRowHeight="14.5"/>
   <cols>
     <col min="1" max="1" width="21.26953125" style="49" customWidth="1"/>
     <col min="2" max="8" width="14.1796875" customWidth="1"/>
@@ -13190,7 +13275,7 @@
     <col min="44" max="51" width="15.81640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:44" s="43" customFormat="1" ht="180" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:44" s="43" customFormat="1" ht="180" customHeight="1">
       <c r="A1" s="48" t="s">
         <v>283</v>
       </c>
@@ -13324,7 +13409,7 @@
         <v>326</v>
       </c>
     </row>
-    <row r="2" spans="1:44" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:44">
       <c r="A2" t="s">
         <v>327</v>
       </c>
@@ -13464,7 +13549,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:44" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:44">
       <c r="A3" t="s">
         <v>328</v>
       </c>
@@ -13604,7 +13689,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="4" spans="1:44" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:44">
       <c r="A4" t="s">
         <v>329</v>
       </c>
@@ -13744,7 +13829,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="5" spans="1:44" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:44">
       <c r="A5" t="s">
         <v>330</v>
       </c>
@@ -13884,7 +13969,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="6" spans="1:44" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:44">
       <c r="A6" t="s">
         <v>331</v>
       </c>
@@ -14024,7 +14109,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="7" spans="1:44" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:44">
       <c r="A7" t="s">
         <v>332</v>
       </c>
@@ -14164,7 +14249,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="8" spans="1:44" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:44">
       <c r="A8" t="s">
         <v>333</v>
       </c>
@@ -14304,7 +14389,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="9" spans="1:44" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:44">
       <c r="A9" s="49" t="s">
         <v>334</v>
       </c>
@@ -14444,7 +14529,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="10" spans="1:44" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:44">
       <c r="A10" s="49" t="s">
         <v>335</v>
       </c>
@@ -14584,7 +14669,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="11" spans="1:44" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:44">
       <c r="A11" s="49" t="s">
         <v>336</v>
       </c>
@@ -14724,7 +14809,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="12" spans="1:44" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:44">
       <c r="A12" s="49" t="s">
         <v>337</v>
       </c>
@@ -14864,7 +14949,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="13" spans="1:44" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:44">
       <c r="A13" s="49" t="s">
         <v>338</v>
       </c>
@@ -15004,7 +15089,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="14" spans="1:44" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:44">
       <c r="A14" s="49" t="s">
         <v>339</v>
       </c>
@@ -15144,7 +15229,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="15" spans="1:44" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:44">
       <c r="A15" t="s">
         <v>340</v>
       </c>
@@ -15281,7 +15366,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="16" spans="1:44" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:44">
       <c r="A16" s="3" t="s">
         <v>341</v>
       </c>
@@ -15421,7 +15506,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="17" spans="1:44" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:44">
       <c r="I17" s="82"/>
       <c r="T17" s="82"/>
       <c r="Z17" s="82"/>
@@ -15429,7 +15514,7 @@
       <c r="AL17" s="82"/>
       <c r="AR17" s="82"/>
     </row>
-    <row r="18" spans="1:44" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:44">
       <c r="I18" s="84"/>
       <c r="T18" s="84"/>
       <c r="Z18" s="84"/>
@@ -15437,7 +15522,7 @@
       <c r="AL18" s="84"/>
       <c r="AR18" s="84"/>
     </row>
-    <row r="19" spans="1:44" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:44">
       <c r="A19" s="49" t="s">
         <v>342</v>
       </c>
@@ -15614,7 +15699,7 @@
         <v>47.666666666666664</v>
       </c>
     </row>
-    <row r="20" spans="1:44" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:44">
       <c r="A20" s="49" t="s">
         <v>343</v>
       </c>
@@ -15791,7 +15876,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="21" spans="1:44" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:44">
       <c r="A21" s="49" t="s">
         <v>344</v>
       </c>
@@ -15950,7 +16035,7 @@
       </c>
       <c r="AR21" s="84"/>
     </row>
-    <row r="22" spans="1:44" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:44">
       <c r="A22" s="49" t="s">
         <v>279</v>
       </c>
@@ -16127,7 +16212,7 @@
         <v>20.254335220838414</v>
       </c>
     </row>
-    <row r="23" spans="1:44" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:44">
       <c r="A23" s="49" t="s">
         <v>345</v>
       </c>
@@ -16304,7 +16389,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="24" spans="1:44" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:44">
       <c r="A24" s="49" t="s">
         <v>282</v>
       </c>
@@ -16494,14 +16579,14 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
   <dimension ref="A1:AG80"/>
-  <sheetFormatPr defaultColWidth="8.7265625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultColWidth="8.7265625" defaultRowHeight="14.5"/>
   <cols>
     <col min="1" max="1" width="10" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="9.453125" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="10" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:33" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:33">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -16602,13 +16687,13 @@
         <v>376</v>
       </c>
     </row>
-    <row r="2" spans="1:33" hidden="1" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:33" hidden="1">
       <c r="A2" s="41" t="s">
         <v>34</v>
       </c>
       <c r="B2" s="41"/>
     </row>
-    <row r="3" spans="1:33" hidden="1" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:33" hidden="1">
       <c r="A3" s="56" t="s">
         <v>40</v>
       </c>
@@ -16616,7 +16701,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="4" spans="1:33" hidden="1" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:33" hidden="1">
       <c r="A4" s="56" t="s">
         <v>47</v>
       </c>
@@ -16624,7 +16709,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="5" spans="1:33" hidden="1" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:33" hidden="1">
       <c r="A5" s="56" t="s">
         <v>49</v>
       </c>
@@ -16632,7 +16717,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="6" spans="1:33" hidden="1" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:33" hidden="1">
       <c r="A6" s="56" t="s">
         <v>51</v>
       </c>
@@ -16640,7 +16725,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="7" spans="1:33" hidden="1" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:33" hidden="1">
       <c r="A7" s="56" t="s">
         <v>53</v>
       </c>
@@ -16648,7 +16733,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="8" spans="1:33" hidden="1" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:33" hidden="1">
       <c r="A8" s="56" t="s">
         <v>55</v>
       </c>
@@ -16656,7 +16741,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="9" spans="1:33" hidden="1" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:33" hidden="1">
       <c r="A9" s="57" t="s">
         <v>58</v>
       </c>
@@ -16664,7 +16749,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="10" spans="1:33" hidden="1" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:33" hidden="1">
       <c r="A10" s="56" t="s">
         <v>59</v>
       </c>
@@ -16672,7 +16757,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="11" spans="1:33" hidden="1" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:33" hidden="1">
       <c r="A11" s="57" t="s">
         <v>62</v>
       </c>
@@ -16680,7 +16765,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="12" spans="1:33" hidden="1" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:33" hidden="1">
       <c r="A12" s="57" t="s">
         <v>64</v>
       </c>
@@ -16688,7 +16773,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="13" spans="1:33" hidden="1" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:33" hidden="1">
       <c r="A13" s="56" t="s">
         <v>65</v>
       </c>
@@ -16696,7 +16781,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="14" spans="1:33" hidden="1" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:33" hidden="1">
       <c r="A14" s="56" t="s">
         <v>67</v>
       </c>
@@ -16704,7 +16789,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="15" spans="1:33" hidden="1" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:33" hidden="1">
       <c r="A15" s="56" t="s">
         <v>69</v>
       </c>
@@ -16712,7 +16797,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="16" spans="1:33" hidden="1" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:33" hidden="1">
       <c r="A16" s="57" t="s">
         <v>71</v>
       </c>
@@ -16720,7 +16805,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="17" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:2" hidden="1">
       <c r="A17" s="56" t="s">
         <v>73</v>
       </c>
@@ -16728,7 +16813,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="18" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:2" hidden="1">
       <c r="A18" s="56" t="s">
         <v>75</v>
       </c>
@@ -16736,7 +16821,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="19" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:2" hidden="1">
       <c r="A19" s="56" t="s">
         <v>78</v>
       </c>
@@ -16744,7 +16829,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="20" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:2" hidden="1">
       <c r="A20" s="70" t="s">
         <v>81</v>
       </c>
@@ -16752,7 +16837,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="21" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:2" hidden="1">
       <c r="A21" s="61" t="s">
         <v>85</v>
       </c>
@@ -16760,7 +16845,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="22" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:2" hidden="1">
       <c r="A22" s="61" t="s">
         <v>87</v>
       </c>
@@ -16768,7 +16853,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="23" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:2" hidden="1">
       <c r="A23" s="71" t="s">
         <v>89</v>
       </c>
@@ -16776,7 +16861,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="24" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:2" hidden="1">
       <c r="A24" s="61" t="s">
         <v>91</v>
       </c>
@@ -16784,7 +16869,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="25" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:2" hidden="1">
       <c r="A25" s="61" t="s">
         <v>94</v>
       </c>
@@ -16792,7 +16877,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="26" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:2" hidden="1">
       <c r="A26" s="61" t="s">
         <v>96</v>
       </c>
@@ -16800,7 +16885,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="27" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:2" hidden="1">
       <c r="A27" s="69" t="s">
         <v>98</v>
       </c>
@@ -16808,7 +16893,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="28" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:2" hidden="1">
       <c r="A28" s="61" t="s">
         <v>100</v>
       </c>
@@ -16816,7 +16901,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="29" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:2" hidden="1">
       <c r="A29" s="61" t="s">
         <v>102</v>
       </c>
@@ -16824,7 +16909,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="30" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:2" hidden="1">
       <c r="A30" s="61" t="s">
         <v>104</v>
       </c>
@@ -16832,7 +16917,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="31" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:2" hidden="1">
       <c r="A31" s="61" t="s">
         <v>107</v>
       </c>
@@ -16840,7 +16925,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="32" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:2" hidden="1">
       <c r="A32" s="62" t="s">
         <v>109</v>
       </c>
@@ -16848,7 +16933,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="33" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:2" hidden="1">
       <c r="A33" s="61" t="s">
         <v>112</v>
       </c>
@@ -16856,7 +16941,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="34" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:2" hidden="1">
       <c r="A34" s="61" t="s">
         <v>116</v>
       </c>
@@ -16864,7 +16949,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="35" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:2" hidden="1">
       <c r="A35" s="61" t="s">
         <v>119</v>
       </c>
@@ -16872,7 +16957,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="36" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:2" hidden="1">
       <c r="A36" s="61" t="s">
         <v>122</v>
       </c>
@@ -16880,7 +16965,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="37" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:2" hidden="1">
       <c r="A37" s="61" t="s">
         <v>125</v>
       </c>
@@ -16888,7 +16973,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="38" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:2" hidden="1">
       <c r="A38" s="61" t="s">
         <v>127</v>
       </c>
@@ -16896,7 +16981,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="39" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:2" hidden="1">
       <c r="A39" s="61" t="s">
         <v>129</v>
       </c>
@@ -16904,7 +16989,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="40" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:2" hidden="1">
       <c r="A40" s="61" t="s">
         <v>131</v>
       </c>
@@ -16912,7 +16997,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="41" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:2" hidden="1">
       <c r="A41" s="61" t="s">
         <v>134</v>
       </c>
@@ -16920,7 +17005,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="42" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:2" hidden="1">
       <c r="A42" s="62" t="s">
         <v>136</v>
       </c>
@@ -16928,7 +17013,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="43" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:2" hidden="1">
       <c r="A43" s="61" t="s">
         <v>137</v>
       </c>
@@ -16936,7 +17021,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="44" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:2" hidden="1">
       <c r="A44" s="61" t="s">
         <v>140</v>
       </c>
@@ -16944,7 +17029,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="45" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:2" hidden="1">
       <c r="A45" s="61" t="s">
         <v>143</v>
       </c>
@@ -16952,7 +17037,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="46" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:2" hidden="1">
       <c r="A46" s="61" t="s">
         <v>145</v>
       </c>
@@ -16960,7 +17045,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="47" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:2" hidden="1">
       <c r="A47" s="61" t="s">
         <v>147</v>
       </c>
@@ -16968,7 +17053,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="48" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:2" hidden="1">
       <c r="A48" s="61" t="s">
         <v>150</v>
       </c>
@@ -16976,7 +17061,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="49" spans="1:33" hidden="1" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:33" hidden="1">
       <c r="A49" s="61" t="s">
         <v>152</v>
       </c>
@@ -16984,7 +17069,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="50" spans="1:33" hidden="1" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:33" hidden="1">
       <c r="A50" s="61" t="s">
         <v>153</v>
       </c>
@@ -16992,7 +17077,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="51" spans="1:33" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:33">
       <c r="A51" s="56" t="s">
         <v>156</v>
       </c>
@@ -17090,7 +17175,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="52" spans="1:33" hidden="1" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:33" hidden="1">
       <c r="A52" s="61" t="s">
         <v>159</v>
       </c>
@@ -17098,7 +17183,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="53" spans="1:33" hidden="1" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:33" hidden="1">
       <c r="A53" s="61" t="s">
         <v>160</v>
       </c>
@@ -17106,7 +17191,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="54" spans="1:33" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:33">
       <c r="A54" s="56" t="s">
         <v>162</v>
       </c>
@@ -17204,7 +17289,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="55" spans="1:33" hidden="1" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:33" hidden="1">
       <c r="A55" s="61" t="s">
         <v>165</v>
       </c>
@@ -17212,7 +17297,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="56" spans="1:33" hidden="1" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:33" hidden="1">
       <c r="A56" s="61" t="s">
         <v>168</v>
       </c>
@@ -17304,7 +17389,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="57" spans="1:33" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:33">
       <c r="A57" s="56" t="s">
         <v>169</v>
       </c>
@@ -17402,7 +17487,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="58" spans="1:33" hidden="1" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:33" hidden="1">
       <c r="A58" s="61" t="s">
         <v>172</v>
       </c>
@@ -17410,7 +17495,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="59" spans="1:33" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:33">
       <c r="A59" s="80" t="s">
         <v>174</v>
       </c>
@@ -17508,7 +17593,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="60" spans="1:33" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:33">
       <c r="A60" s="56" t="s">
         <v>177</v>
       </c>
@@ -17606,7 +17691,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="61" spans="1:33" hidden="1" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:33" hidden="1">
       <c r="A61" s="61" t="s">
         <v>180</v>
       </c>
@@ -17704,7 +17789,7 @@
         <v>0.5</v>
       </c>
     </row>
-    <row r="62" spans="1:33" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:33">
       <c r="A62" s="80" t="s">
         <v>181</v>
       </c>
@@ -17802,7 +17887,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="63" spans="1:33" hidden="1" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:33" hidden="1">
       <c r="A63" s="61" t="s">
         <v>184</v>
       </c>
@@ -17810,7 +17895,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="64" spans="1:33" hidden="1" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:33" hidden="1">
       <c r="A64" s="62" t="s">
         <v>185</v>
       </c>
@@ -17818,7 +17903,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="65" spans="1:33" hidden="1" x14ac:dyDescent="0.35">
+    <row r="65" spans="1:33" hidden="1">
       <c r="A65" s="61" t="s">
         <v>186</v>
       </c>
@@ -17826,7 +17911,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="66" spans="1:33" x14ac:dyDescent="0.35">
+    <row r="66" spans="1:33">
       <c r="A66" s="56" t="s">
         <v>187</v>
       </c>
@@ -17924,7 +18009,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="67" spans="1:33" hidden="1" x14ac:dyDescent="0.35">
+    <row r="67" spans="1:33" hidden="1">
       <c r="A67" s="61" t="s">
         <v>190</v>
       </c>
@@ -17932,7 +18017,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="68" spans="1:33" x14ac:dyDescent="0.35">
+    <row r="68" spans="1:33">
       <c r="A68" s="56" t="s">
         <v>194</v>
       </c>
@@ -18030,7 +18115,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="69" spans="1:33" x14ac:dyDescent="0.35">
+    <row r="69" spans="1:33">
       <c r="A69" s="80" t="s">
         <v>197</v>
       </c>
@@ -18128,7 +18213,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="70" spans="1:33" x14ac:dyDescent="0.35">
+    <row r="70" spans="1:33">
       <c r="A70" s="56" t="s">
         <v>200</v>
       </c>
@@ -18226,7 +18311,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="71" spans="1:33" x14ac:dyDescent="0.35">
+    <row r="71" spans="1:33">
       <c r="A71" s="56" t="s">
         <v>204</v>
       </c>
@@ -18324,7 +18409,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="72" spans="1:33" x14ac:dyDescent="0.35">
+    <row r="72" spans="1:33">
       <c r="A72" s="56" t="s">
         <v>206</v>
       </c>
@@ -18422,7 +18507,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="73" spans="1:33" x14ac:dyDescent="0.35">
+    <row r="73" spans="1:33">
       <c r="A73" s="56" t="s">
         <v>209</v>
       </c>
@@ -18520,7 +18605,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="74" spans="1:33" x14ac:dyDescent="0.35">
+    <row r="74" spans="1:33">
       <c r="A74" s="56" t="s">
         <v>212</v>
       </c>
@@ -18618,7 +18703,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="75" spans="1:33" x14ac:dyDescent="0.35">
+    <row r="75" spans="1:33">
       <c r="A75" s="80" t="s">
         <v>215</v>
       </c>
@@ -18713,7 +18798,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="77" spans="1:33" x14ac:dyDescent="0.35">
+    <row r="77" spans="1:33">
       <c r="A77" t="s">
         <v>278</v>
       </c>
@@ -18839,7 +18924,7 @@
         <v>0.36666666666666664</v>
       </c>
     </row>
-    <row r="78" spans="1:33" x14ac:dyDescent="0.35">
+    <row r="78" spans="1:33">
       <c r="A78" t="s">
         <v>377</v>
       </c>
@@ -18965,7 +19050,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="79" spans="1:33" x14ac:dyDescent="0.35">
+    <row r="79" spans="1:33">
       <c r="A79" t="s">
         <v>282</v>
       </c>
@@ -18986,7 +19071,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="80" spans="1:33" x14ac:dyDescent="0.35">
+    <row r="80" spans="1:33">
       <c r="A80" t="s">
         <v>378</v>
       </c>
@@ -19019,12 +19104,12 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
   <dimension ref="A1:CA99"/>
-  <sheetFormatPr defaultColWidth="8.7265625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultColWidth="8.7265625" defaultRowHeight="14.5"/>
   <cols>
     <col min="1" max="1" width="20.1796875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:79" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:79" ht="15.75" customHeight="1" thickBot="1">
       <c r="A1" s="13" t="s">
         <v>379</v>
       </c>
@@ -19263,7 +19348,7 @@
         <v>457</v>
       </c>
     </row>
-    <row r="2" spans="1:79" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:79" ht="15.75" customHeight="1" thickBot="1">
       <c r="A2" s="19" t="s">
         <v>458</v>
       </c>
@@ -19493,7 +19578,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="3" spans="1:79" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:79">
       <c r="A3" s="20" t="s">
         <v>459</v>
       </c>
@@ -19521,7 +19606,7 @@
       <c r="BO3" s="9"/>
       <c r="BT3" s="9"/>
     </row>
-    <row r="4" spans="1:79" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:79">
       <c r="A4" s="1" t="s">
         <v>460</v>
       </c>
@@ -19740,7 +19825,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:79" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:79">
       <c r="A5" s="1" t="s">
         <v>466</v>
       </c>
@@ -19959,7 +20044,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:79" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:79" ht="15.75" customHeight="1" thickBot="1">
       <c r="A6" s="31" t="s">
         <v>468</v>
       </c>
@@ -20184,7 +20269,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="1:79" ht="15.75" customHeight="1" thickTop="1" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:79" ht="15.75" customHeight="1" thickTop="1">
       <c r="A7" s="1" t="s">
         <v>469</v>
       </c>
@@ -20401,7 +20486,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="8" spans="1:79" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:79">
       <c r="A8" s="1" t="s">
         <v>471</v>
       </c>
@@ -20618,7 +20703,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="9" spans="1:79" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="9" spans="1:79" ht="15.75" customHeight="1" thickBot="1">
       <c r="A9" s="31" t="s">
         <v>472</v>
       </c>
@@ -20841,7 +20926,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="10" spans="1:79" ht="15.75" customHeight="1" thickTop="1" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:79" ht="15.75" customHeight="1" thickTop="1">
       <c r="A10" t="s">
         <v>474</v>
       </c>
@@ -21055,7 +21140,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="11" spans="1:79" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:79">
       <c r="A11" t="s">
         <v>477</v>
       </c>
@@ -21272,7 +21357,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="12" spans="1:79" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="12" spans="1:79" ht="15.75" customHeight="1" thickBot="1">
       <c r="A12" s="32" t="s">
         <v>479</v>
       </c>
@@ -21493,7 +21578,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="13" spans="1:79" ht="15.75" customHeight="1" thickTop="1" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:79" ht="15.75" customHeight="1" thickTop="1">
       <c r="A13" t="s">
         <v>480</v>
       </c>
@@ -21710,7 +21795,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="14" spans="1:79" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:79">
       <c r="A14" t="s">
         <v>482</v>
       </c>
@@ -21927,7 +22012,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="15" spans="1:79" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="15" spans="1:79" ht="15.75" customHeight="1" thickBot="1">
       <c r="A15" s="32" t="s">
         <v>483</v>
       </c>
@@ -22150,7 +22235,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="16" spans="1:79" ht="15.75" customHeight="1" thickTop="1" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:79" ht="15.75" customHeight="1" thickTop="1">
       <c r="A16" t="s">
         <v>484</v>
       </c>
@@ -22367,7 +22452,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="17" spans="1:79" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:79">
       <c r="A17" t="s">
         <v>485</v>
       </c>
@@ -22584,7 +22669,7 @@
         <v>486</v>
       </c>
     </row>
-    <row r="18" spans="1:79" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="18" spans="1:79" ht="15.75" customHeight="1" thickBot="1">
       <c r="A18" s="32" t="s">
         <v>487</v>
       </c>
@@ -22807,7 +22892,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="19" spans="1:79" ht="15.75" customHeight="1" thickTop="1" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:79" ht="15.75" customHeight="1" thickTop="1">
       <c r="A19" t="s">
         <v>488</v>
       </c>
@@ -23024,7 +23109,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="20" spans="1:79" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:79">
       <c r="A20" t="s">
         <v>490</v>
       </c>
@@ -23241,7 +23326,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="21" spans="1:79" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="21" spans="1:79" ht="15.75" customHeight="1" thickBot="1">
       <c r="A21" s="32" t="s">
         <v>491</v>
       </c>
@@ -23464,7 +23549,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="22" spans="1:79" ht="15.75" customHeight="1" thickTop="1" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:79" ht="15.75" customHeight="1" thickTop="1">
       <c r="A22" t="s">
         <v>492</v>
       </c>
@@ -23679,7 +23764,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="23" spans="1:79" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:79">
       <c r="A23" t="s">
         <v>494</v>
       </c>
@@ -23894,7 +23979,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="24" spans="1:79" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="24" spans="1:79" ht="15.75" customHeight="1" thickBot="1">
       <c r="A24" s="32" t="s">
         <v>495</v>
       </c>
@@ -24115,7 +24200,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="25" spans="1:79" ht="15.75" customHeight="1" thickTop="1" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:79" ht="15.75" customHeight="1" thickTop="1">
       <c r="A25" t="s">
         <v>496</v>
       </c>
@@ -24328,7 +24413,7 @@
         <v>467</v>
       </c>
     </row>
-    <row r="26" spans="1:79" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:79">
       <c r="A26" t="s">
         <v>497</v>
       </c>
@@ -24541,7 +24626,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="27" spans="1:79" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="27" spans="1:79" ht="15.75" customHeight="1" thickBot="1">
       <c r="A27" s="32" t="s">
         <v>499</v>
       </c>
@@ -24760,7 +24845,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="28" spans="1:79" ht="15.75" customHeight="1" thickTop="1" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:79" ht="15.75" customHeight="1" thickTop="1">
       <c r="A28" t="s">
         <v>500</v>
       </c>
@@ -24973,7 +25058,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="29" spans="1:79" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:79">
       <c r="A29" t="s">
         <v>501</v>
       </c>
@@ -25186,7 +25271,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="30" spans="1:79" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="30" spans="1:79" ht="15.75" customHeight="1" thickBot="1">
       <c r="A30" s="32" t="s">
         <v>502</v>
       </c>
@@ -25405,7 +25490,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="31" spans="1:79" ht="15.75" customHeight="1" thickTop="1" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:79" ht="15.75" customHeight="1" thickTop="1">
       <c r="A31" t="s">
         <v>504</v>
       </c>
@@ -25618,7 +25703,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="32" spans="1:79" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:79">
       <c r="A32" t="s">
         <v>505</v>
       </c>
@@ -25831,7 +25916,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="33" spans="1:79" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="33" spans="1:79" ht="15.75" customHeight="1" thickBot="1">
       <c r="A33" s="32" t="s">
         <v>506</v>
       </c>
@@ -26050,7 +26135,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="34" spans="1:79" ht="15.75" customHeight="1" thickTop="1" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:79" ht="15.75" customHeight="1" thickTop="1">
       <c r="A34" t="s">
         <v>507</v>
       </c>
@@ -26261,7 +26346,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="35" spans="1:79" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:79">
       <c r="A35" t="s">
         <v>508</v>
       </c>
@@ -26472,7 +26557,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="36" spans="1:79" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="36" spans="1:79" ht="15.75" customHeight="1" thickBot="1">
       <c r="A36" s="32" t="s">
         <v>509</v>
       </c>
@@ -26689,7 +26774,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="37" spans="1:79" ht="15.75" customHeight="1" thickTop="1" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:79" ht="15.75" customHeight="1" thickTop="1">
       <c r="A37" t="s">
         <v>510</v>
       </c>
@@ -26900,7 +26985,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="38" spans="1:79" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:79">
       <c r="A38" t="s">
         <v>511</v>
       </c>
@@ -27111,7 +27196,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="39" spans="1:79" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="39" spans="1:79" ht="15.75" customHeight="1" thickBot="1">
       <c r="A39" s="32" t="s">
         <v>512</v>
       </c>
@@ -27328,7 +27413,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="40" spans="1:79" ht="15.75" customHeight="1" thickTop="1" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:79" ht="15.75" customHeight="1" thickTop="1">
       <c r="A40" t="s">
         <v>513</v>
       </c>
@@ -27539,7 +27624,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="41" spans="1:79" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:79">
       <c r="A41" t="s">
         <v>514</v>
       </c>
@@ -27750,7 +27835,7 @@
         <v>486</v>
       </c>
     </row>
-    <row r="42" spans="1:79" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="42" spans="1:79" ht="15.75" customHeight="1" thickBot="1">
       <c r="A42" s="32" t="s">
         <v>515</v>
       </c>
@@ -27967,7 +28052,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="43" spans="1:79" ht="15.75" customHeight="1" thickTop="1" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:79" ht="15.75" customHeight="1" thickTop="1">
       <c r="A43" t="s">
         <v>516</v>
       </c>
@@ -28180,7 +28265,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="44" spans="1:79" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:79">
       <c r="A44" t="s">
         <v>517</v>
       </c>
@@ -28393,7 +28478,7 @@
         <v>486</v>
       </c>
     </row>
-    <row r="45" spans="1:79" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="45" spans="1:79" ht="15.75" customHeight="1" thickBot="1">
       <c r="A45" s="32" t="s">
         <v>518</v>
       </c>
@@ -28612,7 +28697,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="46" spans="1:79" ht="15.75" customHeight="1" thickTop="1" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:79" ht="15.75" customHeight="1" thickTop="1">
       <c r="A46" t="s">
         <v>519</v>
       </c>
@@ -28802,7 +28887,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="47" spans="1:79" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:79">
       <c r="A47" t="s">
         <v>520</v>
       </c>
@@ -28992,7 +29077,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="48" spans="1:79" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="48" spans="1:79" ht="15.75" customHeight="1" thickBot="1">
       <c r="A48" s="37" t="s">
         <v>521</v>
       </c>
@@ -29195,7 +29280,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="49" spans="1:79" ht="15.75" customHeight="1" thickTop="1" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:79" ht="15.75" customHeight="1" thickTop="1">
       <c r="A49" t="s">
         <v>522</v>
       </c>
@@ -29367,7 +29452,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="50" spans="1:79" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:79">
       <c r="A50" t="s">
         <v>523</v>
       </c>
@@ -29539,7 +29624,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="51" spans="1:79" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="51" spans="1:79" ht="15.75" customHeight="1" thickBot="1">
       <c r="A51" s="37" t="s">
         <v>524</v>
       </c>
@@ -29730,7 +29815,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="52" spans="1:79" ht="15.75" customHeight="1" thickTop="1" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:79" ht="15.75" customHeight="1" thickTop="1">
       <c r="A52" t="s">
         <v>525</v>
       </c>
@@ -29899,7 +29984,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="53" spans="1:79" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:79">
       <c r="A53" t="s">
         <v>526</v>
       </c>
@@ -30068,7 +30153,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="54" spans="1:79" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="54" spans="1:79" ht="15.75" customHeight="1" thickBot="1">
       <c r="A54" t="s">
         <v>527</v>
       </c>
@@ -30237,7 +30322,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="55" spans="1:79" ht="15.75" customHeight="1" thickTop="1" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:79" ht="15.75" customHeight="1" thickTop="1">
       <c r="A55" s="72" t="s">
         <v>528</v>
       </c>
@@ -30474,7 +30559,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="56" spans="1:79" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:79">
       <c r="A56" t="s">
         <v>529</v>
       </c>
@@ -30710,7 +30795,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="57" spans="1:79" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="57" spans="1:79" ht="15.75" customHeight="1" thickBot="1">
       <c r="A57" t="s">
         <v>530</v>
       </c>
@@ -30946,7 +31031,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="58" spans="1:79" ht="15.75" customHeight="1" thickTop="1" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:79" ht="15.75" customHeight="1" thickTop="1">
       <c r="A58" s="7" t="s">
         <v>531</v>
       </c>
@@ -31103,7 +31188,7 @@
       <c r="BZ58" s="7"/>
       <c r="CA58" s="7"/>
     </row>
-    <row r="59" spans="1:79" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:79">
       <c r="A59" t="s">
         <v>532</v>
       </c>
@@ -31227,7 +31312,7 @@
       <c r="BO59" s="9"/>
       <c r="BT59" s="9"/>
     </row>
-    <row r="60" spans="1:79" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:79">
       <c r="A60" t="s">
         <v>533</v>
       </c>
@@ -31351,7 +31436,7 @@
       <c r="BO60" s="9"/>
       <c r="BT60" s="9"/>
     </row>
-    <row r="61" spans="1:79" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:79">
       <c r="A61" t="s">
         <v>534</v>
       </c>
@@ -31475,7 +31560,7 @@
       <c r="BO61" s="9"/>
       <c r="BT61" s="9"/>
     </row>
-    <row r="62" spans="1:79" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:79">
       <c r="A62" t="s">
         <v>535</v>
       </c>
@@ -31599,7 +31684,7 @@
       <c r="BO62" s="9"/>
       <c r="BT62" s="9"/>
     </row>
-    <row r="63" spans="1:79" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:79">
       <c r="A63" t="s">
         <v>536</v>
       </c>
@@ -31631,7 +31716,7 @@
       <c r="BO63" s="9"/>
       <c r="BT63" s="9"/>
     </row>
-    <row r="64" spans="1:79" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:79">
       <c r="A64" t="s">
         <v>537</v>
       </c>
@@ -31755,7 +31840,7 @@
       <c r="BO64" s="9"/>
       <c r="BT64" s="9"/>
     </row>
-    <row r="65" spans="1:79" x14ac:dyDescent="0.35">
+    <row r="65" spans="1:79">
       <c r="A65" t="s">
         <v>538</v>
       </c>
@@ -31879,7 +31964,7 @@
       <c r="BO65" s="9"/>
       <c r="BT65" s="9"/>
     </row>
-    <row r="66" spans="1:79" x14ac:dyDescent="0.35">
+    <row r="66" spans="1:79">
       <c r="A66" t="s">
         <v>539</v>
       </c>
@@ -32003,7 +32088,7 @@
       <c r="BO66" s="9"/>
       <c r="BT66" s="9"/>
     </row>
-    <row r="67" spans="1:79" x14ac:dyDescent="0.35">
+    <row r="67" spans="1:79">
       <c r="A67" t="s">
         <v>540</v>
       </c>
@@ -32127,7 +32212,7 @@
       <c r="BO67" s="9"/>
       <c r="BT67" s="9"/>
     </row>
-    <row r="68" spans="1:79" x14ac:dyDescent="0.35">
+    <row r="68" spans="1:79">
       <c r="A68" t="s">
         <v>541</v>
       </c>
@@ -32251,7 +32336,7 @@
       <c r="BO68" s="9"/>
       <c r="BT68" s="9"/>
     </row>
-    <row r="69" spans="1:79" x14ac:dyDescent="0.35">
+    <row r="69" spans="1:79">
       <c r="A69" t="s">
         <v>542</v>
       </c>
@@ -32375,7 +32460,7 @@
       <c r="BO69" s="9"/>
       <c r="BT69" s="9"/>
     </row>
-    <row r="70" spans="1:79" x14ac:dyDescent="0.35">
+    <row r="70" spans="1:79">
       <c r="A70" t="s">
         <v>543</v>
       </c>
@@ -32499,7 +32584,7 @@
       <c r="BO70" s="9"/>
       <c r="BT70" s="9"/>
     </row>
-    <row r="71" spans="1:79" x14ac:dyDescent="0.35">
+    <row r="71" spans="1:79">
       <c r="A71" t="s">
         <v>544</v>
       </c>
@@ -32623,7 +32708,7 @@
       <c r="BO71" s="9"/>
       <c r="BT71" s="9"/>
     </row>
-    <row r="72" spans="1:79" x14ac:dyDescent="0.35">
+    <row r="72" spans="1:79">
       <c r="A72" t="s">
         <v>545</v>
       </c>
@@ -32747,7 +32832,7 @@
       <c r="BO72" s="9"/>
       <c r="BT72" s="9"/>
     </row>
-    <row r="73" spans="1:79" x14ac:dyDescent="0.35">
+    <row r="73" spans="1:79">
       <c r="A73" t="s">
         <v>546</v>
       </c>
@@ -32871,7 +32956,7 @@
       <c r="BO73" s="9"/>
       <c r="BT73" s="9"/>
     </row>
-    <row r="74" spans="1:79" x14ac:dyDescent="0.35">
+    <row r="74" spans="1:79">
       <c r="A74" s="5" t="s">
         <v>547</v>
       </c>
@@ -32994,7 +33079,7 @@
       <c r="BZ74" s="5"/>
       <c r="CA74" s="5"/>
     </row>
-    <row r="75" spans="1:79" x14ac:dyDescent="0.35">
+    <row r="75" spans="1:79">
       <c r="A75" t="s">
         <v>548</v>
       </c>
@@ -33070,7 +33155,7 @@
       <c r="BO75" s="9"/>
       <c r="BT75" s="9"/>
     </row>
-    <row r="76" spans="1:79" x14ac:dyDescent="0.35">
+    <row r="76" spans="1:79">
       <c r="A76" t="s">
         <v>549</v>
       </c>
@@ -33146,7 +33231,7 @@
       <c r="BO76" s="9"/>
       <c r="BT76" s="9"/>
     </row>
-    <row r="77" spans="1:79" x14ac:dyDescent="0.35">
+    <row r="77" spans="1:79">
       <c r="A77" t="s">
         <v>550</v>
       </c>
@@ -33219,7 +33304,7 @@
       <c r="BO77" s="9"/>
       <c r="BT77" s="9"/>
     </row>
-    <row r="78" spans="1:79" x14ac:dyDescent="0.35">
+    <row r="78" spans="1:79">
       <c r="A78" t="s">
         <v>551</v>
       </c>
@@ -33292,7 +33377,7 @@
       <c r="BO78" s="9"/>
       <c r="BT78" s="9"/>
     </row>
-    <row r="79" spans="1:79" x14ac:dyDescent="0.35">
+    <row r="79" spans="1:79">
       <c r="A79" t="s">
         <v>552</v>
       </c>
@@ -33365,7 +33450,7 @@
       <c r="BO79" s="9"/>
       <c r="BT79" s="9"/>
     </row>
-    <row r="80" spans="1:79" x14ac:dyDescent="0.35">
+    <row r="80" spans="1:79">
       <c r="A80" t="s">
         <v>553</v>
       </c>
@@ -33441,7 +33526,7 @@
       <c r="BO80" s="9"/>
       <c r="BT80" s="9"/>
     </row>
-    <row r="81" spans="1:79" x14ac:dyDescent="0.35">
+    <row r="81" spans="1:79">
       <c r="A81" t="s">
         <v>554</v>
       </c>
@@ -33517,7 +33602,7 @@
       <c r="BO81" s="9"/>
       <c r="BT81" s="9"/>
     </row>
-    <row r="82" spans="1:79" x14ac:dyDescent="0.35">
+    <row r="82" spans="1:79">
       <c r="A82" t="s">
         <v>555</v>
       </c>
@@ -33593,7 +33678,7 @@
       <c r="BO82" s="9"/>
       <c r="BT82" s="9"/>
     </row>
-    <row r="83" spans="1:79" x14ac:dyDescent="0.35">
+    <row r="83" spans="1:79">
       <c r="A83" s="5" t="s">
         <v>556</v>
       </c>
@@ -33680,7 +33765,7 @@
       <c r="BZ83" s="5"/>
       <c r="CA83" s="5"/>
     </row>
-    <row r="84" spans="1:79" x14ac:dyDescent="0.35">
+    <row r="84" spans="1:79">
       <c r="A84" s="5" t="s">
         <v>557</v>
       </c>
@@ -33781,7 +33866,7 @@
       <c r="BZ84" s="5"/>
       <c r="CA84" s="5"/>
     </row>
-    <row r="85" spans="1:79" x14ac:dyDescent="0.35">
+    <row r="85" spans="1:79">
       <c r="A85" t="s">
         <v>558</v>
       </c>
@@ -33823,7 +33908,7 @@
       <c r="BO85" s="9"/>
       <c r="BT85" s="9"/>
     </row>
-    <row r="86" spans="1:79" x14ac:dyDescent="0.35">
+    <row r="86" spans="1:79">
       <c r="A86" t="s">
         <v>559</v>
       </c>
@@ -33865,7 +33950,7 @@
       <c r="BO86" s="9"/>
       <c r="BT86" s="9"/>
     </row>
-    <row r="87" spans="1:79" x14ac:dyDescent="0.35">
+    <row r="87" spans="1:79">
       <c r="A87" t="s">
         <v>560</v>
       </c>
@@ -33904,7 +33989,7 @@
       <c r="BO87" s="9"/>
       <c r="BT87" s="9"/>
     </row>
-    <row r="88" spans="1:79" x14ac:dyDescent="0.35">
+    <row r="88" spans="1:79">
       <c r="A88" t="s">
         <v>561</v>
       </c>
@@ -33943,7 +34028,7 @@
       <c r="BO88" s="9"/>
       <c r="BT88" s="9"/>
     </row>
-    <row r="89" spans="1:79" x14ac:dyDescent="0.35">
+    <row r="89" spans="1:79">
       <c r="A89" t="s">
         <v>562</v>
       </c>
@@ -33982,7 +34067,7 @@
       <c r="BO89" s="9"/>
       <c r="BT89" s="9"/>
     </row>
-    <row r="90" spans="1:79" x14ac:dyDescent="0.35">
+    <row r="90" spans="1:79">
       <c r="A90" t="s">
         <v>563</v>
       </c>
@@ -34021,7 +34106,7 @@
       <c r="BO90" s="9"/>
       <c r="BT90" s="9"/>
     </row>
-    <row r="91" spans="1:79" x14ac:dyDescent="0.35">
+    <row r="91" spans="1:79">
       <c r="A91" t="s">
         <v>564</v>
       </c>
@@ -34063,7 +34148,7 @@
       <c r="BO91" s="9"/>
       <c r="BT91" s="9"/>
     </row>
-    <row r="92" spans="1:79" x14ac:dyDescent="0.35">
+    <row r="92" spans="1:79">
       <c r="A92" t="s">
         <v>565</v>
       </c>
@@ -34102,7 +34187,7 @@
       <c r="BO92" s="9"/>
       <c r="BT92" s="9"/>
     </row>
-    <row r="93" spans="1:79" x14ac:dyDescent="0.35">
+    <row r="93" spans="1:79">
       <c r="A93" t="s">
         <v>566</v>
       </c>
@@ -34141,7 +34226,7 @@
       <c r="BO93" s="9"/>
       <c r="BT93" s="9"/>
     </row>
-    <row r="94" spans="1:79" x14ac:dyDescent="0.35">
+    <row r="94" spans="1:79">
       <c r="H94" s="16"/>
       <c r="I94" s="9"/>
       <c r="K94" s="9"/>
@@ -34159,7 +34244,7 @@
       <c r="BO94" s="9"/>
       <c r="BT94" s="9"/>
     </row>
-    <row r="95" spans="1:79" x14ac:dyDescent="0.35">
+    <row r="95" spans="1:79">
       <c r="H95" s="16"/>
       <c r="I95" s="9"/>
       <c r="K95" s="9"/>
@@ -34177,7 +34262,7 @@
       <c r="BO95" s="9"/>
       <c r="BT95" s="9"/>
     </row>
-    <row r="96" spans="1:79" x14ac:dyDescent="0.35">
+    <row r="96" spans="1:79">
       <c r="H96" s="16"/>
       <c r="I96" s="9"/>
       <c r="K96" s="9"/>
@@ -34195,7 +34280,7 @@
       <c r="BO96" s="9"/>
       <c r="BT96" s="9"/>
     </row>
-    <row r="97" spans="1:72" x14ac:dyDescent="0.35">
+    <row r="97" spans="1:72">
       <c r="A97" s="23" t="s">
         <v>567</v>
       </c>
@@ -34216,7 +34301,7 @@
       <c r="BO97" s="9"/>
       <c r="BT97" s="9"/>
     </row>
-    <row r="98" spans="1:72" x14ac:dyDescent="0.35">
+    <row r="98" spans="1:72">
       <c r="A98" s="29" t="s">
         <v>568</v>
       </c>
@@ -34237,7 +34322,7 @@
       <c r="BO98" s="9"/>
       <c r="BT98" s="9"/>
     </row>
-    <row r="99" spans="1:72" x14ac:dyDescent="0.35">
+    <row r="99" spans="1:72">
       <c r="A99" s="30" t="s">
         <v>569</v>
       </c>
@@ -34270,9 +34355,9 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0700-000000000000}">
   <dimension ref="A1:E11"/>
-  <sheetFormatPr defaultColWidth="8.7265625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultColWidth="8.7265625" defaultRowHeight="14.5"/>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:5">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -34289,7 +34374,7 @@
         <v>573</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:5">
       <c r="A2" s="3" t="s">
         <v>215</v>
       </c>
@@ -34310,7 +34395,7 @@
         <v>0.5</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:5">
       <c r="A3" s="3" t="s">
         <v>212</v>
       </c>
@@ -34331,7 +34416,7 @@
         <v>0.5</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:5">
       <c r="A4" s="3" t="s">
         <v>206</v>
       </c>
@@ -34352,7 +34437,7 @@
         <v>0.5</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:5">
       <c r="A5" s="3" t="s">
         <v>204</v>
       </c>
@@ -34373,7 +34458,7 @@
         <v>0.45</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:5">
       <c r="A6" s="3" t="s">
         <v>197</v>
       </c>
@@ -34394,7 +34479,7 @@
         <v>0.44444444444444442</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:5">
       <c r="A7" s="3" t="s">
         <v>194</v>
       </c>
@@ -34415,7 +34500,7 @@
         <v>0.40909090909090912</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:5">
       <c r="A8" s="3" t="s">
         <v>190</v>
       </c>
@@ -34436,7 +34521,7 @@
         <v>0.51282051282051277</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:5">
       <c r="A9" s="3" t="s">
         <v>185</v>
       </c>
@@ -34457,7 +34542,7 @@
         <v>0.5</v>
       </c>
     </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:5">
       <c r="A10" t="s">
         <v>278</v>
       </c>
@@ -34478,7 +34563,7 @@
         <v>0.47704448329448329</v>
       </c>
     </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:5">
       <c r="A11" t="s">
         <v>574</v>
       </c>

</xml_diff>

<commit_message>
update 019 SJ_pre2 IK setup
</commit_message>
<xml_diff>
--- a/ParticipantData and Labelling.xlsx
+++ b/ParticipantData and Labelling.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29231"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Basilio\Documents\Thesis Gigler\squatting_fais\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Git\research_data\Projects\squatting_fais\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2A917EB8-5361-4629-8C83-464B9CC74714}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7E2CEF6C-F7C1-4689-9D80-2821F3376766}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="10" yWindow="0" windowWidth="25480" windowHeight="13800" tabRatio="798" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="798" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Demographics" sheetId="1" r:id="rId1"/>
@@ -25,6 +25,19 @@
     <sheet name="Add&amp;GracEMGLocation" sheetId="8" r:id="rId10"/>
   </sheets>
   <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
@@ -621,7 +634,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1443" uniqueCount="436">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1444" uniqueCount="437">
   <si>
     <t>Subject</t>
   </si>
@@ -2017,6 +2030,9 @@
   </si>
   <si>
     <t>Run inverse dynamics from GUI</t>
+  </si>
+  <si>
+    <t>3.355, 3.715, 4.3</t>
   </si>
 </sst>
 </file>
@@ -2337,7 +2353,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="79">
+  <cellXfs count="78">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
@@ -2497,9 +2513,6 @@
       <alignment vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="17" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="17" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="16" borderId="0" xfId="0" quotePrefix="1" applyFill="1" applyAlignment="1">
@@ -3020,10 +3033,6 @@
 </styleSheet>
 </file>
 
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
-</file>
-
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Table1" displayName="Table1" ref="A1:AI68" totalsRowShown="0" headerRowDxfId="105" tableBorderDxfId="104">
   <autoFilter ref="A1:AI68" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
@@ -3312,9 +3321,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -3352,7 +3361,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -3458,7 +3467,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -3600,7 +3609,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -3609,25 +3618,25 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:AI74"/>
-  <sheetFormatPr defaultColWidth="9.1796875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="10" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="7.81640625" customWidth="1"/>
-    <col min="4" max="5" width="7.54296875" customWidth="1"/>
-    <col min="6" max="6" width="12.81640625" bestFit="1" customWidth="1"/>
-    <col min="7" max="20" width="7.54296875" customWidth="1"/>
+    <col min="2" max="2" width="7.85546875" customWidth="1"/>
+    <col min="4" max="5" width="7.5703125" customWidth="1"/>
+    <col min="6" max="6" width="12.85546875" bestFit="1" customWidth="1"/>
+    <col min="7" max="20" width="7.5703125" customWidth="1"/>
     <col min="21" max="21" width="10" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="9.26953125" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="22.26953125" customWidth="1"/>
-    <col min="24" max="24" width="26.7265625" customWidth="1"/>
-    <col min="25" max="27" width="14.453125" customWidth="1"/>
-    <col min="28" max="32" width="8.7265625" customWidth="1"/>
-    <col min="33" max="34" width="8.7265625" style="11" customWidth="1"/>
-    <col min="35" max="35" width="12.453125" style="11" customWidth="1"/>
-    <col min="36" max="36" width="15.7265625" customWidth="1"/>
+    <col min="22" max="22" width="9.28515625" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="22.28515625" customWidth="1"/>
+    <col min="24" max="24" width="26.7109375" customWidth="1"/>
+    <col min="25" max="27" width="14.42578125" customWidth="1"/>
+    <col min="28" max="32" width="8.7109375" customWidth="1"/>
+    <col min="33" max="34" width="8.7109375" style="11" customWidth="1"/>
+    <col min="35" max="35" width="12.42578125" style="11" customWidth="1"/>
+    <col min="36" max="36" width="15.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:35" ht="45" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:35" ht="45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -3734,7 +3743,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="2" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A2" s="26" t="s">
         <v>59</v>
       </c>
@@ -3823,7 +3832,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="3" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A3" s="26" t="s">
         <v>62</v>
       </c>
@@ -3911,7 +3920,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="4" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A4" s="26" t="s">
         <v>64</v>
       </c>
@@ -3975,7 +3984,7 @@
       <c r="AG4"/>
       <c r="AH4"/>
     </row>
-    <row r="5" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A5" s="26" t="s">
         <v>65</v>
       </c>
@@ -4059,7 +4068,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="6" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A6" s="26" t="s">
         <v>67</v>
       </c>
@@ -4146,7 +4155,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="7" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A7" s="26" t="s">
         <v>69</v>
       </c>
@@ -4229,7 +4238,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="8" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A8" s="26" t="s">
         <v>71</v>
       </c>
@@ -4314,7 +4323,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="9" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A9" s="26" t="s">
         <v>73</v>
       </c>
@@ -4401,7 +4410,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="10" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A10" s="26" t="s">
         <v>75</v>
       </c>
@@ -4488,7 +4497,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="11" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A11" s="26" t="s">
         <v>78</v>
       </c>
@@ -4581,7 +4590,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="12" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A12" s="31" t="s">
         <v>81</v>
       </c>
@@ -4669,7 +4678,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="13" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A13" s="31" t="s">
         <v>85</v>
       </c>
@@ -4753,7 +4762,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="14" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A14" s="31" t="s">
         <v>87</v>
       </c>
@@ -4843,7 +4852,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="15" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A15" s="31" t="s">
         <v>89</v>
       </c>
@@ -4931,7 +4940,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="16" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A16" s="31" t="s">
         <v>91</v>
       </c>
@@ -5018,7 +5027,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="17" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A17" s="31" t="s">
         <v>94</v>
       </c>
@@ -5102,7 +5111,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="18" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A18" s="31" t="s">
         <v>96</v>
       </c>
@@ -5186,7 +5195,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="19" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A19" s="31" t="s">
         <v>98</v>
       </c>
@@ -5267,7 +5276,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="20" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A20" s="31" t="s">
         <v>100</v>
       </c>
@@ -5351,7 +5360,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="21" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A21" s="31" t="s">
         <v>102</v>
       </c>
@@ -5436,7 +5445,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="22" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A22" s="31" t="s">
         <v>104</v>
       </c>
@@ -5526,7 +5535,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="23" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A23" s="31" t="s">
         <v>107</v>
       </c>
@@ -5616,7 +5625,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="24" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A24" s="31" t="s">
         <v>109</v>
       </c>
@@ -5701,7 +5710,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="25" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A25" s="31" t="s">
         <v>112</v>
       </c>
@@ -5795,7 +5804,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="26" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A26" s="31" t="s">
         <v>116</v>
       </c>
@@ -5883,7 +5892,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="27" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A27" s="31" t="s">
         <v>119</v>
       </c>
@@ -5953,11 +5962,11 @@
       <c r="AG27"/>
       <c r="AH27"/>
     </row>
-    <row r="28" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A28" s="74" t="s">
+    <row r="28" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A28" s="73" t="s">
         <v>122</v>
       </c>
-      <c r="B28" s="75">
+      <c r="B28" s="74">
         <f t="shared" si="1"/>
         <v>21</v>
       </c>
@@ -5970,19 +5979,19 @@
       <c r="E28" s="70" t="s">
         <v>35</v>
       </c>
-      <c r="F28" s="71" t="s">
+      <c r="F28" s="70" t="s">
         <v>38</v>
       </c>
-      <c r="G28" s="71" t="s">
+      <c r="G28" s="70" t="s">
         <v>56</v>
       </c>
-      <c r="H28" s="71">
+      <c r="H28" s="70">
         <v>45.5</v>
       </c>
-      <c r="I28" s="71">
+      <c r="I28" s="70">
         <v>27.8</v>
       </c>
-      <c r="J28" s="71" t="s">
+      <c r="J28" s="70" t="s">
         <v>42</v>
       </c>
       <c r="K28" s="11" t="s">
@@ -6046,7 +6055,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="29" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A29" s="31" t="s">
         <v>125</v>
       </c>
@@ -6136,11 +6145,11 @@
         <v>7</v>
       </c>
     </row>
-    <row r="30" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A30" s="72" t="s">
+    <row r="30" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A30" s="71" t="s">
         <v>127</v>
       </c>
-      <c r="B30" s="73">
+      <c r="B30" s="72">
         <f t="shared" si="1"/>
         <v>23</v>
       </c>
@@ -6229,11 +6238,11 @@
         <v>7</v>
       </c>
     </row>
-    <row r="31" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A31" s="72" t="s">
+    <row r="31" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A31" s="71" t="s">
         <v>129</v>
       </c>
-      <c r="B31" s="73">
+      <c r="B31" s="72">
         <f t="shared" si="1"/>
         <v>42</v>
       </c>
@@ -6322,11 +6331,11 @@
         <v>7</v>
       </c>
     </row>
-    <row r="32" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A32" s="72" t="s">
+    <row r="32" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A32" s="71" t="s">
         <v>131</v>
       </c>
-      <c r="B32" s="73">
+      <c r="B32" s="72">
         <f t="shared" si="1"/>
         <v>18</v>
       </c>
@@ -6415,11 +6424,11 @@
         <v>7</v>
       </c>
     </row>
-    <row r="33" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A33" s="72" t="s">
+    <row r="33" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A33" s="71" t="s">
         <v>134</v>
       </c>
-      <c r="B33" s="73">
+      <c r="B33" s="72">
         <f t="shared" si="1"/>
         <v>31</v>
       </c>
@@ -6508,7 +6517,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="34" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A34" s="31" t="s">
         <v>136</v>
       </c>
@@ -6572,7 +6581,7 @@
       <c r="AG34"/>
       <c r="AH34"/>
     </row>
-    <row r="35" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A35" s="31" t="s">
         <v>137</v>
       </c>
@@ -6599,7 +6608,7 @@
       <c r="I35" s="70">
         <v>23.2</v>
       </c>
-      <c r="J35" s="71" t="s">
+      <c r="J35" s="70" t="s">
         <v>42</v>
       </c>
       <c r="K35" s="11" t="s">
@@ -6663,11 +6672,11 @@
         <v>7</v>
       </c>
     </row>
-    <row r="36" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A36" s="72" t="s">
+    <row r="36" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A36" s="71" t="s">
         <v>140</v>
       </c>
-      <c r="B36" s="73">
+      <c r="B36" s="72">
         <f t="shared" si="1"/>
         <v>24</v>
       </c>
@@ -6756,7 +6765,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="37" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A37" s="31" t="s">
         <v>143</v>
       </c>
@@ -6838,7 +6847,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="38" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A38" s="31" t="s">
         <v>145</v>
       </c>
@@ -6906,11 +6915,11 @@
       <c r="AG38"/>
       <c r="AH38"/>
     </row>
-    <row r="39" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A39" s="72" t="s">
+    <row r="39" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A39" s="71" t="s">
         <v>147</v>
       </c>
-      <c r="B39" s="73">
+      <c r="B39" s="72">
         <f t="shared" si="1"/>
         <v>24</v>
       </c>
@@ -7001,7 +7010,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="40" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A40" s="31" t="s">
         <v>150</v>
       </c>
@@ -7093,7 +7102,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="41" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A41" s="31" t="s">
         <v>152</v>
       </c>
@@ -7166,7 +7175,7 @@
       <c r="AG41"/>
       <c r="AH41"/>
     </row>
-    <row r="42" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A42" s="31" t="s">
         <v>153</v>
       </c>
@@ -7258,7 +7267,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="43" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A43" s="31" t="s">
         <v>156</v>
       </c>
@@ -7358,7 +7367,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="44" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A44" s="31" t="s">
         <v>159</v>
       </c>
@@ -7425,11 +7434,11 @@
       <c r="AG44"/>
       <c r="AH44"/>
     </row>
-    <row r="45" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A45" s="72" t="s">
+    <row r="45" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A45" s="71" t="s">
         <v>160</v>
       </c>
-      <c r="B45" s="73">
+      <c r="B45" s="72">
         <f t="shared" si="3"/>
         <v>34</v>
       </c>
@@ -7518,7 +7527,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="46" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A46" s="31" t="s">
         <v>162</v>
       </c>
@@ -7624,7 +7633,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="47" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A47" s="31" t="s">
         <v>165</v>
       </c>
@@ -7714,7 +7723,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="48" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A48" s="31" t="s">
         <v>168</v>
       </c>
@@ -7784,7 +7793,7 @@
       <c r="AG48"/>
       <c r="AH48"/>
     </row>
-    <row r="49" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A49" s="31" t="s">
         <v>169</v>
       </c>
@@ -7893,7 +7902,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="50" spans="1:35" s="11" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:35" s="11" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A50" s="31" t="s">
         <v>172</v>
       </c>
@@ -7966,7 +7975,7 @@
       <c r="AG50"/>
       <c r="AH50"/>
     </row>
-    <row r="51" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A51" s="31" t="s">
         <v>174</v>
       </c>
@@ -8075,7 +8084,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="52" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A52" s="31" t="s">
         <v>177</v>
       </c>
@@ -8185,7 +8194,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="53" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A53" s="31" t="s">
         <v>180</v>
       </c>
@@ -8259,11 +8268,11 @@
       <c r="AG53"/>
       <c r="AH53"/>
     </row>
-    <row r="54" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A54" s="72" t="s">
+    <row r="54" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A54" s="71" t="s">
         <v>181</v>
       </c>
-      <c r="B54" s="73">
+      <c r="B54" s="72">
         <f>ROUNDDOWN((R54-Q54)/365.25,0)</f>
         <v>22</v>
       </c>
@@ -8276,7 +8285,7 @@
       <c r="E54" s="66" t="s">
         <v>35</v>
       </c>
-      <c r="F54" s="76" t="s">
+      <c r="F54" s="75" t="s">
         <v>38</v>
       </c>
       <c r="G54" s="66" t="s">
@@ -8365,7 +8374,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="55" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A55" s="31" t="s">
         <v>184</v>
       </c>
@@ -8438,7 +8447,7 @@
       <c r="AG55"/>
       <c r="AH55"/>
     </row>
-    <row r="56" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A56" s="31" t="s">
         <v>185</v>
       </c>
@@ -8519,7 +8528,7 @@
       <c r="AG56"/>
       <c r="AH56"/>
     </row>
-    <row r="57" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A57" s="31" t="s">
         <v>186</v>
       </c>
@@ -8592,7 +8601,7 @@
       <c r="AG57"/>
       <c r="AH57"/>
     </row>
-    <row r="58" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A58" s="31" t="s">
         <v>187</v>
       </c>
@@ -8701,7 +8710,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="59" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A59" s="31" t="s">
         <v>190</v>
       </c>
@@ -8808,7 +8817,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="60" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A60" s="31" t="s">
         <v>194</v>
       </c>
@@ -8917,11 +8926,11 @@
         <v>7</v>
       </c>
     </row>
-    <row r="61" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A61" s="72" t="s">
+    <row r="61" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A61" s="71" t="s">
         <v>197</v>
       </c>
-      <c r="B61" s="73">
+      <c r="B61" s="72">
         <f t="shared" si="5"/>
         <v>33</v>
       </c>
@@ -8934,7 +8943,7 @@
       <c r="E61" s="66" t="s">
         <v>35</v>
       </c>
-      <c r="F61" s="76" t="s">
+      <c r="F61" s="75" t="s">
         <v>38</v>
       </c>
       <c r="G61" s="66" t="s">
@@ -9029,7 +9038,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="62" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A62" s="31" t="s">
         <v>200</v>
       </c>
@@ -9139,11 +9148,11 @@
         <v>7</v>
       </c>
     </row>
-    <row r="63" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A63" s="72" t="s">
+    <row r="63" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A63" s="71" t="s">
         <v>204</v>
       </c>
-      <c r="B63" s="73">
+      <c r="B63" s="72">
         <f t="shared" si="5"/>
         <v>26</v>
       </c>
@@ -9251,11 +9260,11 @@
         <v>5</v>
       </c>
     </row>
-    <row r="64" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A64" s="72" t="s">
+    <row r="64" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A64" s="71" t="s">
         <v>206</v>
       </c>
-      <c r="B64" s="73">
+      <c r="B64" s="72">
         <f t="shared" si="5"/>
         <v>39</v>
       </c>
@@ -9363,11 +9372,11 @@
         <v>7</v>
       </c>
     </row>
-    <row r="65" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A65" s="72" t="s">
+    <row r="65" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A65" s="71" t="s">
         <v>209</v>
       </c>
-      <c r="B65" s="73">
+      <c r="B65" s="72">
         <f t="shared" si="5"/>
         <v>32</v>
       </c>
@@ -9475,7 +9484,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="66" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="66" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A66" s="31" t="s">
         <v>212</v>
       </c>
@@ -9586,7 +9595,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="67" spans="1:35" s="11" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="67" spans="1:35" s="11" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A67" s="31" t="s">
         <v>215</v>
       </c>
@@ -9602,17 +9611,17 @@
       <c r="E67" s="11" t="s">
         <v>35</v>
       </c>
-      <c r="F67" s="71"/>
-      <c r="G67" s="71" t="s">
+      <c r="F67" s="70"/>
+      <c r="G67" s="70" t="s">
         <v>56</v>
       </c>
-      <c r="H67" s="71">
+      <c r="H67" s="70">
         <v>59.9</v>
       </c>
-      <c r="I67" s="71">
+      <c r="I67" s="70">
         <v>22.6</v>
       </c>
-      <c r="J67" s="71" t="s">
+      <c r="J67" s="70" t="s">
         <v>157</v>
       </c>
       <c r="K67" s="11" t="s">
@@ -9694,7 +9703,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="68" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="68" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A68" s="1"/>
       <c r="B68" s="36"/>
       <c r="Q68" s="63"/>
@@ -9712,7 +9721,7 @@
       <c r="AG68"/>
       <c r="AH68"/>
     </row>
-    <row r="69" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="69" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A69" s="64"/>
       <c r="B69" s="64"/>
       <c r="C69" s="64"/>
@@ -9749,7 +9758,7 @@
       <c r="AH69" s="64"/>
       <c r="AI69" s="64"/>
     </row>
-    <row r="70" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="70" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A70" s="64"/>
       <c r="B70" s="64"/>
       <c r="C70" s="64"/>
@@ -9786,7 +9795,7 @@
       <c r="AH70" s="64"/>
       <c r="AI70" s="64"/>
     </row>
-    <row r="71" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="71" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A71" s="64"/>
       <c r="B71" s="64"/>
       <c r="C71" s="64"/>
@@ -9823,7 +9832,7 @@
       <c r="AH71" s="64"/>
       <c r="AI71" s="64"/>
     </row>
-    <row r="72" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="72" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A72" s="64"/>
       <c r="B72" s="64"/>
       <c r="C72" s="64"/>
@@ -9860,7 +9869,7 @@
       <c r="AH72" s="64"/>
       <c r="AI72" s="64"/>
     </row>
-    <row r="73" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="73" spans="1:35" x14ac:dyDescent="0.25">
       <c r="B73" s="36">
         <f>AVERAGE(B3,B11,B21,B23,B28,B30,B36,B45,B63,B64,B65,B67)</f>
         <v>26.833333333333332</v>
@@ -9873,7 +9882,7 @@
       <c r="AG73"/>
       <c r="AH73"/>
     </row>
-    <row r="74" spans="1:35" x14ac:dyDescent="0.35">
+    <row r="74" spans="1:35" x14ac:dyDescent="0.25">
       <c r="R74" s="64"/>
       <c r="AG74"/>
       <c r="AH74"/>
@@ -9891,9 +9900,9 @@
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0700-000000000000}">
   <dimension ref="A1:E11"/>
-  <sheetFormatPr defaultColWidth="8.7265625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -9910,7 +9919,7 @@
         <v>406</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>215</v>
       </c>
@@ -9931,7 +9940,7 @@
         <v>0.5</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>212</v>
       </c>
@@ -9952,7 +9961,7 @@
         <v>0.5</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
         <v>206</v>
       </c>
@@ -9973,7 +9982,7 @@
         <v>0.5</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
         <v>204</v>
       </c>
@@ -9994,7 +10003,7 @@
         <v>0.45</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
         <v>197</v>
       </c>
@@ -10015,7 +10024,7 @@
         <v>0.44444444444444442</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
         <v>194</v>
       </c>
@@ -10036,7 +10045,7 @@
         <v>0.40909090909090912</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
         <v>190</v>
       </c>
@@ -10057,7 +10066,7 @@
         <v>0.51282051282051277</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
         <v>185</v>
       </c>
@@ -10078,7 +10087,7 @@
         <v>0.5</v>
       </c>
     </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>274</v>
       </c>
@@ -10099,7 +10108,7 @@
         <v>0.47704448329448329</v>
       </c>
     </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>407</v>
       </c>
@@ -10128,9 +10137,9 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{89B2075C-5F56-4EF1-95BD-F5E1A85C949C}">
   <dimension ref="A1:B4"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1">
         <v>1</v>
       </c>
@@ -10138,7 +10147,7 @@
         <v>434</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>2</v>
       </c>
@@ -10146,7 +10155,7 @@
         <v>433</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>3</v>
       </c>
@@ -10154,7 +10163,7 @@
         <v>409</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>4</v>
       </c>
@@ -10170,12 +10179,12 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{12AC9CB0-5B51-495B-9318-23D7E97CB111}">
   <dimension ref="A2:J20"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="11.453125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="11.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>417</v>
       </c>
@@ -10194,13 +10203,13 @@
       <c r="F2" t="s">
         <v>423</v>
       </c>
-      <c r="H2" s="77" t="s">
+      <c r="H2" s="76" t="s">
         <v>425</v>
       </c>
-      <c r="I2" s="77"/>
-      <c r="J2" s="77"/>
-    </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="I2" s="76"/>
+      <c r="J2" s="76"/>
+    </row>
+    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>10</v>
       </c>
@@ -10226,7 +10235,7 @@
         <v>0.1</v>
       </c>
     </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
       <c r="H4" t="s">
         <v>426</v>
       </c>
@@ -10234,113 +10243,113 @@
         <v>7.0000000000000007E-2</v>
       </c>
     </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="F10" s="77" t="s">
+    <row r="10" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="F10" s="76" t="s">
         <v>429</v>
       </c>
-      <c r="G10" s="77"/>
-      <c r="H10" s="77"/>
-      <c r="I10" s="77"/>
-      <c r="J10" s="77"/>
-    </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A11" s="78" t="s">
+      <c r="G10" s="76"/>
+      <c r="H10" s="76"/>
+      <c r="I10" s="76"/>
+      <c r="J10" s="76"/>
+    </row>
+    <row r="11" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A11" s="77" t="s">
         <v>427</v>
       </c>
-      <c r="B11" s="78"/>
-      <c r="C11" s="78"/>
-      <c r="D11" s="78"/>
-    </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A12" s="78"/>
-      <c r="B12" s="78"/>
-      <c r="C12" s="78"/>
-      <c r="D12" s="78"/>
-      <c r="F12" s="78" t="s">
+      <c r="B11" s="77"/>
+      <c r="C11" s="77"/>
+      <c r="D11" s="77"/>
+    </row>
+    <row r="12" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A12" s="77"/>
+      <c r="B12" s="77"/>
+      <c r="C12" s="77"/>
+      <c r="D12" s="77"/>
+      <c r="F12" s="77" t="s">
         <v>428</v>
       </c>
-      <c r="G12" s="78"/>
-      <c r="H12" s="78"/>
-      <c r="I12" s="78"/>
-      <c r="J12" s="78"/>
-    </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A13" s="78"/>
-      <c r="B13" s="78"/>
-      <c r="C13" s="78"/>
-      <c r="D13" s="78"/>
-      <c r="F13" s="78"/>
-      <c r="G13" s="78"/>
-      <c r="H13" s="78"/>
-      <c r="I13" s="78"/>
-      <c r="J13" s="78"/>
-    </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A14" s="78"/>
-      <c r="B14" s="78"/>
-      <c r="C14" s="78"/>
-      <c r="D14" s="78"/>
-      <c r="F14" s="78"/>
-      <c r="G14" s="78"/>
-      <c r="H14" s="78"/>
-      <c r="I14" s="78"/>
-      <c r="J14" s="78"/>
-    </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A15" s="78"/>
-      <c r="B15" s="78"/>
-      <c r="C15" s="78"/>
-      <c r="D15" s="78"/>
-      <c r="F15" s="78"/>
-      <c r="G15" s="78"/>
-      <c r="H15" s="78"/>
-      <c r="I15" s="78"/>
-      <c r="J15" s="78"/>
-    </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A16" s="78"/>
-      <c r="B16" s="78"/>
-      <c r="C16" s="78"/>
-      <c r="D16" s="78"/>
-      <c r="F16" s="78"/>
-      <c r="G16" s="78"/>
-      <c r="H16" s="78"/>
-      <c r="I16" s="78"/>
-      <c r="J16" s="78"/>
-    </row>
-    <row r="17" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A17" s="78"/>
-      <c r="B17" s="78"/>
-      <c r="C17" s="78"/>
-      <c r="D17" s="78"/>
-      <c r="F17" s="78"/>
-      <c r="G17" s="78"/>
-      <c r="H17" s="78"/>
-      <c r="I17" s="78"/>
-      <c r="J17" s="78"/>
-    </row>
-    <row r="18" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A18" s="78"/>
-      <c r="B18" s="78"/>
-      <c r="C18" s="78"/>
-      <c r="D18" s="78"/>
-      <c r="F18" s="78"/>
-      <c r="G18" s="78"/>
-      <c r="H18" s="78"/>
-      <c r="I18" s="78"/>
-      <c r="J18" s="78"/>
-    </row>
-    <row r="19" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A19" s="78"/>
-      <c r="B19" s="78"/>
-      <c r="C19" s="78"/>
-      <c r="D19" s="78"/>
-    </row>
-    <row r="20" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A20" s="78"/>
-      <c r="B20" s="78"/>
-      <c r="C20" s="78"/>
-      <c r="D20" s="78"/>
+      <c r="G12" s="77"/>
+      <c r="H12" s="77"/>
+      <c r="I12" s="77"/>
+      <c r="J12" s="77"/>
+    </row>
+    <row r="13" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A13" s="77"/>
+      <c r="B13" s="77"/>
+      <c r="C13" s="77"/>
+      <c r="D13" s="77"/>
+      <c r="F13" s="77"/>
+      <c r="G13" s="77"/>
+      <c r="H13" s="77"/>
+      <c r="I13" s="77"/>
+      <c r="J13" s="77"/>
+    </row>
+    <row r="14" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A14" s="77"/>
+      <c r="B14" s="77"/>
+      <c r="C14" s="77"/>
+      <c r="D14" s="77"/>
+      <c r="F14" s="77"/>
+      <c r="G14" s="77"/>
+      <c r="H14" s="77"/>
+      <c r="I14" s="77"/>
+      <c r="J14" s="77"/>
+    </row>
+    <row r="15" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A15" s="77"/>
+      <c r="B15" s="77"/>
+      <c r="C15" s="77"/>
+      <c r="D15" s="77"/>
+      <c r="F15" s="77"/>
+      <c r="G15" s="77"/>
+      <c r="H15" s="77"/>
+      <c r="I15" s="77"/>
+      <c r="J15" s="77"/>
+    </row>
+    <row r="16" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A16" s="77"/>
+      <c r="B16" s="77"/>
+      <c r="C16" s="77"/>
+      <c r="D16" s="77"/>
+      <c r="F16" s="77"/>
+      <c r="G16" s="77"/>
+      <c r="H16" s="77"/>
+      <c r="I16" s="77"/>
+      <c r="J16" s="77"/>
+    </row>
+    <row r="17" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A17" s="77"/>
+      <c r="B17" s="77"/>
+      <c r="C17" s="77"/>
+      <c r="D17" s="77"/>
+      <c r="F17" s="77"/>
+      <c r="G17" s="77"/>
+      <c r="H17" s="77"/>
+      <c r="I17" s="77"/>
+      <c r="J17" s="77"/>
+    </row>
+    <row r="18" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A18" s="77"/>
+      <c r="B18" s="77"/>
+      <c r="C18" s="77"/>
+      <c r="D18" s="77"/>
+      <c r="F18" s="77"/>
+      <c r="G18" s="77"/>
+      <c r="H18" s="77"/>
+      <c r="I18" s="77"/>
+      <c r="J18" s="77"/>
+    </row>
+    <row r="19" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A19" s="77"/>
+      <c r="B19" s="77"/>
+      <c r="C19" s="77"/>
+      <c r="D19" s="77"/>
+    </row>
+    <row r="20" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A20" s="77"/>
+      <c r="B20" s="77"/>
+      <c r="C20" s="77"/>
+      <c r="D20" s="77"/>
     </row>
   </sheetData>
   <mergeCells count="4">
@@ -10356,13 +10365,13 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
   <dimension ref="A1:M31"/>
-  <sheetFormatPr defaultColWidth="8.7265625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="20.1796875" customWidth="1"/>
-    <col min="2" max="13" width="12.6328125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="20.140625" customWidth="1"/>
+    <col min="2" max="13" width="12.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
         <v>375</v>
       </c>
@@ -10403,7 +10412,7 @@
         <v>387</v>
       </c>
     </row>
-    <row r="2" spans="1:13" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:13" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="3" t="s">
         <v>8</v>
       </c>
@@ -10444,7 +10453,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="3" spans="1:13" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:13" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A3" s="5" t="s">
         <v>389</v>
       </c>
@@ -10485,7 +10494,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="4" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>390</v>
       </c>
@@ -10523,7 +10532,7 @@
         <v>415</v>
       </c>
     </row>
-    <row r="5" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>391</v>
       </c>
@@ -10561,7 +10570,7 @@
         <v>415</v>
       </c>
     </row>
-    <row r="6" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>392</v>
       </c>
@@ -10599,7 +10608,7 @@
         <v>415</v>
       </c>
     </row>
-    <row r="7" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>393</v>
       </c>
@@ -10637,7 +10646,7 @@
         <v>415</v>
       </c>
     </row>
-    <row r="8" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>394</v>
       </c>
@@ -10675,7 +10684,7 @@
         <v>415</v>
       </c>
     </row>
-    <row r="9" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>395</v>
       </c>
@@ -10713,7 +10722,7 @@
         <v>415</v>
       </c>
     </row>
-    <row r="10" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>396</v>
       </c>
@@ -10751,7 +10760,7 @@
         <v>415</v>
       </c>
     </row>
-    <row r="11" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>397</v>
       </c>
@@ -10789,7 +10798,7 @@
         <v>415</v>
       </c>
     </row>
-    <row r="12" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>398</v>
       </c>
@@ -10827,7 +10836,7 @@
         <v>415</v>
       </c>
     </row>
-    <row r="13" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>399</v>
       </c>
@@ -10865,7 +10874,7 @@
         <v>415</v>
       </c>
     </row>
-    <row r="14" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>410</v>
       </c>
@@ -10903,7 +10912,7 @@
         <v>415</v>
       </c>
     </row>
-    <row r="15" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>411</v>
       </c>
@@ -10941,7 +10950,7 @@
         <v>415</v>
       </c>
     </row>
-    <row r="16" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>412</v>
       </c>
@@ -10979,7 +10988,7 @@
         <v>415</v>
       </c>
     </row>
-    <row r="17" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>413</v>
       </c>
@@ -11017,7 +11026,7 @@
         <v>415</v>
       </c>
     </row>
-    <row r="18" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>414</v>
       </c>
@@ -11055,22 +11064,22 @@
         <v>415</v>
       </c>
     </row>
-    <row r="20" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>416</v>
       </c>
     </row>
-    <row r="29" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A29" s="6" t="s">
         <v>400</v>
       </c>
     </row>
-    <row r="30" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A30" s="8" t="s">
         <v>401</v>
       </c>
     </row>
-    <row r="31" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A31" s="9" t="s">
         <v>402</v>
       </c>
@@ -11086,13 +11095,13 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{68654364-EAB1-4DEC-A6E8-9FEA32BD138C}">
   <dimension ref="A1:M30"/>
-  <sheetFormatPr defaultColWidth="8.7265625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="20.1796875" customWidth="1"/>
-    <col min="2" max="13" width="12.6328125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="20.140625" customWidth="1"/>
+    <col min="2" max="13" width="12.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:13" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1" s="3" t="s">
         <v>375</v>
       </c>
@@ -11133,7 +11142,7 @@
         <v>388</v>
       </c>
     </row>
-    <row r="2" spans="1:13" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:13" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="5" t="s">
         <v>389</v>
       </c>
@@ -11174,32 +11183,32 @@
         <v>41</v>
       </c>
     </row>
-    <row r="3" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>390</v>
       </c>
     </row>
-    <row r="4" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>391</v>
       </c>
     </row>
-    <row r="5" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>392</v>
       </c>
     </row>
-    <row r="6" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>393</v>
       </c>
     </row>
-    <row r="7" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>394</v>
       </c>
     </row>
-    <row r="8" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>395</v>
       </c>
@@ -11207,67 +11216,70 @@
         <v>430</v>
       </c>
     </row>
-    <row r="9" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>396</v>
       </c>
-    </row>
-    <row r="10" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="B9" t="s">
+        <v>436</v>
+      </c>
+    </row>
+    <row r="10" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>397</v>
       </c>
     </row>
-    <row r="11" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>398</v>
       </c>
     </row>
-    <row r="12" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>399</v>
       </c>
     </row>
-    <row r="13" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>410</v>
       </c>
     </row>
-    <row r="14" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>411</v>
       </c>
     </row>
-    <row r="15" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>412</v>
       </c>
     </row>
-    <row r="16" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>413</v>
       </c>
     </row>
-    <row r="17" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>414</v>
       </c>
     </row>
-    <row r="19" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>416</v>
       </c>
     </row>
-    <row r="28" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A28" s="6" t="s">
         <v>400</v>
       </c>
     </row>
-    <row r="29" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A29" s="8" t="s">
         <v>401</v>
       </c>
     </row>
-    <row r="30" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A30" s="9" t="s">
         <v>402</v>
       </c>
@@ -11283,12 +11295,12 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:O23"/>
-  <sheetFormatPr defaultColWidth="8.7265625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="15" width="14.26953125" customWidth="1"/>
+    <col min="1" max="15" width="14.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" s="13" customFormat="1" ht="57" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:15" s="13" customFormat="1" ht="57" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="13" t="s">
         <v>0</v>
       </c>
@@ -11335,7 +11347,7 @@
         <v>234</v>
       </c>
     </row>
-    <row r="2" spans="1:15" s="13" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:15" s="13" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A2" s="18" t="s">
         <v>204</v>
       </c>
@@ -11382,7 +11394,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A3" s="19" t="s">
         <v>206</v>
       </c>
@@ -11429,7 +11441,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A4" s="19" t="s">
         <v>209</v>
       </c>
@@ -11476,7 +11488,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A5" s="19" t="s">
         <v>200</v>
       </c>
@@ -11523,7 +11535,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A6" s="19" t="s">
         <v>197</v>
       </c>
@@ -11570,7 +11582,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A7" s="19" t="s">
         <v>194</v>
       </c>
@@ -11617,7 +11629,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="8" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A8" s="19" t="s">
         <v>190</v>
       </c>
@@ -11664,7 +11676,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="9" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A9" s="19" t="s">
         <v>187</v>
       </c>
@@ -11711,7 +11723,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="10" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A10" s="19" t="s">
         <v>177</v>
       </c>
@@ -11758,7 +11770,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="11" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A11" s="19" t="s">
         <v>174</v>
       </c>
@@ -11805,7 +11817,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="12" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A12" s="19" t="s">
         <v>169</v>
       </c>
@@ -11852,7 +11864,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="13" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A13" s="19" t="s">
         <v>162</v>
       </c>
@@ -11899,7 +11911,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="14" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A14" s="19" t="s">
         <v>156</v>
       </c>
@@ -11946,7 +11958,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="15" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A15" s="19" t="s">
         <v>212</v>
       </c>
@@ -11993,7 +12005,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="16" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A16" s="19" t="s">
         <v>215</v>
       </c>
@@ -12040,31 +12052,31 @@
         <v>1</v>
       </c>
     </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A17" s="19"/>
       <c r="F17" s="22"/>
     </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A18" s="19"/>
       <c r="F18" s="22"/>
     </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A19" s="19"/>
       <c r="F19" s="22"/>
     </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A20" s="19"/>
       <c r="F20" s="22"/>
     </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A21" s="19"/>
       <c r="F21" s="22"/>
     </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A22" s="19"/>
       <c r="F22" s="22"/>
     </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A23" s="19"/>
     </row>
   </sheetData>
@@ -12078,20 +12090,20 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:AJ23"/>
-  <sheetFormatPr defaultColWidth="14.453125" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultColWidth="14.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="16" width="25.453125" style="11" customWidth="1"/>
-    <col min="17" max="17" width="25.453125" style="14" customWidth="1"/>
-    <col min="18" max="22" width="25.453125" style="11" customWidth="1"/>
-    <col min="23" max="23" width="25.453125" style="14" customWidth="1"/>
-    <col min="24" max="26" width="25.453125" style="11" customWidth="1"/>
-    <col min="27" max="27" width="25.453125" style="14" customWidth="1"/>
-    <col min="28" max="34" width="25.453125" style="11" customWidth="1"/>
-    <col min="35" max="35" width="14.453125" style="11" customWidth="1"/>
-    <col min="36" max="16384" width="14.453125" style="11"/>
+    <col min="1" max="16" width="25.42578125" style="11" customWidth="1"/>
+    <col min="17" max="17" width="25.42578125" style="14" customWidth="1"/>
+    <col min="18" max="22" width="25.42578125" style="11" customWidth="1"/>
+    <col min="23" max="23" width="25.42578125" style="14" customWidth="1"/>
+    <col min="24" max="26" width="25.42578125" style="11" customWidth="1"/>
+    <col min="27" max="27" width="25.42578125" style="14" customWidth="1"/>
+    <col min="28" max="34" width="25.42578125" style="11" customWidth="1"/>
+    <col min="35" max="35" width="14.42578125" style="11" customWidth="1"/>
+    <col min="36" max="16384" width="14.42578125" style="11"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:36" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:36" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B1" s="12" t="s">
         <v>235</v>
       </c>
@@ -12105,7 +12117,7 @@
         <v>238</v>
       </c>
     </row>
-    <row r="2" spans="1:36" s="13" customFormat="1" ht="90" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:36" s="13" customFormat="1" ht="90" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="13" t="s">
         <v>0</v>
       </c>
@@ -12215,7 +12227,7 @@
         <v>273</v>
       </c>
     </row>
-    <row r="3" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A3" s="44" t="s">
         <v>156</v>
       </c>
@@ -12327,7 +12339,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="4" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A4" s="44" t="s">
         <v>162</v>
       </c>
@@ -12436,7 +12448,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="5" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A5" s="44" t="s">
         <v>169</v>
       </c>
@@ -12542,7 +12554,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="6" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A6" s="46" t="s">
         <v>174</v>
       </c>
@@ -12651,7 +12663,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="7" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A7" s="46" t="s">
         <v>177</v>
       </c>
@@ -12752,7 +12764,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="8" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A8" s="48" t="s">
         <v>181</v>
       </c>
@@ -12760,7 +12772,7 @@
       <c r="W8" s="11"/>
       <c r="AA8" s="11"/>
     </row>
-    <row r="9" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A9" s="11" t="s">
         <v>187</v>
       </c>
@@ -12858,7 +12870,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="10" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A10" s="11" t="s">
         <v>194</v>
       </c>
@@ -12970,7 +12982,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="11" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A11" s="45" t="s">
         <v>197</v>
       </c>
@@ -13082,7 +13094,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="12" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A12" s="19" t="s">
         <v>200</v>
       </c>
@@ -13188,7 +13200,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="13" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A13" s="45" t="s">
         <v>204</v>
       </c>
@@ -13300,7 +13312,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="14" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A14" s="19" t="s">
         <v>206</v>
       </c>
@@ -13406,7 +13418,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="15" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A15" s="45" t="s">
         <v>209</v>
       </c>
@@ -13512,7 +13524,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="16" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A16" s="19" t="s">
         <v>212</v>
       </c>
@@ -13624,7 +13636,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="17" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:36" x14ac:dyDescent="0.25">
       <c r="A17" s="45" t="s">
         <v>215</v>
       </c>
@@ -13732,7 +13744,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="19" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:36" x14ac:dyDescent="0.25">
       <c r="AH19" s="11" t="s">
         <v>274</v>
       </c>
@@ -13745,7 +13757,7 @@
         <v>31.5</v>
       </c>
     </row>
-    <row r="20" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:36" x14ac:dyDescent="0.25">
       <c r="AH20" s="11" t="s">
         <v>275</v>
       </c>
@@ -13758,7 +13770,7 @@
         <v>1.5566235649883124</v>
       </c>
     </row>
-    <row r="21" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:36" x14ac:dyDescent="0.25">
       <c r="AH21" s="11" t="s">
         <v>276</v>
       </c>
@@ -13771,7 +13783,7 @@
         <v>31.5</v>
       </c>
     </row>
-    <row r="22" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:36" x14ac:dyDescent="0.25">
       <c r="AH22" s="11" t="s">
         <v>277</v>
       </c>
@@ -13784,7 +13796,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="23" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:36" x14ac:dyDescent="0.25">
       <c r="AH23" s="11" t="s">
         <v>278</v>
       </c>
@@ -13809,24 +13821,24 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A1:AR24"/>
-  <sheetFormatPr defaultColWidth="8.7265625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="21.26953125" style="19" customWidth="1"/>
-    <col min="2" max="8" width="14.1796875" customWidth="1"/>
-    <col min="9" max="9" width="14.1796875" style="17" customWidth="1"/>
-    <col min="10" max="19" width="14.1796875" customWidth="1"/>
-    <col min="20" max="20" width="14.1796875" style="17" customWidth="1"/>
-    <col min="21" max="25" width="14.1796875" customWidth="1"/>
-    <col min="26" max="26" width="14.1796875" style="17" customWidth="1"/>
-    <col min="27" max="34" width="14.1796875" customWidth="1"/>
-    <col min="35" max="35" width="14.1796875" style="17" customWidth="1"/>
-    <col min="36" max="37" width="14.1796875" customWidth="1"/>
-    <col min="38" max="38" width="14.1796875" style="17" customWidth="1"/>
-    <col min="39" max="43" width="14.1796875" customWidth="1"/>
-    <col min="44" max="51" width="15.81640625" customWidth="1"/>
+    <col min="1" max="1" width="21.28515625" style="19" customWidth="1"/>
+    <col min="2" max="8" width="14.140625" customWidth="1"/>
+    <col min="9" max="9" width="14.140625" style="17" customWidth="1"/>
+    <col min="10" max="19" width="14.140625" customWidth="1"/>
+    <col min="20" max="20" width="14.140625" style="17" customWidth="1"/>
+    <col min="21" max="25" width="14.140625" customWidth="1"/>
+    <col min="26" max="26" width="14.140625" style="17" customWidth="1"/>
+    <col min="27" max="34" width="14.140625" customWidth="1"/>
+    <col min="35" max="35" width="14.140625" style="17" customWidth="1"/>
+    <col min="36" max="37" width="14.140625" customWidth="1"/>
+    <col min="38" max="38" width="14.140625" style="17" customWidth="1"/>
+    <col min="39" max="43" width="14.140625" customWidth="1"/>
+    <col min="44" max="51" width="15.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:44" s="13" customFormat="1" ht="180" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:44" s="13" customFormat="1" ht="180" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="18" t="s">
         <v>279</v>
       </c>
@@ -13960,7 +13972,7 @@
         <v>322</v>
       </c>
     </row>
-    <row r="2" spans="1:44" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:44" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>323</v>
       </c>
@@ -14100,7 +14112,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:44" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:44" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>324</v>
       </c>
@@ -14240,7 +14252,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="4" spans="1:44" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:44" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>325</v>
       </c>
@@ -14380,7 +14392,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="5" spans="1:44" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:44" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>326</v>
       </c>
@@ -14520,7 +14532,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="6" spans="1:44" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:44" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>327</v>
       </c>
@@ -14660,7 +14672,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="7" spans="1:44" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:44" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>328</v>
       </c>
@@ -14800,7 +14812,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="8" spans="1:44" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:44" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>329</v>
       </c>
@@ -14940,7 +14952,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="9" spans="1:44" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:44" x14ac:dyDescent="0.25">
       <c r="A9" s="19" t="s">
         <v>330</v>
       </c>
@@ -15080,7 +15092,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="10" spans="1:44" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:44" x14ac:dyDescent="0.25">
       <c r="A10" s="19" t="s">
         <v>331</v>
       </c>
@@ -15220,7 +15232,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="11" spans="1:44" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:44" x14ac:dyDescent="0.25">
       <c r="A11" s="19" t="s">
         <v>332</v>
       </c>
@@ -15360,7 +15372,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="12" spans="1:44" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:44" x14ac:dyDescent="0.25">
       <c r="A12" s="19" t="s">
         <v>333</v>
       </c>
@@ -15500,7 +15512,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="13" spans="1:44" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:44" x14ac:dyDescent="0.25">
       <c r="A13" s="19" t="s">
         <v>334</v>
       </c>
@@ -15640,7 +15652,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="14" spans="1:44" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:44" x14ac:dyDescent="0.25">
       <c r="A14" s="19" t="s">
         <v>335</v>
       </c>
@@ -15780,7 +15792,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="15" spans="1:44" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:44" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>336</v>
       </c>
@@ -15917,7 +15929,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="16" spans="1:44" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:44" x14ac:dyDescent="0.25">
       <c r="A16" s="1" t="s">
         <v>337</v>
       </c>
@@ -16057,7 +16069,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="17" spans="1:44" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:44" x14ac:dyDescent="0.25">
       <c r="I17" s="49"/>
       <c r="T17" s="49"/>
       <c r="Z17" s="49"/>
@@ -16065,7 +16077,7 @@
       <c r="AL17" s="49"/>
       <c r="AR17" s="49"/>
     </row>
-    <row r="18" spans="1:44" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:44" x14ac:dyDescent="0.25">
       <c r="I18" s="51"/>
       <c r="T18" s="51"/>
       <c r="Z18" s="51"/>
@@ -16073,7 +16085,7 @@
       <c r="AL18" s="51"/>
       <c r="AR18" s="51"/>
     </row>
-    <row r="19" spans="1:44" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:44" x14ac:dyDescent="0.25">
       <c r="A19" s="19" t="s">
         <v>338</v>
       </c>
@@ -16250,7 +16262,7 @@
         <v>47.666666666666664</v>
       </c>
     </row>
-    <row r="20" spans="1:44" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:44" x14ac:dyDescent="0.25">
       <c r="A20" s="19" t="s">
         <v>339</v>
       </c>
@@ -16427,7 +16439,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="21" spans="1:44" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:44" x14ac:dyDescent="0.25">
       <c r="A21" s="19" t="s">
         <v>340</v>
       </c>
@@ -16586,7 +16598,7 @@
       </c>
       <c r="AR21" s="51"/>
     </row>
-    <row r="22" spans="1:44" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:44" x14ac:dyDescent="0.25">
       <c r="A22" s="19" t="s">
         <v>275</v>
       </c>
@@ -16763,7 +16775,7 @@
         <v>20.254335220838414</v>
       </c>
     </row>
-    <row r="23" spans="1:44" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:44" x14ac:dyDescent="0.25">
       <c r="A23" s="19" t="s">
         <v>341</v>
       </c>
@@ -16940,7 +16952,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="24" spans="1:44" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:44" x14ac:dyDescent="0.25">
       <c r="A24" s="19" t="s">
         <v>278</v>
       </c>
@@ -17130,14 +17142,14 @@
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
   <dimension ref="A1:AG80"/>
-  <sheetFormatPr defaultColWidth="8.7265625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="10" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="9.453125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="9.42578125" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="10" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:33" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -17238,13 +17250,13 @@
         <v>372</v>
       </c>
     </row>
-    <row r="2" spans="1:33" hidden="1" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:33" hidden="1" x14ac:dyDescent="0.25">
       <c r="A2" s="11" t="s">
         <v>34</v>
       </c>
       <c r="B2" s="11"/>
     </row>
-    <row r="3" spans="1:33" hidden="1" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:33" hidden="1" x14ac:dyDescent="0.25">
       <c r="A3" s="26" t="s">
         <v>40</v>
       </c>
@@ -17252,7 +17264,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="4" spans="1:33" hidden="1" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:33" hidden="1" x14ac:dyDescent="0.25">
       <c r="A4" s="26" t="s">
         <v>47</v>
       </c>
@@ -17260,7 +17272,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="5" spans="1:33" hidden="1" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:33" hidden="1" x14ac:dyDescent="0.25">
       <c r="A5" s="26" t="s">
         <v>49</v>
       </c>
@@ -17268,7 +17280,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="6" spans="1:33" hidden="1" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:33" hidden="1" x14ac:dyDescent="0.25">
       <c r="A6" s="26" t="s">
         <v>51</v>
       </c>
@@ -17276,7 +17288,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="7" spans="1:33" hidden="1" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:33" hidden="1" x14ac:dyDescent="0.25">
       <c r="A7" s="26" t="s">
         <v>53</v>
       </c>
@@ -17284,7 +17296,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="8" spans="1:33" hidden="1" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:33" hidden="1" x14ac:dyDescent="0.25">
       <c r="A8" s="26" t="s">
         <v>55</v>
       </c>
@@ -17292,7 +17304,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="9" spans="1:33" hidden="1" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:33" hidden="1" x14ac:dyDescent="0.25">
       <c r="A9" s="27" t="s">
         <v>58</v>
       </c>
@@ -17300,7 +17312,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="10" spans="1:33" hidden="1" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:33" hidden="1" x14ac:dyDescent="0.25">
       <c r="A10" s="26" t="s">
         <v>59</v>
       </c>
@@ -17308,7 +17320,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="11" spans="1:33" hidden="1" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:33" hidden="1" x14ac:dyDescent="0.25">
       <c r="A11" s="27" t="s">
         <v>62</v>
       </c>
@@ -17316,7 +17328,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="12" spans="1:33" hidden="1" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:33" hidden="1" x14ac:dyDescent="0.25">
       <c r="A12" s="27" t="s">
         <v>64</v>
       </c>
@@ -17324,7 +17336,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="13" spans="1:33" hidden="1" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:33" hidden="1" x14ac:dyDescent="0.25">
       <c r="A13" s="26" t="s">
         <v>65</v>
       </c>
@@ -17332,7 +17344,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="14" spans="1:33" hidden="1" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:33" hidden="1" x14ac:dyDescent="0.25">
       <c r="A14" s="26" t="s">
         <v>67</v>
       </c>
@@ -17340,7 +17352,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="15" spans="1:33" hidden="1" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:33" hidden="1" x14ac:dyDescent="0.25">
       <c r="A15" s="26" t="s">
         <v>69</v>
       </c>
@@ -17348,7 +17360,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="16" spans="1:33" hidden="1" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:33" hidden="1" x14ac:dyDescent="0.25">
       <c r="A16" s="27" t="s">
         <v>71</v>
       </c>
@@ -17356,7 +17368,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="17" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:2" hidden="1" x14ac:dyDescent="0.25">
       <c r="A17" s="26" t="s">
         <v>73</v>
       </c>
@@ -17364,7 +17376,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="18" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:2" hidden="1" x14ac:dyDescent="0.25">
       <c r="A18" s="26" t="s">
         <v>75</v>
       </c>
@@ -17372,7 +17384,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="19" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:2" hidden="1" x14ac:dyDescent="0.25">
       <c r="A19" s="26" t="s">
         <v>78</v>
       </c>
@@ -17380,7 +17392,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="20" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:2" hidden="1" x14ac:dyDescent="0.25">
       <c r="A20" s="40" t="s">
         <v>81</v>
       </c>
@@ -17388,7 +17400,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="21" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:2" hidden="1" x14ac:dyDescent="0.25">
       <c r="A21" s="31" t="s">
         <v>85</v>
       </c>
@@ -17396,7 +17408,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="22" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:2" hidden="1" x14ac:dyDescent="0.25">
       <c r="A22" s="31" t="s">
         <v>87</v>
       </c>
@@ -17404,7 +17416,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="23" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:2" hidden="1" x14ac:dyDescent="0.25">
       <c r="A23" s="41" t="s">
         <v>89</v>
       </c>
@@ -17412,7 +17424,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="24" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:2" hidden="1" x14ac:dyDescent="0.25">
       <c r="A24" s="31" t="s">
         <v>91</v>
       </c>
@@ -17420,7 +17432,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="25" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:2" hidden="1" x14ac:dyDescent="0.25">
       <c r="A25" s="31" t="s">
         <v>94</v>
       </c>
@@ -17428,7 +17440,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="26" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:2" hidden="1" x14ac:dyDescent="0.25">
       <c r="A26" s="31" t="s">
         <v>96</v>
       </c>
@@ -17436,7 +17448,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="27" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:2" hidden="1" x14ac:dyDescent="0.25">
       <c r="A27" s="39" t="s">
         <v>98</v>
       </c>
@@ -17444,7 +17456,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="28" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:2" hidden="1" x14ac:dyDescent="0.25">
       <c r="A28" s="31" t="s">
         <v>100</v>
       </c>
@@ -17452,7 +17464,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="29" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:2" hidden="1" x14ac:dyDescent="0.25">
       <c r="A29" s="31" t="s">
         <v>102</v>
       </c>
@@ -17460,7 +17472,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="30" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:2" hidden="1" x14ac:dyDescent="0.25">
       <c r="A30" s="31" t="s">
         <v>104</v>
       </c>
@@ -17468,7 +17480,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="31" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:2" hidden="1" x14ac:dyDescent="0.25">
       <c r="A31" s="31" t="s">
         <v>107</v>
       </c>
@@ -17476,7 +17488,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="32" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:2" hidden="1" x14ac:dyDescent="0.25">
       <c r="A32" s="32" t="s">
         <v>109</v>
       </c>
@@ -17484,7 +17496,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="33" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:2" hidden="1" x14ac:dyDescent="0.25">
       <c r="A33" s="31" t="s">
         <v>112</v>
       </c>
@@ -17492,7 +17504,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="34" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:2" hidden="1" x14ac:dyDescent="0.25">
       <c r="A34" s="31" t="s">
         <v>116</v>
       </c>
@@ -17500,7 +17512,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="35" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:2" hidden="1" x14ac:dyDescent="0.25">
       <c r="A35" s="31" t="s">
         <v>119</v>
       </c>
@@ -17508,7 +17520,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="36" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:2" hidden="1" x14ac:dyDescent="0.25">
       <c r="A36" s="31" t="s">
         <v>122</v>
       </c>
@@ -17516,7 +17528,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="37" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:2" hidden="1" x14ac:dyDescent="0.25">
       <c r="A37" s="31" t="s">
         <v>125</v>
       </c>
@@ -17524,7 +17536,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="38" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:2" hidden="1" x14ac:dyDescent="0.25">
       <c r="A38" s="31" t="s">
         <v>127</v>
       </c>
@@ -17532,7 +17544,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="39" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:2" hidden="1" x14ac:dyDescent="0.25">
       <c r="A39" s="31" t="s">
         <v>129</v>
       </c>
@@ -17540,7 +17552,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="40" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:2" hidden="1" x14ac:dyDescent="0.25">
       <c r="A40" s="31" t="s">
         <v>131</v>
       </c>
@@ -17548,7 +17560,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="41" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:2" hidden="1" x14ac:dyDescent="0.25">
       <c r="A41" s="31" t="s">
         <v>134</v>
       </c>
@@ -17556,7 +17568,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="42" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:2" hidden="1" x14ac:dyDescent="0.25">
       <c r="A42" s="32" t="s">
         <v>136</v>
       </c>
@@ -17564,7 +17576,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="43" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:2" hidden="1" x14ac:dyDescent="0.25">
       <c r="A43" s="31" t="s">
         <v>137</v>
       </c>
@@ -17572,7 +17584,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="44" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:2" hidden="1" x14ac:dyDescent="0.25">
       <c r="A44" s="31" t="s">
         <v>140</v>
       </c>
@@ -17580,7 +17592,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="45" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:2" hidden="1" x14ac:dyDescent="0.25">
       <c r="A45" s="31" t="s">
         <v>143</v>
       </c>
@@ -17588,7 +17600,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="46" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:2" hidden="1" x14ac:dyDescent="0.25">
       <c r="A46" s="31" t="s">
         <v>145</v>
       </c>
@@ -17596,7 +17608,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="47" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:2" hidden="1" x14ac:dyDescent="0.25">
       <c r="A47" s="31" t="s">
         <v>147</v>
       </c>
@@ -17604,7 +17616,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="48" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:2" hidden="1" x14ac:dyDescent="0.25">
       <c r="A48" s="31" t="s">
         <v>150</v>
       </c>
@@ -17612,7 +17624,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="49" spans="1:33" hidden="1" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:33" hidden="1" x14ac:dyDescent="0.25">
       <c r="A49" s="31" t="s">
         <v>152</v>
       </c>
@@ -17620,7 +17632,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="50" spans="1:33" hidden="1" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:33" hidden="1" x14ac:dyDescent="0.25">
       <c r="A50" s="31" t="s">
         <v>153</v>
       </c>
@@ -17628,7 +17640,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="51" spans="1:33" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A51" s="26" t="s">
         <v>156</v>
       </c>
@@ -17726,7 +17738,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="52" spans="1:33" hidden="1" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:33" hidden="1" x14ac:dyDescent="0.25">
       <c r="A52" s="31" t="s">
         <v>159</v>
       </c>
@@ -17734,7 +17746,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="53" spans="1:33" hidden="1" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:33" hidden="1" x14ac:dyDescent="0.25">
       <c r="A53" s="31" t="s">
         <v>160</v>
       </c>
@@ -17742,7 +17754,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="54" spans="1:33" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A54" s="26" t="s">
         <v>162</v>
       </c>
@@ -17840,7 +17852,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="55" spans="1:33" hidden="1" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:33" hidden="1" x14ac:dyDescent="0.25">
       <c r="A55" s="31" t="s">
         <v>165</v>
       </c>
@@ -17848,7 +17860,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="56" spans="1:33" hidden="1" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:33" hidden="1" x14ac:dyDescent="0.25">
       <c r="A56" s="31" t="s">
         <v>168</v>
       </c>
@@ -17940,7 +17952,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="57" spans="1:33" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A57" s="26" t="s">
         <v>169</v>
       </c>
@@ -18038,7 +18050,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="58" spans="1:33" hidden="1" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:33" hidden="1" x14ac:dyDescent="0.25">
       <c r="A58" s="31" t="s">
         <v>172</v>
       </c>
@@ -18046,7 +18058,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="59" spans="1:33" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A59" s="47" t="s">
         <v>174</v>
       </c>
@@ -18144,7 +18156,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="60" spans="1:33" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A60" s="26" t="s">
         <v>177</v>
       </c>
@@ -18242,7 +18254,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="61" spans="1:33" hidden="1" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:33" hidden="1" x14ac:dyDescent="0.25">
       <c r="A61" s="31" t="s">
         <v>180</v>
       </c>
@@ -18340,7 +18352,7 @@
         <v>0.5</v>
       </c>
     </row>
-    <row r="62" spans="1:33" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A62" s="47" t="s">
         <v>181</v>
       </c>
@@ -18438,7 +18450,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="63" spans="1:33" hidden="1" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:33" hidden="1" x14ac:dyDescent="0.25">
       <c r="A63" s="31" t="s">
         <v>184</v>
       </c>
@@ -18446,7 +18458,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="64" spans="1:33" hidden="1" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:33" hidden="1" x14ac:dyDescent="0.25">
       <c r="A64" s="32" t="s">
         <v>185</v>
       </c>
@@ -18454,7 +18466,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="65" spans="1:33" hidden="1" x14ac:dyDescent="0.35">
+    <row r="65" spans="1:33" hidden="1" x14ac:dyDescent="0.25">
       <c r="A65" s="31" t="s">
         <v>186</v>
       </c>
@@ -18462,7 +18474,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="66" spans="1:33" x14ac:dyDescent="0.35">
+    <row r="66" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A66" s="26" t="s">
         <v>187</v>
       </c>
@@ -18560,7 +18572,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="67" spans="1:33" hidden="1" x14ac:dyDescent="0.35">
+    <row r="67" spans="1:33" hidden="1" x14ac:dyDescent="0.25">
       <c r="A67" s="31" t="s">
         <v>190</v>
       </c>
@@ -18568,7 +18580,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="68" spans="1:33" x14ac:dyDescent="0.35">
+    <row r="68" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A68" s="26" t="s">
         <v>194</v>
       </c>
@@ -18666,7 +18678,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="69" spans="1:33" x14ac:dyDescent="0.35">
+    <row r="69" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A69" s="47" t="s">
         <v>197</v>
       </c>
@@ -18764,7 +18776,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="70" spans="1:33" x14ac:dyDescent="0.35">
+    <row r="70" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A70" s="26" t="s">
         <v>200</v>
       </c>
@@ -18862,7 +18874,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="71" spans="1:33" x14ac:dyDescent="0.35">
+    <row r="71" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A71" s="26" t="s">
         <v>204</v>
       </c>
@@ -18960,7 +18972,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="72" spans="1:33" x14ac:dyDescent="0.35">
+    <row r="72" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A72" s="26" t="s">
         <v>206</v>
       </c>
@@ -19058,7 +19070,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="73" spans="1:33" x14ac:dyDescent="0.35">
+    <row r="73" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A73" s="26" t="s">
         <v>209</v>
       </c>
@@ -19156,7 +19168,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="74" spans="1:33" x14ac:dyDescent="0.35">
+    <row r="74" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A74" s="26" t="s">
         <v>212</v>
       </c>
@@ -19254,7 +19266,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="75" spans="1:33" x14ac:dyDescent="0.35">
+    <row r="75" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A75" s="47" t="s">
         <v>215</v>
       </c>
@@ -19349,7 +19361,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="77" spans="1:33" x14ac:dyDescent="0.35">
+    <row r="77" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
         <v>274</v>
       </c>
@@ -19475,7 +19487,7 @@
         <v>0.36666666666666664</v>
       </c>
     </row>
-    <row r="78" spans="1:33" x14ac:dyDescent="0.35">
+    <row r="78" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
         <v>373</v>
       </c>
@@ -19601,7 +19613,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="79" spans="1:33" x14ac:dyDescent="0.35">
+    <row r="79" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
         <v>278</v>
       </c>
@@ -19622,7 +19634,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="80" spans="1:33" x14ac:dyDescent="0.35">
+    <row r="80" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
         <v>374</v>
       </c>

</xml_diff>

<commit_message>
IK/ID 019 SO/MA til SLS_front_pre3
</commit_message>
<xml_diff>
--- a/ParticipantData and Labelling.xlsx
+++ b/ParticipantData and Labelling.xlsx
@@ -1,23 +1,23 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29231"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Git\research_data\Projects\squatting_fais\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Basilio\Documents\Thesis_Gigler\squatting_fais\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7E2CEF6C-F7C1-4689-9D80-2821F3376766}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A4EE349B-463E-4031-AFF8-76C492EAC905}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="798" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="14020" tabRatio="798" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Demographics" sheetId="1" r:id="rId1"/>
-    <sheet name="Next steps" sheetId="9" r:id="rId2"/>
-    <sheet name="Marker weighings" sheetId="11" r:id="rId3"/>
+    <sheet name="Marker weighings" sheetId="11" r:id="rId2"/>
+    <sheet name="Next steps" sheetId="9" r:id="rId3"/>
     <sheet name="Processing" sheetId="7" r:id="rId4"/>
-    <sheet name="Events" sheetId="12" r:id="rId5"/>
+    <sheet name="Analysis IK;ID;SO" sheetId="12" r:id="rId5"/>
     <sheet name="PreviousTreatments" sheetId="3" r:id="rId6"/>
     <sheet name="iHOT" sheetId="4" r:id="rId7"/>
     <sheet name="HAGOS" sheetId="5" r:id="rId8"/>
@@ -25,19 +25,6 @@
     <sheet name="Add&amp;GracEMGLocation" sheetId="8" r:id="rId10"/>
   </sheets>
   <calcPr calcId="191029"/>
-  <extLst>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
-  </extLst>
 </workbook>
 </file>
 
@@ -634,7 +621,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1444" uniqueCount="437">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1625" uniqueCount="559">
   <si>
     <t>Subject</t>
   </si>
@@ -1951,9 +1938,6 @@
     <t>Squat_used</t>
   </si>
   <si>
-    <t>Run Inverse kinematics from GUI for one single participant (all trials)</t>
-  </si>
-  <si>
     <t>SLSback1</t>
   </si>
   <si>
@@ -2014,25 +1998,394 @@
     <t xml:space="preserve">Best IK so far </t>
   </si>
   <si>
-    <t>2.75,3.4</t>
-  </si>
-  <si>
     <t>CAM</t>
   </si>
   <si>
     <t>Control</t>
   </si>
   <si>
-    <t xml:space="preserve">export patient 064 c3d </t>
-  </si>
-  <si>
-    <t>complete processing tab with participants group</t>
-  </si>
-  <si>
-    <t>Run inverse dynamics from GUI</t>
-  </si>
-  <si>
-    <t>3.355, 3.715, 4.3</t>
+    <t>done</t>
+  </si>
+  <si>
+    <t xml:space="preserve">done </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Notes </t>
+  </si>
+  <si>
+    <t>average marker Errors: below 0.05</t>
+  </si>
+  <si>
+    <t xml:space="preserve">041: SJ1-5 long plataeu lowest point &amp; jump </t>
+  </si>
+  <si>
+    <t>077 long plataeus</t>
+  </si>
+  <si>
+    <t>2,2 -5,6</t>
+  </si>
+  <si>
+    <t>2,6-5,65</t>
+  </si>
+  <si>
+    <t>2 - 5,45</t>
+  </si>
+  <si>
+    <t>1,6-5,5</t>
+  </si>
+  <si>
+    <t>5,5-8,6</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2,0 - 6,0 </t>
+  </si>
+  <si>
+    <t>2,7 - 6,2</t>
+  </si>
+  <si>
+    <t>1,5-5,25</t>
+  </si>
+  <si>
+    <t>2,4 - 6,1</t>
+  </si>
+  <si>
+    <t>2,0-5,9</t>
+  </si>
+  <si>
+    <t>1,75 - 6,0</t>
+  </si>
+  <si>
+    <t>2,7 - 6,7</t>
+  </si>
+  <si>
+    <t>3,0-7,5</t>
+  </si>
+  <si>
+    <t>2,9-7,2</t>
+  </si>
+  <si>
+    <t>2,0 -6,9</t>
+  </si>
+  <si>
+    <t>1,5 - 5</t>
+  </si>
+  <si>
+    <t>2,4 -5,6</t>
+  </si>
+  <si>
+    <t>0,9-5,4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1,6 - 6,0 </t>
+  </si>
+  <si>
+    <t>2,2 - 6,0</t>
+  </si>
+  <si>
+    <t>2,5 - 7,1</t>
+  </si>
+  <si>
+    <t>1,0 - 6,85</t>
+  </si>
+  <si>
+    <t>2,2 - 8,5</t>
+  </si>
+  <si>
+    <t>2,75 - 8,6</t>
+  </si>
+  <si>
+    <t>2,5 - 8,0</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1,4 - 4,9 </t>
+  </si>
+  <si>
+    <t>2,0 - 7,0</t>
+  </si>
+  <si>
+    <t>3,0 -8,5</t>
+  </si>
+  <si>
+    <t>1,6 - 7,3</t>
+  </si>
+  <si>
+    <t>1,3 -4,25</t>
+  </si>
+  <si>
+    <t>2,45 -5,7</t>
+  </si>
+  <si>
+    <t>2,5 -5,8</t>
+  </si>
+  <si>
+    <t>1,3 -4,2</t>
+  </si>
+  <si>
+    <t>1,4 - 4,9</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fehlversuch </t>
+  </si>
+  <si>
+    <t>1,9 - 4,4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1,5 - 4,0 </t>
+  </si>
+  <si>
+    <t>1,0 -3,75</t>
+  </si>
+  <si>
+    <t>1,25 - 5,0</t>
+  </si>
+  <si>
+    <t>1,0 -4,6</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3,5 -6,9 </t>
+  </si>
+  <si>
+    <t>3,6 - 7,4</t>
+  </si>
+  <si>
+    <t>2,0 -6,0</t>
+  </si>
+  <si>
+    <t>1,25 -4,9</t>
+  </si>
+  <si>
+    <t>1,7 -5,4</t>
+  </si>
+  <si>
+    <t>1,6 -5,6</t>
+  </si>
+  <si>
+    <t>2- 5,5</t>
+  </si>
+  <si>
+    <t>2,5-6,3</t>
+  </si>
+  <si>
+    <t>1,3 -5</t>
+  </si>
+  <si>
+    <t>1,5-4,9</t>
+  </si>
+  <si>
+    <t>3,1 -7,0</t>
+  </si>
+  <si>
+    <t>2,0 - 5,2</t>
+  </si>
+  <si>
+    <t>1,8 - 5,5</t>
+  </si>
+  <si>
+    <t>2,25 -5,55</t>
+  </si>
+  <si>
+    <t>2,0 -5,25</t>
+  </si>
+  <si>
+    <t>1,9 -6,0</t>
+  </si>
+  <si>
+    <t>1,9 - 4,9</t>
+  </si>
+  <si>
+    <t>1,4 -4,55</t>
+  </si>
+  <si>
+    <t>2,25 - 5,4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1,7 -5,1 </t>
+  </si>
+  <si>
+    <t>1,5 -5,5</t>
+  </si>
+  <si>
+    <t>1,9 -5,1</t>
+  </si>
+  <si>
+    <t>1,5 - 5,2</t>
+  </si>
+  <si>
+    <t>1,5 - 4,5</t>
+  </si>
+  <si>
+    <t>1,25 -4,75</t>
+  </si>
+  <si>
+    <t>1,75 -5,6</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2,6 -6,0 </t>
+  </si>
+  <si>
+    <t xml:space="preserve">1,25- 4,5 </t>
+  </si>
+  <si>
+    <t>3,8 - 6,9</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2,8 -5,9 </t>
+  </si>
+  <si>
+    <t>2,6 -5,5</t>
+  </si>
+  <si>
+    <t>2,9 -6,1</t>
+  </si>
+  <si>
+    <t>2,0 -5,1</t>
+  </si>
+  <si>
+    <t>2,0 -5,0</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2,1-5,7 </t>
+  </si>
+  <si>
+    <t>2,25-5,25</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1,0 -5,8 </t>
+  </si>
+  <si>
+    <t>0,9 -5,25</t>
+  </si>
+  <si>
+    <t>1,2 -5,5</t>
+  </si>
+  <si>
+    <t>1,2 -5,25</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1,6 -6,0 </t>
+  </si>
+  <si>
+    <t>1,2 - 5,1</t>
+  </si>
+  <si>
+    <t>1,0 - 5,0</t>
+  </si>
+  <si>
+    <t>1,0 - 5,2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0,5 - 4,5 </t>
+  </si>
+  <si>
+    <t>1,7 - 4,45</t>
+  </si>
+  <si>
+    <t>1,6 - 4,5</t>
+  </si>
+  <si>
+    <t>1,75 - 4,5</t>
+  </si>
+  <si>
+    <t>1,7 - 4,25</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1,4 - 4,0 </t>
+  </si>
+  <si>
+    <t>1,2 - 4,6</t>
+  </si>
+  <si>
+    <t>1,45 - 5,5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1,8 -4,8 </t>
+  </si>
+  <si>
+    <t>1,75 -5,1</t>
+  </si>
+  <si>
+    <t>1,4 - 5,4</t>
+  </si>
+  <si>
+    <t>6,0 -10,1</t>
+  </si>
+  <si>
+    <t>4,0 - 7,9</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3,5 - 6,9 </t>
+  </si>
+  <si>
+    <t>3,5 - 7,0</t>
+  </si>
+  <si>
+    <t>2,0 - 5,8</t>
+  </si>
+  <si>
+    <t>1,6 - 5,8</t>
+  </si>
+  <si>
+    <t>3,1 - 7,1</t>
+  </si>
+  <si>
+    <t>2,5 - 6,25</t>
+  </si>
+  <si>
+    <t>2,8 - 6,45</t>
+  </si>
+  <si>
+    <t>3,2 - 7,1</t>
+  </si>
+  <si>
+    <t>2,3 -5,85</t>
+  </si>
+  <si>
+    <t>3,0 - 5,7</t>
+  </si>
+  <si>
+    <t>2,6 - 6,1</t>
+  </si>
+  <si>
+    <t>2,1 - 4,9</t>
+  </si>
+  <si>
+    <t>3,0 - 5,9</t>
+  </si>
+  <si>
+    <t>9,6 - 12,95</t>
+  </si>
+  <si>
+    <t>5,0 - 8,0</t>
+  </si>
+  <si>
+    <t>1,25 - 5,1</t>
+  </si>
+  <si>
+    <t>2,9 - 5,6</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2,0 - 5,1 </t>
+  </si>
+  <si>
+    <t>1,5 - 5,25</t>
+  </si>
+  <si>
+    <t xml:space="preserve">17.08 Update </t>
+  </si>
+  <si>
+    <t xml:space="preserve">All events detected for all trials </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Until 18.08 </t>
+  </si>
+  <si>
+    <t xml:space="preserve">IK, ID &amp; SO for all trials </t>
+  </si>
+  <si>
+    <t xml:space="preserve">If time until 18.08 </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Angle, Moment &amp; muscel force analysis for all trials 1 Participant </t>
   </si>
 </sst>
 </file>
@@ -2149,7 +2502,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="18">
+  <fills count="19">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -2249,6 +2602,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="0"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFF0000"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -2353,7 +2712,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="78">
+  <cellXfs count="85">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
@@ -2531,11 +2890,26 @@
       <alignment vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="18" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="17" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="16" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -3321,9 +3695,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
-    <a:clrScheme name="Office 2013 - 2022">
+    <a:clrScheme name="Office">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -3361,7 +3735,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office 2013 - 2022">
+    <a:fontScheme name="Office">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -3467,7 +3841,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office 2013 - 2022">
+    <a:fmtScheme name="Office">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -3609,7 +3983,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -3618,25 +3992,25 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:AI74"/>
-  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="9.1796875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="10" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="7.85546875" customWidth="1"/>
-    <col min="4" max="5" width="7.5703125" customWidth="1"/>
-    <col min="6" max="6" width="12.85546875" bestFit="1" customWidth="1"/>
-    <col min="7" max="20" width="7.5703125" customWidth="1"/>
+    <col min="2" max="2" width="7.81640625" customWidth="1"/>
+    <col min="4" max="5" width="7.54296875" customWidth="1"/>
+    <col min="6" max="6" width="12.81640625" bestFit="1" customWidth="1"/>
+    <col min="7" max="20" width="7.54296875" customWidth="1"/>
     <col min="21" max="21" width="10" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="9.28515625" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="22.28515625" customWidth="1"/>
-    <col min="24" max="24" width="26.7109375" customWidth="1"/>
-    <col min="25" max="27" width="14.42578125" customWidth="1"/>
-    <col min="28" max="32" width="8.7109375" customWidth="1"/>
-    <col min="33" max="34" width="8.7109375" style="11" customWidth="1"/>
-    <col min="35" max="35" width="12.42578125" style="11" customWidth="1"/>
-    <col min="36" max="36" width="15.7109375" customWidth="1"/>
+    <col min="22" max="22" width="9.26953125" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="22.26953125" customWidth="1"/>
+    <col min="24" max="24" width="26.7265625" customWidth="1"/>
+    <col min="25" max="27" width="14.453125" customWidth="1"/>
+    <col min="28" max="32" width="8.7265625" customWidth="1"/>
+    <col min="33" max="34" width="8.7265625" style="11" customWidth="1"/>
+    <col min="35" max="35" width="12.453125" style="11" customWidth="1"/>
+    <col min="36" max="36" width="15.7265625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:35" ht="45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:35" ht="45" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -3743,7 +4117,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="2" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A2" s="26" t="s">
         <v>59</v>
       </c>
@@ -3832,7 +4206,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="3" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A3" s="26" t="s">
         <v>62</v>
       </c>
@@ -3920,7 +4294,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="4" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A4" s="26" t="s">
         <v>64</v>
       </c>
@@ -3984,7 +4358,7 @@
       <c r="AG4"/>
       <c r="AH4"/>
     </row>
-    <row r="5" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A5" s="26" t="s">
         <v>65</v>
       </c>
@@ -4068,7 +4442,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="6" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A6" s="26" t="s">
         <v>67</v>
       </c>
@@ -4155,7 +4529,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="7" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A7" s="26" t="s">
         <v>69</v>
       </c>
@@ -4238,7 +4612,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="8" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A8" s="26" t="s">
         <v>71</v>
       </c>
@@ -4323,7 +4697,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="9" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A9" s="26" t="s">
         <v>73</v>
       </c>
@@ -4410,7 +4784,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="10" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A10" s="26" t="s">
         <v>75</v>
       </c>
@@ -4497,7 +4871,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="11" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A11" s="26" t="s">
         <v>78</v>
       </c>
@@ -4590,7 +4964,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="12" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A12" s="31" t="s">
         <v>81</v>
       </c>
@@ -4678,7 +5052,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="13" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A13" s="31" t="s">
         <v>85</v>
       </c>
@@ -4762,7 +5136,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="14" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A14" s="31" t="s">
         <v>87</v>
       </c>
@@ -4852,7 +5226,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="15" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A15" s="31" t="s">
         <v>89</v>
       </c>
@@ -4940,7 +5314,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="16" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A16" s="31" t="s">
         <v>91</v>
       </c>
@@ -5027,7 +5401,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="17" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A17" s="31" t="s">
         <v>94</v>
       </c>
@@ -5111,7 +5485,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="18" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A18" s="31" t="s">
         <v>96</v>
       </c>
@@ -5195,7 +5569,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="19" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A19" s="31" t="s">
         <v>98</v>
       </c>
@@ -5276,7 +5650,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="20" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A20" s="31" t="s">
         <v>100</v>
       </c>
@@ -5360,7 +5734,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="21" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A21" s="31" t="s">
         <v>102</v>
       </c>
@@ -5445,7 +5819,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="22" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A22" s="31" t="s">
         <v>104</v>
       </c>
@@ -5535,7 +5909,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="23" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A23" s="31" t="s">
         <v>107</v>
       </c>
@@ -5625,7 +5999,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="24" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A24" s="31" t="s">
         <v>109</v>
       </c>
@@ -5710,7 +6084,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="25" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A25" s="31" t="s">
         <v>112</v>
       </c>
@@ -5804,7 +6178,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="26" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A26" s="31" t="s">
         <v>116</v>
       </c>
@@ -5892,7 +6266,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="27" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A27" s="31" t="s">
         <v>119</v>
       </c>
@@ -5962,7 +6336,7 @@
       <c r="AG27"/>
       <c r="AH27"/>
     </row>
-    <row r="28" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A28" s="73" t="s">
         <v>122</v>
       </c>
@@ -6055,7 +6429,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="29" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A29" s="31" t="s">
         <v>125</v>
       </c>
@@ -6145,7 +6519,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="30" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A30" s="71" t="s">
         <v>127</v>
       </c>
@@ -6238,7 +6612,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="31" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A31" s="71" t="s">
         <v>129</v>
       </c>
@@ -6331,7 +6705,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="32" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A32" s="71" t="s">
         <v>131</v>
       </c>
@@ -6424,7 +6798,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="33" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A33" s="71" t="s">
         <v>134</v>
       </c>
@@ -6517,7 +6891,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="34" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A34" s="31" t="s">
         <v>136</v>
       </c>
@@ -6581,7 +6955,7 @@
       <c r="AG34"/>
       <c r="AH34"/>
     </row>
-    <row r="35" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A35" s="31" t="s">
         <v>137</v>
       </c>
@@ -6672,7 +7046,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="36" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A36" s="71" t="s">
         <v>140</v>
       </c>
@@ -6765,7 +7139,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="37" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A37" s="31" t="s">
         <v>143</v>
       </c>
@@ -6847,7 +7221,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="38" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A38" s="31" t="s">
         <v>145</v>
       </c>
@@ -6915,7 +7289,7 @@
       <c r="AG38"/>
       <c r="AH38"/>
     </row>
-    <row r="39" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A39" s="71" t="s">
         <v>147</v>
       </c>
@@ -7010,7 +7384,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="40" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A40" s="31" t="s">
         <v>150</v>
       </c>
@@ -7102,7 +7476,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="41" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A41" s="31" t="s">
         <v>152</v>
       </c>
@@ -7175,7 +7549,7 @@
       <c r="AG41"/>
       <c r="AH41"/>
     </row>
-    <row r="42" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A42" s="31" t="s">
         <v>153</v>
       </c>
@@ -7267,7 +7641,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="43" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A43" s="31" t="s">
         <v>156</v>
       </c>
@@ -7367,7 +7741,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="44" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A44" s="31" t="s">
         <v>159</v>
       </c>
@@ -7434,7 +7808,7 @@
       <c r="AG44"/>
       <c r="AH44"/>
     </row>
-    <row r="45" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A45" s="71" t="s">
         <v>160</v>
       </c>
@@ -7527,7 +7901,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="46" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A46" s="31" t="s">
         <v>162</v>
       </c>
@@ -7633,7 +8007,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="47" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A47" s="31" t="s">
         <v>165</v>
       </c>
@@ -7723,7 +8097,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="48" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A48" s="31" t="s">
         <v>168</v>
       </c>
@@ -7793,7 +8167,7 @@
       <c r="AG48"/>
       <c r="AH48"/>
     </row>
-    <row r="49" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A49" s="31" t="s">
         <v>169</v>
       </c>
@@ -7902,7 +8276,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="50" spans="1:35" s="11" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:35" s="11" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A50" s="31" t="s">
         <v>172</v>
       </c>
@@ -7975,7 +8349,7 @@
       <c r="AG50"/>
       <c r="AH50"/>
     </row>
-    <row r="51" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A51" s="31" t="s">
         <v>174</v>
       </c>
@@ -8084,7 +8458,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="52" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A52" s="31" t="s">
         <v>177</v>
       </c>
@@ -8194,7 +8568,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="53" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A53" s="31" t="s">
         <v>180</v>
       </c>
@@ -8268,7 +8642,7 @@
       <c r="AG53"/>
       <c r="AH53"/>
     </row>
-    <row r="54" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A54" s="71" t="s">
         <v>181</v>
       </c>
@@ -8374,7 +8748,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="55" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A55" s="31" t="s">
         <v>184</v>
       </c>
@@ -8447,7 +8821,7 @@
       <c r="AG55"/>
       <c r="AH55"/>
     </row>
-    <row r="56" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A56" s="31" t="s">
         <v>185</v>
       </c>
@@ -8528,7 +8902,7 @@
       <c r="AG56"/>
       <c r="AH56"/>
     </row>
-    <row r="57" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A57" s="31" t="s">
         <v>186</v>
       </c>
@@ -8601,7 +8975,7 @@
       <c r="AG57"/>
       <c r="AH57"/>
     </row>
-    <row r="58" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A58" s="31" t="s">
         <v>187</v>
       </c>
@@ -8710,7 +9084,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="59" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A59" s="31" t="s">
         <v>190</v>
       </c>
@@ -8817,7 +9191,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="60" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A60" s="31" t="s">
         <v>194</v>
       </c>
@@ -8926,7 +9300,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="61" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A61" s="71" t="s">
         <v>197</v>
       </c>
@@ -9038,7 +9412,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="62" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A62" s="31" t="s">
         <v>200</v>
       </c>
@@ -9148,7 +9522,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="63" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A63" s="71" t="s">
         <v>204</v>
       </c>
@@ -9260,7 +9634,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="64" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A64" s="71" t="s">
         <v>206</v>
       </c>
@@ -9372,7 +9746,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="65" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A65" s="71" t="s">
         <v>209</v>
       </c>
@@ -9484,7 +9858,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="66" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:35" s="11" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A66" s="31" t="s">
         <v>212</v>
       </c>
@@ -9595,7 +9969,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="67" spans="1:35" s="11" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:35" s="11" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A67" s="31" t="s">
         <v>215</v>
       </c>
@@ -9703,7 +10077,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="68" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A68" s="1"/>
       <c r="B68" s="36"/>
       <c r="Q68" s="63"/>
@@ -9721,7 +10095,7 @@
       <c r="AG68"/>
       <c r="AH68"/>
     </row>
-    <row r="69" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A69" s="64"/>
       <c r="B69" s="64"/>
       <c r="C69" s="64"/>
@@ -9758,7 +10132,7 @@
       <c r="AH69" s="64"/>
       <c r="AI69" s="64"/>
     </row>
-    <row r="70" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A70" s="64"/>
       <c r="B70" s="64"/>
       <c r="C70" s="64"/>
@@ -9795,7 +10169,7 @@
       <c r="AH70" s="64"/>
       <c r="AI70" s="64"/>
     </row>
-    <row r="71" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A71" s="64"/>
       <c r="B71" s="64"/>
       <c r="C71" s="64"/>
@@ -9832,7 +10206,7 @@
       <c r="AH71" s="64"/>
       <c r="AI71" s="64"/>
     </row>
-    <row r="72" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A72" s="64"/>
       <c r="B72" s="64"/>
       <c r="C72" s="64"/>
@@ -9869,7 +10243,7 @@
       <c r="AH72" s="64"/>
       <c r="AI72" s="64"/>
     </row>
-    <row r="73" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:35" x14ac:dyDescent="0.35">
       <c r="B73" s="36">
         <f>AVERAGE(B3,B11,B21,B23,B28,B30,B36,B45,B63,B64,B65,B67)</f>
         <v>26.833333333333332</v>
@@ -9882,7 +10256,7 @@
       <c r="AG73"/>
       <c r="AH73"/>
     </row>
-    <row r="74" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:35" x14ac:dyDescent="0.35">
       <c r="R74" s="64"/>
       <c r="AG74"/>
       <c r="AH74"/>
@@ -9900,9 +10274,9 @@
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0700-000000000000}">
   <dimension ref="A1:E11"/>
-  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="8.7265625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -9919,7 +10293,7 @@
         <v>406</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A2" s="1" t="s">
         <v>215</v>
       </c>
@@ -9940,7 +10314,7 @@
         <v>0.5</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A3" s="1" t="s">
         <v>212</v>
       </c>
@@ -9961,7 +10335,7 @@
         <v>0.5</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A4" s="1" t="s">
         <v>206</v>
       </c>
@@ -9982,7 +10356,7 @@
         <v>0.5</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A5" s="1" t="s">
         <v>204</v>
       </c>
@@ -10003,7 +10377,7 @@
         <v>0.45</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A6" s="1" t="s">
         <v>197</v>
       </c>
@@ -10024,7 +10398,7 @@
         <v>0.44444444444444442</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A7" s="1" t="s">
         <v>194</v>
       </c>
@@ -10045,7 +10419,7 @@
         <v>0.40909090909090912</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A8" s="1" t="s">
         <v>190</v>
       </c>
@@ -10066,7 +10440,7 @@
         <v>0.51282051282051277</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A9" s="1" t="s">
         <v>185</v>
       </c>
@@ -10087,7 +10461,7 @@
         <v>0.5</v>
       </c>
     </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>274</v>
       </c>
@@ -10108,7 +10482,7 @@
         <v>0.47704448329448329</v>
       </c>
     </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>407</v>
       </c>
@@ -10135,81 +10509,39 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{89B2075C-5F56-4EF1-95BD-F5E1A85C949C}">
-  <dimension ref="A1:B4"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A1">
-        <v>1</v>
-      </c>
-      <c r="B1" t="s">
-        <v>434</v>
-      </c>
-    </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A2">
-        <v>2</v>
-      </c>
-      <c r="B2" t="s">
-        <v>433</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A3">
-        <v>3</v>
-      </c>
-      <c r="B3" t="s">
-        <v>409</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A4">
-        <v>4</v>
-      </c>
-      <c r="B4" t="s">
-        <v>435</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{12AC9CB0-5B51-495B-9318-23D7E97CB111}">
   <dimension ref="A2:J20"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="11.42578125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="11.453125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
+        <v>416</v>
+      </c>
+      <c r="B2" t="s">
         <v>417</v>
       </c>
-      <c r="B2" t="s">
+      <c r="C2" t="s">
         <v>418</v>
       </c>
-      <c r="C2" t="s">
+      <c r="D2" t="s">
         <v>419</v>
       </c>
-      <c r="D2" t="s">
+      <c r="E2" t="s">
         <v>420</v>
       </c>
-      <c r="E2" t="s">
-        <v>421</v>
-      </c>
       <c r="F2" t="s">
-        <v>423</v>
-      </c>
-      <c r="H2" s="76" t="s">
-        <v>425</v>
-      </c>
-      <c r="I2" s="76"/>
-      <c r="J2" s="76"/>
-    </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
+        <v>422</v>
+      </c>
+      <c r="H2" s="82" t="s">
+        <v>424</v>
+      </c>
+      <c r="I2" s="82"/>
+      <c r="J2" s="82"/>
+    </row>
+    <row r="3" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A3">
         <v>10</v>
       </c>
@@ -10223,133 +10555,133 @@
         <v>7</v>
       </c>
       <c r="E3" t="s">
-        <v>422</v>
+        <v>421</v>
       </c>
       <c r="F3">
         <v>1</v>
       </c>
       <c r="H3" t="s">
-        <v>424</v>
+        <v>423</v>
       </c>
       <c r="I3">
         <v>0.1</v>
       </c>
     </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:10" x14ac:dyDescent="0.35">
       <c r="H4" t="s">
-        <v>426</v>
+        <v>425</v>
       </c>
       <c r="I4">
         <v>7.0000000000000007E-2</v>
       </c>
     </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="F10" s="76" t="s">
-        <v>429</v>
-      </c>
-      <c r="G10" s="76"/>
-      <c r="H10" s="76"/>
-      <c r="I10" s="76"/>
-      <c r="J10" s="76"/>
-    </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A11" s="77" t="s">
+    <row r="10" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="F10" s="82" t="s">
+        <v>428</v>
+      </c>
+      <c r="G10" s="82"/>
+      <c r="H10" s="82"/>
+      <c r="I10" s="82"/>
+      <c r="J10" s="82"/>
+    </row>
+    <row r="11" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A11" s="83" t="s">
+        <v>426</v>
+      </c>
+      <c r="B11" s="83"/>
+      <c r="C11" s="83"/>
+      <c r="D11" s="83"/>
+    </row>
+    <row r="12" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A12" s="83"/>
+      <c r="B12" s="83"/>
+      <c r="C12" s="83"/>
+      <c r="D12" s="83"/>
+      <c r="F12" s="83" t="s">
         <v>427</v>
       </c>
-      <c r="B11" s="77"/>
-      <c r="C11" s="77"/>
-      <c r="D11" s="77"/>
-    </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A12" s="77"/>
-      <c r="B12" s="77"/>
-      <c r="C12" s="77"/>
-      <c r="D12" s="77"/>
-      <c r="F12" s="77" t="s">
-        <v>428</v>
-      </c>
-      <c r="G12" s="77"/>
-      <c r="H12" s="77"/>
-      <c r="I12" s="77"/>
-      <c r="J12" s="77"/>
-    </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A13" s="77"/>
-      <c r="B13" s="77"/>
-      <c r="C13" s="77"/>
-      <c r="D13" s="77"/>
-      <c r="F13" s="77"/>
-      <c r="G13" s="77"/>
-      <c r="H13" s="77"/>
-      <c r="I13" s="77"/>
-      <c r="J13" s="77"/>
-    </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A14" s="77"/>
-      <c r="B14" s="77"/>
-      <c r="C14" s="77"/>
-      <c r="D14" s="77"/>
-      <c r="F14" s="77"/>
-      <c r="G14" s="77"/>
-      <c r="H14" s="77"/>
-      <c r="I14" s="77"/>
-      <c r="J14" s="77"/>
-    </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A15" s="77"/>
-      <c r="B15" s="77"/>
-      <c r="C15" s="77"/>
-      <c r="D15" s="77"/>
-      <c r="F15" s="77"/>
-      <c r="G15" s="77"/>
-      <c r="H15" s="77"/>
-      <c r="I15" s="77"/>
-      <c r="J15" s="77"/>
-    </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A16" s="77"/>
-      <c r="B16" s="77"/>
-      <c r="C16" s="77"/>
-      <c r="D16" s="77"/>
-      <c r="F16" s="77"/>
-      <c r="G16" s="77"/>
-      <c r="H16" s="77"/>
-      <c r="I16" s="77"/>
-      <c r="J16" s="77"/>
-    </row>
-    <row r="17" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A17" s="77"/>
-      <c r="B17" s="77"/>
-      <c r="C17" s="77"/>
-      <c r="D17" s="77"/>
-      <c r="F17" s="77"/>
-      <c r="G17" s="77"/>
-      <c r="H17" s="77"/>
-      <c r="I17" s="77"/>
-      <c r="J17" s="77"/>
-    </row>
-    <row r="18" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A18" s="77"/>
-      <c r="B18" s="77"/>
-      <c r="C18" s="77"/>
-      <c r="D18" s="77"/>
-      <c r="F18" s="77"/>
-      <c r="G18" s="77"/>
-      <c r="H18" s="77"/>
-      <c r="I18" s="77"/>
-      <c r="J18" s="77"/>
-    </row>
-    <row r="19" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A19" s="77"/>
-      <c r="B19" s="77"/>
-      <c r="C19" s="77"/>
-      <c r="D19" s="77"/>
-    </row>
-    <row r="20" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A20" s="77"/>
-      <c r="B20" s="77"/>
-      <c r="C20" s="77"/>
-      <c r="D20" s="77"/>
+      <c r="G12" s="83"/>
+      <c r="H12" s="83"/>
+      <c r="I12" s="83"/>
+      <c r="J12" s="83"/>
+    </row>
+    <row r="13" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A13" s="83"/>
+      <c r="B13" s="83"/>
+      <c r="C13" s="83"/>
+      <c r="D13" s="83"/>
+      <c r="F13" s="83"/>
+      <c r="G13" s="83"/>
+      <c r="H13" s="83"/>
+      <c r="I13" s="83"/>
+      <c r="J13" s="83"/>
+    </row>
+    <row r="14" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A14" s="83"/>
+      <c r="B14" s="83"/>
+      <c r="C14" s="83"/>
+      <c r="D14" s="83"/>
+      <c r="F14" s="83"/>
+      <c r="G14" s="83"/>
+      <c r="H14" s="83"/>
+      <c r="I14" s="83"/>
+      <c r="J14" s="83"/>
+    </row>
+    <row r="15" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A15" s="83"/>
+      <c r="B15" s="83"/>
+      <c r="C15" s="83"/>
+      <c r="D15" s="83"/>
+      <c r="F15" s="83"/>
+      <c r="G15" s="83"/>
+      <c r="H15" s="83"/>
+      <c r="I15" s="83"/>
+      <c r="J15" s="83"/>
+    </row>
+    <row r="16" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A16" s="83"/>
+      <c r="B16" s="83"/>
+      <c r="C16" s="83"/>
+      <c r="D16" s="83"/>
+      <c r="F16" s="83"/>
+      <c r="G16" s="83"/>
+      <c r="H16" s="83"/>
+      <c r="I16" s="83"/>
+      <c r="J16" s="83"/>
+    </row>
+    <row r="17" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A17" s="83"/>
+      <c r="B17" s="83"/>
+      <c r="C17" s="83"/>
+      <c r="D17" s="83"/>
+      <c r="F17" s="83"/>
+      <c r="G17" s="83"/>
+      <c r="H17" s="83"/>
+      <c r="I17" s="83"/>
+      <c r="J17" s="83"/>
+    </row>
+    <row r="18" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A18" s="83"/>
+      <c r="B18" s="83"/>
+      <c r="C18" s="83"/>
+      <c r="D18" s="83"/>
+      <c r="F18" s="83"/>
+      <c r="G18" s="83"/>
+      <c r="H18" s="83"/>
+      <c r="I18" s="83"/>
+      <c r="J18" s="83"/>
+    </row>
+    <row r="19" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A19" s="83"/>
+      <c r="B19" s="83"/>
+      <c r="C19" s="83"/>
+      <c r="D19" s="83"/>
+    </row>
+    <row r="20" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A20" s="83"/>
+      <c r="B20" s="83"/>
+      <c r="C20" s="83"/>
+      <c r="D20" s="83"/>
     </row>
   </sheetData>
   <mergeCells count="4">
@@ -10362,16 +10694,113 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{89B2075C-5F56-4EF1-95BD-F5E1A85C949C}">
+  <dimension ref="A3:H14"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="25.6328125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A3" s="84" t="s">
+        <v>553</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
+        <v>554</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A6" s="84" t="s">
+        <v>555</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A7" t="s">
+        <v>556</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A9" s="84" t="s">
+        <v>557</v>
+      </c>
+      <c r="B9" s="77"/>
+      <c r="C9" s="77"/>
+      <c r="D9" s="77"/>
+      <c r="E9" s="77"/>
+      <c r="F9" s="77"/>
+      <c r="G9" s="77"/>
+      <c r="H9" s="77"/>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A10" t="s">
+        <v>558</v>
+      </c>
+      <c r="B10" s="77"/>
+      <c r="C10" s="77"/>
+      <c r="D10" s="77"/>
+      <c r="E10" s="77"/>
+      <c r="F10" s="77"/>
+      <c r="G10" s="77"/>
+      <c r="H10" s="77"/>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A11" s="77"/>
+      <c r="B11" s="77"/>
+      <c r="C11" s="77"/>
+      <c r="D11" s="77"/>
+      <c r="E11" s="77"/>
+      <c r="F11" s="77"/>
+      <c r="G11" s="77"/>
+      <c r="H11" s="77"/>
+    </row>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A12" s="77"/>
+      <c r="B12" s="77"/>
+      <c r="C12" s="77"/>
+      <c r="D12" s="77"/>
+      <c r="E12" s="77"/>
+      <c r="F12" s="77"/>
+      <c r="G12" s="77"/>
+      <c r="H12" s="77"/>
+    </row>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A13" s="76"/>
+      <c r="B13" s="77"/>
+      <c r="C13" s="77"/>
+      <c r="D13" s="77"/>
+      <c r="E13" s="77"/>
+      <c r="F13" s="77"/>
+      <c r="G13" s="77"/>
+      <c r="H13" s="77"/>
+    </row>
+    <row r="14" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A14" s="77"/>
+      <c r="B14" s="77"/>
+      <c r="C14" s="77"/>
+      <c r="D14" s="77"/>
+      <c r="E14" s="77"/>
+      <c r="F14" s="77"/>
+      <c r="G14" s="77"/>
+      <c r="H14" s="77"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
   <dimension ref="A1:M31"/>
-  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="8.7265625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="20.140625" customWidth="1"/>
-    <col min="2" max="13" width="12.5703125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="20.1796875" customWidth="1"/>
+    <col min="2" max="13" width="12.54296875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="3" t="s">
         <v>375</v>
       </c>
@@ -10412,33 +10841,33 @@
         <v>387</v>
       </c>
     </row>
-    <row r="2" spans="1:13" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:13" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A2" s="3" t="s">
         <v>8</v>
       </c>
       <c r="B2" t="s">
-        <v>432</v>
+        <v>430</v>
       </c>
       <c r="C2" t="s">
-        <v>432</v>
+        <v>430</v>
       </c>
       <c r="D2" t="s">
-        <v>432</v>
+        <v>430</v>
       </c>
       <c r="E2" t="s">
-        <v>432</v>
+        <v>430</v>
       </c>
       <c r="F2" t="s">
-        <v>431</v>
+        <v>429</v>
       </c>
       <c r="G2" t="s">
-        <v>431</v>
+        <v>429</v>
       </c>
       <c r="H2" t="s">
-        <v>431</v>
+        <v>429</v>
       </c>
       <c r="I2" t="s">
-        <v>431</v>
+        <v>429</v>
       </c>
       <c r="J2" t="s">
         <v>157</v>
@@ -10453,7 +10882,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="3" spans="1:13" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:13" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A3" s="5" t="s">
         <v>389</v>
       </c>
@@ -10494,592 +10923,592 @@
         <v>41</v>
       </c>
     </row>
-    <row r="4" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>390</v>
       </c>
       <c r="B4" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
       <c r="C4" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
       <c r="D4" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
       <c r="E4" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
       <c r="F4" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
       <c r="G4" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
       <c r="H4" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
       <c r="I4" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
       <c r="K4" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
       <c r="L4" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
       <c r="M4" t="s">
-        <v>415</v>
-      </c>
-    </row>
-    <row r="5" spans="1:13" x14ac:dyDescent="0.25">
+        <v>414</v>
+      </c>
+    </row>
+    <row r="5" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>391</v>
       </c>
       <c r="B5" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
       <c r="C5" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
       <c r="D5" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
       <c r="E5" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
       <c r="F5" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
       <c r="G5" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
       <c r="H5" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
       <c r="I5" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
       <c r="K5" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
       <c r="L5" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
       <c r="M5" t="s">
-        <v>415</v>
-      </c>
-    </row>
-    <row r="6" spans="1:13" x14ac:dyDescent="0.25">
+        <v>414</v>
+      </c>
+    </row>
+    <row r="6" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>392</v>
       </c>
       <c r="B6" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
       <c r="C6" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
       <c r="D6" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
       <c r="E6" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
       <c r="F6" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
       <c r="G6" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
       <c r="H6" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
       <c r="I6" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
       <c r="K6" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
       <c r="L6" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
       <c r="M6" t="s">
-        <v>415</v>
-      </c>
-    </row>
-    <row r="7" spans="1:13" x14ac:dyDescent="0.25">
+        <v>414</v>
+      </c>
+    </row>
+    <row r="7" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>393</v>
       </c>
       <c r="B7" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
       <c r="C7" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
       <c r="D7" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
       <c r="E7" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
       <c r="F7" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
       <c r="G7" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
       <c r="H7" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
       <c r="I7" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
       <c r="K7" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
       <c r="L7" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
       <c r="M7" t="s">
-        <v>415</v>
-      </c>
-    </row>
-    <row r="8" spans="1:13" x14ac:dyDescent="0.25">
+        <v>414</v>
+      </c>
+    </row>
+    <row r="8" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>394</v>
       </c>
       <c r="B8" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
       <c r="C8" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
       <c r="D8" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
       <c r="E8" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
       <c r="F8" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
       <c r="G8" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
       <c r="H8" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
       <c r="I8" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
       <c r="K8" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
       <c r="L8" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
       <c r="M8" t="s">
-        <v>415</v>
-      </c>
-    </row>
-    <row r="9" spans="1:13" x14ac:dyDescent="0.25">
+        <v>414</v>
+      </c>
+    </row>
+    <row r="9" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>395</v>
       </c>
       <c r="B9" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
       <c r="C9" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
       <c r="D9" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
       <c r="E9" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
       <c r="F9" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
       <c r="G9" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
       <c r="H9" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
       <c r="I9" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
       <c r="K9" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
       <c r="L9" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
       <c r="M9" t="s">
-        <v>415</v>
-      </c>
-    </row>
-    <row r="10" spans="1:13" x14ac:dyDescent="0.25">
+        <v>414</v>
+      </c>
+    </row>
+    <row r="10" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>396</v>
       </c>
       <c r="B10" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
       <c r="C10" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
       <c r="D10" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
       <c r="E10" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
       <c r="F10" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
       <c r="G10" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
       <c r="H10" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
       <c r="I10" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
       <c r="K10" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
       <c r="L10" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
       <c r="M10" t="s">
-        <v>415</v>
-      </c>
-    </row>
-    <row r="11" spans="1:13" x14ac:dyDescent="0.25">
+        <v>414</v>
+      </c>
+    </row>
+    <row r="11" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>397</v>
       </c>
       <c r="B11" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
       <c r="C11" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
       <c r="D11" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
       <c r="E11" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
       <c r="F11" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
       <c r="G11" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
       <c r="H11" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
       <c r="I11" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
       <c r="K11" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
       <c r="L11" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
       <c r="M11" t="s">
-        <v>415</v>
-      </c>
-    </row>
-    <row r="12" spans="1:13" x14ac:dyDescent="0.25">
+        <v>414</v>
+      </c>
+    </row>
+    <row r="12" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>398</v>
       </c>
       <c r="B12" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
       <c r="C12" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
       <c r="D12" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
       <c r="E12" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
       <c r="F12" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
       <c r="G12" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
       <c r="H12" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
       <c r="I12" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
       <c r="K12" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
       <c r="L12" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
       <c r="M12" t="s">
-        <v>415</v>
-      </c>
-    </row>
-    <row r="13" spans="1:13" x14ac:dyDescent="0.25">
+        <v>414</v>
+      </c>
+    </row>
+    <row r="13" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>399</v>
       </c>
       <c r="B13" t="s">
+        <v>414</v>
+      </c>
+      <c r="C13" t="s">
+        <v>414</v>
+      </c>
+      <c r="D13" t="s">
+        <v>414</v>
+      </c>
+      <c r="E13" t="s">
+        <v>414</v>
+      </c>
+      <c r="F13" t="s">
+        <v>414</v>
+      </c>
+      <c r="G13" t="s">
+        <v>414</v>
+      </c>
+      <c r="H13" t="s">
+        <v>414</v>
+      </c>
+      <c r="I13" t="s">
+        <v>414</v>
+      </c>
+      <c r="K13" t="s">
+        <v>414</v>
+      </c>
+      <c r="L13" t="s">
+        <v>414</v>
+      </c>
+      <c r="M13" t="s">
+        <v>414</v>
+      </c>
+    </row>
+    <row r="14" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A14" t="s">
+        <v>409</v>
+      </c>
+      <c r="B14" t="s">
+        <v>414</v>
+      </c>
+      <c r="C14" t="s">
+        <v>414</v>
+      </c>
+      <c r="D14" t="s">
+        <v>414</v>
+      </c>
+      <c r="E14" t="s">
+        <v>414</v>
+      </c>
+      <c r="F14" t="s">
+        <v>414</v>
+      </c>
+      <c r="G14" t="s">
+        <v>414</v>
+      </c>
+      <c r="H14" t="s">
+        <v>414</v>
+      </c>
+      <c r="I14" t="s">
+        <v>414</v>
+      </c>
+      <c r="K14" t="s">
+        <v>414</v>
+      </c>
+      <c r="L14" t="s">
+        <v>414</v>
+      </c>
+      <c r="M14" t="s">
+        <v>414</v>
+      </c>
+    </row>
+    <row r="15" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A15" t="s">
+        <v>410</v>
+      </c>
+      <c r="B15" t="s">
+        <v>414</v>
+      </c>
+      <c r="C15" t="s">
+        <v>414</v>
+      </c>
+      <c r="D15" t="s">
+        <v>414</v>
+      </c>
+      <c r="E15" t="s">
+        <v>414</v>
+      </c>
+      <c r="F15" t="s">
+        <v>414</v>
+      </c>
+      <c r="G15" t="s">
+        <v>414</v>
+      </c>
+      <c r="H15" t="s">
+        <v>414</v>
+      </c>
+      <c r="I15" t="s">
+        <v>414</v>
+      </c>
+      <c r="K15" t="s">
+        <v>414</v>
+      </c>
+      <c r="L15" t="s">
+        <v>414</v>
+      </c>
+      <c r="M15" t="s">
+        <v>414</v>
+      </c>
+    </row>
+    <row r="16" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A16" t="s">
+        <v>411</v>
+      </c>
+      <c r="B16" t="s">
+        <v>414</v>
+      </c>
+      <c r="C16" t="s">
+        <v>414</v>
+      </c>
+      <c r="D16" t="s">
+        <v>414</v>
+      </c>
+      <c r="E16" t="s">
+        <v>414</v>
+      </c>
+      <c r="F16" t="s">
+        <v>414</v>
+      </c>
+      <c r="G16" t="s">
+        <v>414</v>
+      </c>
+      <c r="H16" t="s">
+        <v>414</v>
+      </c>
+      <c r="I16" t="s">
+        <v>414</v>
+      </c>
+      <c r="K16" t="s">
+        <v>414</v>
+      </c>
+      <c r="L16" t="s">
+        <v>414</v>
+      </c>
+      <c r="M16" t="s">
+        <v>414</v>
+      </c>
+    </row>
+    <row r="17" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A17" t="s">
+        <v>412</v>
+      </c>
+      <c r="B17" t="s">
+        <v>414</v>
+      </c>
+      <c r="C17" t="s">
+        <v>414</v>
+      </c>
+      <c r="D17" t="s">
+        <v>414</v>
+      </c>
+      <c r="E17" t="s">
+        <v>414</v>
+      </c>
+      <c r="F17" t="s">
+        <v>414</v>
+      </c>
+      <c r="G17" t="s">
+        <v>414</v>
+      </c>
+      <c r="H17" t="s">
+        <v>414</v>
+      </c>
+      <c r="I17" t="s">
+        <v>414</v>
+      </c>
+      <c r="K17" t="s">
+        <v>414</v>
+      </c>
+      <c r="L17" t="s">
+        <v>414</v>
+      </c>
+      <c r="M17" t="s">
+        <v>414</v>
+      </c>
+    </row>
+    <row r="18" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A18" t="s">
+        <v>413</v>
+      </c>
+      <c r="B18" t="s">
+        <v>414</v>
+      </c>
+      <c r="C18" t="s">
+        <v>414</v>
+      </c>
+      <c r="D18" t="s">
+        <v>414</v>
+      </c>
+      <c r="E18" t="s">
+        <v>414</v>
+      </c>
+      <c r="F18" t="s">
+        <v>414</v>
+      </c>
+      <c r="G18" t="s">
+        <v>414</v>
+      </c>
+      <c r="H18" t="s">
+        <v>414</v>
+      </c>
+      <c r="I18" t="s">
+        <v>414</v>
+      </c>
+      <c r="K18" t="s">
+        <v>414</v>
+      </c>
+      <c r="L18" t="s">
+        <v>414</v>
+      </c>
+      <c r="M18" t="s">
+        <v>414</v>
+      </c>
+    </row>
+    <row r="20" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A20" t="s">
         <v>415</v>
       </c>
-      <c r="C13" t="s">
-        <v>415</v>
-      </c>
-      <c r="D13" t="s">
-        <v>415</v>
-      </c>
-      <c r="E13" t="s">
-        <v>415</v>
-      </c>
-      <c r="F13" t="s">
-        <v>415</v>
-      </c>
-      <c r="G13" t="s">
-        <v>415</v>
-      </c>
-      <c r="H13" t="s">
-        <v>415</v>
-      </c>
-      <c r="I13" t="s">
-        <v>415</v>
-      </c>
-      <c r="K13" t="s">
-        <v>415</v>
-      </c>
-      <c r="L13" t="s">
-        <v>415</v>
-      </c>
-      <c r="M13" t="s">
-        <v>415</v>
-      </c>
-    </row>
-    <row r="14" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A14" t="s">
-        <v>410</v>
-      </c>
-      <c r="B14" t="s">
-        <v>415</v>
-      </c>
-      <c r="C14" t="s">
-        <v>415</v>
-      </c>
-      <c r="D14" t="s">
-        <v>415</v>
-      </c>
-      <c r="E14" t="s">
-        <v>415</v>
-      </c>
-      <c r="F14" t="s">
-        <v>415</v>
-      </c>
-      <c r="G14" t="s">
-        <v>415</v>
-      </c>
-      <c r="H14" t="s">
-        <v>415</v>
-      </c>
-      <c r="I14" t="s">
-        <v>415</v>
-      </c>
-      <c r="K14" t="s">
-        <v>415</v>
-      </c>
-      <c r="L14" t="s">
-        <v>415</v>
-      </c>
-      <c r="M14" t="s">
-        <v>415</v>
-      </c>
-    </row>
-    <row r="15" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A15" t="s">
-        <v>411</v>
-      </c>
-      <c r="B15" t="s">
-        <v>415</v>
-      </c>
-      <c r="C15" t="s">
-        <v>415</v>
-      </c>
-      <c r="D15" t="s">
-        <v>415</v>
-      </c>
-      <c r="E15" t="s">
-        <v>415</v>
-      </c>
-      <c r="F15" t="s">
-        <v>415</v>
-      </c>
-      <c r="G15" t="s">
-        <v>415</v>
-      </c>
-      <c r="H15" t="s">
-        <v>415</v>
-      </c>
-      <c r="I15" t="s">
-        <v>415</v>
-      </c>
-      <c r="K15" t="s">
-        <v>415</v>
-      </c>
-      <c r="L15" t="s">
-        <v>415</v>
-      </c>
-      <c r="M15" t="s">
-        <v>415</v>
-      </c>
-    </row>
-    <row r="16" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A16" t="s">
-        <v>412</v>
-      </c>
-      <c r="B16" t="s">
-        <v>415</v>
-      </c>
-      <c r="C16" t="s">
-        <v>415</v>
-      </c>
-      <c r="D16" t="s">
-        <v>415</v>
-      </c>
-      <c r="E16" t="s">
-        <v>415</v>
-      </c>
-      <c r="F16" t="s">
-        <v>415</v>
-      </c>
-      <c r="G16" t="s">
-        <v>415</v>
-      </c>
-      <c r="H16" t="s">
-        <v>415</v>
-      </c>
-      <c r="I16" t="s">
-        <v>415</v>
-      </c>
-      <c r="K16" t="s">
-        <v>415</v>
-      </c>
-      <c r="L16" t="s">
-        <v>415</v>
-      </c>
-      <c r="M16" t="s">
-        <v>415</v>
-      </c>
-    </row>
-    <row r="17" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A17" t="s">
-        <v>413</v>
-      </c>
-      <c r="B17" t="s">
-        <v>415</v>
-      </c>
-      <c r="C17" t="s">
-        <v>415</v>
-      </c>
-      <c r="D17" t="s">
-        <v>415</v>
-      </c>
-      <c r="E17" t="s">
-        <v>415</v>
-      </c>
-      <c r="F17" t="s">
-        <v>415</v>
-      </c>
-      <c r="G17" t="s">
-        <v>415</v>
-      </c>
-      <c r="H17" t="s">
-        <v>415</v>
-      </c>
-      <c r="I17" t="s">
-        <v>415</v>
-      </c>
-      <c r="K17" t="s">
-        <v>415</v>
-      </c>
-      <c r="L17" t="s">
-        <v>415</v>
-      </c>
-      <c r="M17" t="s">
-        <v>415</v>
-      </c>
-    </row>
-    <row r="18" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A18" t="s">
-        <v>414</v>
-      </c>
-      <c r="B18" t="s">
-        <v>415</v>
-      </c>
-      <c r="C18" t="s">
-        <v>415</v>
-      </c>
-      <c r="D18" t="s">
-        <v>415</v>
-      </c>
-      <c r="E18" t="s">
-        <v>415</v>
-      </c>
-      <c r="F18" t="s">
-        <v>415</v>
-      </c>
-      <c r="G18" t="s">
-        <v>415</v>
-      </c>
-      <c r="H18" t="s">
-        <v>415</v>
-      </c>
-      <c r="I18" t="s">
-        <v>415</v>
-      </c>
-      <c r="K18" t="s">
-        <v>415</v>
-      </c>
-      <c r="L18" t="s">
-        <v>415</v>
-      </c>
-      <c r="M18" t="s">
-        <v>415</v>
-      </c>
-    </row>
-    <row r="20" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A20" t="s">
-        <v>416</v>
-      </c>
-    </row>
-    <row r="29" spans="1:13" x14ac:dyDescent="0.25">
+    </row>
+    <row r="29" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A29" s="6" t="s">
         <v>400</v>
       </c>
     </row>
-    <row r="30" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A30" s="8" t="s">
         <v>401</v>
       </c>
     </row>
-    <row r="31" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A31" s="9" t="s">
         <v>402</v>
       </c>
@@ -11094,14 +11523,14 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{68654364-EAB1-4DEC-A6E8-9FEA32BD138C}">
-  <dimension ref="A1:M30"/>
-  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:M27"/>
+  <sheetFormatPr defaultColWidth="8.7265625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="20.140625" customWidth="1"/>
-    <col min="2" max="13" width="12.5703125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="20.1796875" customWidth="1"/>
+    <col min="2" max="13" width="12.54296875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:13" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A1" s="3" t="s">
         <v>375</v>
       </c>
@@ -11142,7 +11571,7 @@
         <v>388</v>
       </c>
     </row>
-    <row r="2" spans="1:13" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:13" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A2" s="5" t="s">
         <v>389</v>
       </c>
@@ -11183,105 +11612,644 @@
         <v>41</v>
       </c>
     </row>
-    <row r="3" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>390</v>
       </c>
-    </row>
-    <row r="4" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="B3" s="81" t="s">
+        <v>442</v>
+      </c>
+      <c r="C3" t="s">
+        <v>452</v>
+      </c>
+      <c r="D3" t="s">
+        <v>462</v>
+      </c>
+      <c r="E3" t="s">
+        <v>472</v>
+      </c>
+      <c r="F3" t="s">
+        <v>482</v>
+      </c>
+      <c r="G3" t="s">
+        <v>492</v>
+      </c>
+      <c r="H3" t="s">
+        <v>500</v>
+      </c>
+      <c r="I3" t="s">
+        <v>510</v>
+      </c>
+      <c r="J3" t="s">
+        <v>475</v>
+      </c>
+      <c r="K3" t="s">
+        <v>527</v>
+      </c>
+      <c r="L3" t="s">
+        <v>537</v>
+      </c>
+      <c r="M3" t="s">
+        <v>547</v>
+      </c>
+    </row>
+    <row r="4" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>391</v>
       </c>
-    </row>
-    <row r="5" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="B4" t="s">
+        <v>443</v>
+      </c>
+      <c r="C4" t="s">
+        <v>453</v>
+      </c>
+      <c r="D4" t="s">
+        <v>463</v>
+      </c>
+      <c r="E4" t="s">
+        <v>473</v>
+      </c>
+      <c r="F4" t="s">
+        <v>483</v>
+      </c>
+      <c r="G4" t="s">
+        <v>468</v>
+      </c>
+      <c r="H4" t="s">
+        <v>501</v>
+      </c>
+      <c r="I4" t="s">
+        <v>511</v>
+      </c>
+      <c r="J4" t="s">
+        <v>518</v>
+      </c>
+      <c r="K4" t="s">
+        <v>528</v>
+      </c>
+      <c r="L4" t="s">
+        <v>538</v>
+      </c>
+      <c r="M4" t="s">
+        <v>548</v>
+      </c>
+    </row>
+    <row r="5" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>392</v>
       </c>
-    </row>
-    <row r="6" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="B5" t="s">
+        <v>444</v>
+      </c>
+      <c r="C5" t="s">
+        <v>454</v>
+      </c>
+      <c r="D5" t="s">
+        <v>464</v>
+      </c>
+      <c r="E5" t="s">
+        <v>474</v>
+      </c>
+      <c r="F5" t="s">
+        <v>484</v>
+      </c>
+      <c r="G5" t="s">
+        <v>493</v>
+      </c>
+      <c r="H5" t="s">
+        <v>502</v>
+      </c>
+      <c r="I5" t="s">
+        <v>552</v>
+      </c>
+      <c r="J5" t="s">
+        <v>519</v>
+      </c>
+      <c r="K5" t="s">
+        <v>529</v>
+      </c>
+      <c r="L5" t="s">
+        <v>539</v>
+      </c>
+      <c r="M5" t="s">
+        <v>549</v>
+      </c>
+    </row>
+    <row r="6" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>393</v>
       </c>
-    </row>
-    <row r="7" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="B6" t="s">
+        <v>445</v>
+      </c>
+      <c r="C6" t="s">
+        <v>455</v>
+      </c>
+      <c r="D6" t="s">
+        <v>471</v>
+      </c>
+      <c r="E6" t="s">
+        <v>475</v>
+      </c>
+      <c r="F6" t="s">
+        <v>485</v>
+      </c>
+      <c r="G6" t="s">
+        <v>494</v>
+      </c>
+      <c r="H6" t="s">
+        <v>503</v>
+      </c>
+      <c r="I6" t="s">
+        <v>491</v>
+      </c>
+      <c r="J6" t="s">
+        <v>520</v>
+      </c>
+      <c r="K6" t="s">
+        <v>530</v>
+      </c>
+      <c r="L6" t="s">
+        <v>540</v>
+      </c>
+      <c r="M6" t="s">
+        <v>550</v>
+      </c>
+    </row>
+    <row r="7" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>394</v>
       </c>
-    </row>
-    <row r="8" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="B7" t="s">
+        <v>446</v>
+      </c>
+      <c r="C7" t="s">
+        <v>456</v>
+      </c>
+      <c r="D7" t="s">
+        <v>465</v>
+      </c>
+      <c r="E7" t="s">
+        <v>476</v>
+      </c>
+      <c r="F7" t="s">
+        <v>486</v>
+      </c>
+      <c r="G7" t="s">
+        <v>495</v>
+      </c>
+      <c r="H7" t="s">
+        <v>504</v>
+      </c>
+      <c r="I7" t="s">
+        <v>512</v>
+      </c>
+      <c r="J7" t="s">
+        <v>521</v>
+      </c>
+      <c r="K7" t="s">
+        <v>531</v>
+      </c>
+      <c r="L7" t="s">
+        <v>541</v>
+      </c>
+      <c r="M7" t="s">
+        <v>551</v>
+      </c>
+    </row>
+    <row r="8" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>395</v>
       </c>
       <c r="B8" t="s">
-        <v>430</v>
-      </c>
-    </row>
-    <row r="9" spans="1:13" x14ac:dyDescent="0.25">
+        <v>431</v>
+      </c>
+      <c r="C8" t="s">
+        <v>431</v>
+      </c>
+      <c r="D8" t="s">
+        <v>431</v>
+      </c>
+      <c r="E8" t="s">
+        <v>431</v>
+      </c>
+      <c r="F8" s="79" t="s">
+        <v>431</v>
+      </c>
+      <c r="G8" t="s">
+        <v>431</v>
+      </c>
+      <c r="H8" t="s">
+        <v>431</v>
+      </c>
+      <c r="I8" t="s">
+        <v>432</v>
+      </c>
+      <c r="J8" t="s">
+        <v>431</v>
+      </c>
+      <c r="K8" t="s">
+        <v>431</v>
+      </c>
+      <c r="L8" t="s">
+        <v>432</v>
+      </c>
+      <c r="M8" t="s">
+        <v>432</v>
+      </c>
+    </row>
+    <row r="9" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>396</v>
       </c>
       <c r="B9" t="s">
-        <v>436</v>
-      </c>
-    </row>
-    <row r="10" spans="1:13" x14ac:dyDescent="0.25">
+        <v>431</v>
+      </c>
+      <c r="C9" t="s">
+        <v>432</v>
+      </c>
+      <c r="D9" t="s">
+        <v>431</v>
+      </c>
+      <c r="E9" t="s">
+        <v>432</v>
+      </c>
+      <c r="F9" s="79" t="s">
+        <v>432</v>
+      </c>
+      <c r="G9" t="s">
+        <v>431</v>
+      </c>
+      <c r="H9" t="s">
+        <v>431</v>
+      </c>
+      <c r="I9" t="s">
+        <v>432</v>
+      </c>
+      <c r="J9" t="s">
+        <v>431</v>
+      </c>
+      <c r="K9" t="s">
+        <v>431</v>
+      </c>
+      <c r="L9" t="s">
+        <v>432</v>
+      </c>
+      <c r="M9" t="s">
+        <v>432</v>
+      </c>
+    </row>
+    <row r="10" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>397</v>
       </c>
-    </row>
-    <row r="11" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="B10" t="s">
+        <v>431</v>
+      </c>
+      <c r="C10" t="s">
+        <v>431</v>
+      </c>
+      <c r="D10" t="s">
+        <v>431</v>
+      </c>
+      <c r="E10" t="s">
+        <v>431</v>
+      </c>
+      <c r="F10" t="s">
+        <v>432</v>
+      </c>
+      <c r="G10" t="s">
+        <v>431</v>
+      </c>
+      <c r="H10" t="s">
+        <v>431</v>
+      </c>
+      <c r="I10" t="s">
+        <v>432</v>
+      </c>
+      <c r="J10" t="s">
+        <v>431</v>
+      </c>
+      <c r="K10" t="s">
+        <v>431</v>
+      </c>
+      <c r="L10" t="s">
+        <v>432</v>
+      </c>
+      <c r="M10" t="s">
+        <v>432</v>
+      </c>
+    </row>
+    <row r="11" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>398</v>
       </c>
-    </row>
-    <row r="12" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="B11" t="s">
+        <v>431</v>
+      </c>
+      <c r="C11" t="s">
+        <v>431</v>
+      </c>
+      <c r="D11" t="s">
+        <v>431</v>
+      </c>
+      <c r="E11" t="s">
+        <v>432</v>
+      </c>
+      <c r="F11" t="s">
+        <v>431</v>
+      </c>
+      <c r="G11" t="s">
+        <v>431</v>
+      </c>
+      <c r="H11" t="s">
+        <v>432</v>
+      </c>
+      <c r="I11" t="s">
+        <v>432</v>
+      </c>
+      <c r="J11" t="s">
+        <v>432</v>
+      </c>
+      <c r="K11" t="s">
+        <v>431</v>
+      </c>
+      <c r="L11" t="s">
+        <v>432</v>
+      </c>
+      <c r="M11" t="s">
+        <v>432</v>
+      </c>
+    </row>
+    <row r="12" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>399</v>
       </c>
-    </row>
-    <row r="13" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="B12" t="s">
+        <v>431</v>
+      </c>
+      <c r="C12" t="s">
+        <v>431</v>
+      </c>
+      <c r="D12" t="s">
+        <v>431</v>
+      </c>
+      <c r="E12" t="s">
+        <v>431</v>
+      </c>
+      <c r="F12" t="s">
+        <v>431</v>
+      </c>
+      <c r="G12" t="s">
+        <v>431</v>
+      </c>
+      <c r="H12" t="s">
+        <v>431</v>
+      </c>
+      <c r="I12" t="s">
+        <v>432</v>
+      </c>
+      <c r="J12" t="s">
+        <v>431</v>
+      </c>
+      <c r="K12" t="s">
+        <v>431</v>
+      </c>
+      <c r="L12" t="s">
+        <v>432</v>
+      </c>
+      <c r="M12" t="s">
+        <v>432</v>
+      </c>
+    </row>
+    <row r="13" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
+        <v>409</v>
+      </c>
+      <c r="B13" t="s">
+        <v>437</v>
+      </c>
+      <c r="C13" t="s">
+        <v>447</v>
+      </c>
+      <c r="D13" t="s">
+        <v>457</v>
+      </c>
+      <c r="E13" t="s">
+        <v>466</v>
+      </c>
+      <c r="F13" t="s">
+        <v>477</v>
+      </c>
+      <c r="G13" t="s">
+        <v>487</v>
+      </c>
+      <c r="H13" t="s">
+        <v>496</v>
+      </c>
+      <c r="I13" t="s">
+        <v>505</v>
+      </c>
+      <c r="J13" t="s">
+        <v>513</v>
+      </c>
+      <c r="K13" t="s">
+        <v>522</v>
+      </c>
+      <c r="L13" t="s">
+        <v>532</v>
+      </c>
+      <c r="M13" t="s">
+        <v>542</v>
+      </c>
+    </row>
+    <row r="14" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A14" t="s">
         <v>410</v>
       </c>
-    </row>
-    <row r="14" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A14" t="s">
+      <c r="B14" t="s">
+        <v>438</v>
+      </c>
+      <c r="C14" t="s">
+        <v>448</v>
+      </c>
+      <c r="D14" t="s">
+        <v>458</v>
+      </c>
+      <c r="E14" t="s">
+        <v>467</v>
+      </c>
+      <c r="F14" t="s">
+        <v>478</v>
+      </c>
+      <c r="G14" t="s">
+        <v>488</v>
+      </c>
+      <c r="H14" t="s">
+        <v>497</v>
+      </c>
+      <c r="I14" t="s">
+        <v>506</v>
+      </c>
+      <c r="J14" t="s">
+        <v>514</v>
+      </c>
+      <c r="K14" t="s">
+        <v>524</v>
+      </c>
+      <c r="L14" t="s">
+        <v>533</v>
+      </c>
+      <c r="M14" t="s">
+        <v>543</v>
+      </c>
+    </row>
+    <row r="15" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A15" t="s">
         <v>411</v>
       </c>
-    </row>
-    <row r="15" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A15" t="s">
+      <c r="B15" t="s">
+        <v>439</v>
+      </c>
+      <c r="C15" t="s">
+        <v>449</v>
+      </c>
+      <c r="D15" t="s">
+        <v>459</v>
+      </c>
+      <c r="E15" t="s">
+        <v>468</v>
+      </c>
+      <c r="F15" t="s">
+        <v>479</v>
+      </c>
+      <c r="G15" t="s">
+        <v>489</v>
+      </c>
+      <c r="H15" t="s">
+        <v>481</v>
+      </c>
+      <c r="I15" t="s">
+        <v>507</v>
+      </c>
+      <c r="J15" t="s">
+        <v>515</v>
+      </c>
+      <c r="K15" t="s">
+        <v>523</v>
+      </c>
+      <c r="L15" t="s">
+        <v>534</v>
+      </c>
+      <c r="M15" t="s">
+        <v>544</v>
+      </c>
+    </row>
+    <row r="16" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A16" t="s">
         <v>412</v>
       </c>
-    </row>
-    <row r="16" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A16" t="s">
+      <c r="B16" t="s">
+        <v>440</v>
+      </c>
+      <c r="C16" t="s">
+        <v>450</v>
+      </c>
+      <c r="D16" t="s">
+        <v>460</v>
+      </c>
+      <c r="E16" t="s">
+        <v>469</v>
+      </c>
+      <c r="F16" t="s">
+        <v>480</v>
+      </c>
+      <c r="G16" t="s">
+        <v>490</v>
+      </c>
+      <c r="H16" t="s">
+        <v>498</v>
+      </c>
+      <c r="I16" t="s">
+        <v>508</v>
+      </c>
+      <c r="J16" t="s">
+        <v>516</v>
+      </c>
+      <c r="K16" t="s">
+        <v>525</v>
+      </c>
+      <c r="L16" t="s">
+        <v>535</v>
+      </c>
+      <c r="M16" t="s">
+        <v>545</v>
+      </c>
+    </row>
+    <row r="17" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A17" t="s">
         <v>413</v>
       </c>
-    </row>
-    <row r="17" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A17" t="s">
-        <v>414</v>
-      </c>
-    </row>
-    <row r="19" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B17" t="s">
+        <v>441</v>
+      </c>
+      <c r="C17" t="s">
+        <v>451</v>
+      </c>
+      <c r="D17" t="s">
+        <v>461</v>
+      </c>
+      <c r="E17" t="s">
+        <v>470</v>
+      </c>
+      <c r="F17" t="s">
+        <v>481</v>
+      </c>
+      <c r="G17" t="s">
+        <v>491</v>
+      </c>
+      <c r="H17" t="s">
+        <v>499</v>
+      </c>
+      <c r="I17" t="s">
+        <v>509</v>
+      </c>
+      <c r="J17" t="s">
+        <v>517</v>
+      </c>
+      <c r="K17" t="s">
+        <v>526</v>
+      </c>
+      <c r="L17" t="s">
+        <v>536</v>
+      </c>
+      <c r="M17" t="s">
+        <v>546</v>
+      </c>
+    </row>
+    <row r="19" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
-        <v>416</v>
-      </c>
-    </row>
-    <row r="28" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A28" s="6" t="s">
-        <v>400</v>
-      </c>
-    </row>
-    <row r="29" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A29" s="8" t="s">
-        <v>401</v>
-      </c>
-    </row>
-    <row r="30" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A30" s="9" t="s">
-        <v>402</v>
+        <v>415</v>
+      </c>
+    </row>
+    <row r="22" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A22" t="s">
+        <v>433</v>
+      </c>
+    </row>
+    <row r="23" spans="1:13" ht="29" x14ac:dyDescent="0.35">
+      <c r="A23" s="80" t="s">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="25" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A25" t="s">
+        <v>436</v>
+      </c>
+    </row>
+    <row r="27" spans="1:13" ht="29" x14ac:dyDescent="0.35">
+      <c r="A27" s="78" t="s">
+        <v>434</v>
       </c>
     </row>
   </sheetData>
@@ -11295,12 +12263,12 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:O23"/>
-  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="8.7265625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="15" width="14.28515625" customWidth="1"/>
+    <col min="1" max="15" width="14.26953125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" s="13" customFormat="1" ht="57" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:15" s="13" customFormat="1" ht="57" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="13" t="s">
         <v>0</v>
       </c>
@@ -11347,7 +12315,7 @@
         <v>234</v>
       </c>
     </row>
-    <row r="2" spans="1:15" s="13" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:15" s="13" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A2" s="18" t="s">
         <v>204</v>
       </c>
@@ -11394,7 +12362,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A3" s="19" t="s">
         <v>206</v>
       </c>
@@ -11441,7 +12409,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A4" s="19" t="s">
         <v>209</v>
       </c>
@@ -11488,7 +12456,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A5" s="19" t="s">
         <v>200</v>
       </c>
@@ -11535,7 +12503,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A6" s="19" t="s">
         <v>197</v>
       </c>
@@ -11582,7 +12550,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A7" s="19" t="s">
         <v>194</v>
       </c>
@@ -11629,7 +12597,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="8" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A8" s="19" t="s">
         <v>190</v>
       </c>
@@ -11676,7 +12644,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="9" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A9" s="19" t="s">
         <v>187</v>
       </c>
@@ -11723,7 +12691,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="10" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A10" s="19" t="s">
         <v>177</v>
       </c>
@@ -11770,7 +12738,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="11" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A11" s="19" t="s">
         <v>174</v>
       </c>
@@ -11817,7 +12785,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="12" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A12" s="19" t="s">
         <v>169</v>
       </c>
@@ -11864,7 +12832,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="13" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A13" s="19" t="s">
         <v>162</v>
       </c>
@@ -11911,7 +12879,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="14" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A14" s="19" t="s">
         <v>156</v>
       </c>
@@ -11958,7 +12926,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="15" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A15" s="19" t="s">
         <v>212</v>
       </c>
@@ -12005,7 +12973,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="16" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A16" s="19" t="s">
         <v>215</v>
       </c>
@@ -12052,31 +13020,31 @@
         <v>1</v>
       </c>
     </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A17" s="19"/>
       <c r="F17" s="22"/>
     </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A18" s="19"/>
       <c r="F18" s="22"/>
     </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A19" s="19"/>
       <c r="F19" s="22"/>
     </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A20" s="19"/>
       <c r="F20" s="22"/>
     </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A21" s="19"/>
       <c r="F21" s="22"/>
     </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A22" s="19"/>
       <c r="F22" s="22"/>
     </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A23" s="19"/>
     </row>
   </sheetData>
@@ -12090,20 +13058,20 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:AJ23"/>
-  <sheetFormatPr defaultColWidth="14.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="14.453125" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="16" width="25.42578125" style="11" customWidth="1"/>
-    <col min="17" max="17" width="25.42578125" style="14" customWidth="1"/>
-    <col min="18" max="22" width="25.42578125" style="11" customWidth="1"/>
-    <col min="23" max="23" width="25.42578125" style="14" customWidth="1"/>
-    <col min="24" max="26" width="25.42578125" style="11" customWidth="1"/>
-    <col min="27" max="27" width="25.42578125" style="14" customWidth="1"/>
-    <col min="28" max="34" width="25.42578125" style="11" customWidth="1"/>
-    <col min="35" max="35" width="14.42578125" style="11" customWidth="1"/>
-    <col min="36" max="16384" width="14.42578125" style="11"/>
+    <col min="1" max="16" width="25.453125" style="11" customWidth="1"/>
+    <col min="17" max="17" width="25.453125" style="14" customWidth="1"/>
+    <col min="18" max="22" width="25.453125" style="11" customWidth="1"/>
+    <col min="23" max="23" width="25.453125" style="14" customWidth="1"/>
+    <col min="24" max="26" width="25.453125" style="11" customWidth="1"/>
+    <col min="27" max="27" width="25.453125" style="14" customWidth="1"/>
+    <col min="28" max="34" width="25.453125" style="11" customWidth="1"/>
+    <col min="35" max="35" width="14.453125" style="11" customWidth="1"/>
+    <col min="36" max="16384" width="14.453125" style="11"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:36" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:36" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B1" s="12" t="s">
         <v>235</v>
       </c>
@@ -12117,7 +13085,7 @@
         <v>238</v>
       </c>
     </row>
-    <row r="2" spans="1:36" s="13" customFormat="1" ht="90" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:36" s="13" customFormat="1" ht="90" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A2" s="13" t="s">
         <v>0</v>
       </c>
@@ -12227,7 +13195,7 @@
         <v>273</v>
       </c>
     </row>
-    <row r="3" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A3" s="44" t="s">
         <v>156</v>
       </c>
@@ -12339,7 +13307,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="4" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A4" s="44" t="s">
         <v>162</v>
       </c>
@@ -12448,7 +13416,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="5" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A5" s="44" t="s">
         <v>169</v>
       </c>
@@ -12554,7 +13522,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="6" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A6" s="46" t="s">
         <v>174</v>
       </c>
@@ -12663,7 +13631,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="7" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A7" s="46" t="s">
         <v>177</v>
       </c>
@@ -12764,7 +13732,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="8" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A8" s="48" t="s">
         <v>181</v>
       </c>
@@ -12772,7 +13740,7 @@
       <c r="W8" s="11"/>
       <c r="AA8" s="11"/>
     </row>
-    <row r="9" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A9" s="11" t="s">
         <v>187</v>
       </c>
@@ -12870,7 +13838,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="10" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A10" s="11" t="s">
         <v>194</v>
       </c>
@@ -12982,7 +13950,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="11" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A11" s="45" t="s">
         <v>197</v>
       </c>
@@ -13094,7 +14062,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="12" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A12" s="19" t="s">
         <v>200</v>
       </c>
@@ -13200,7 +14168,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="13" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A13" s="45" t="s">
         <v>204</v>
       </c>
@@ -13312,7 +14280,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="14" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A14" s="19" t="s">
         <v>206</v>
       </c>
@@ -13418,7 +14386,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="15" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A15" s="45" t="s">
         <v>209</v>
       </c>
@@ -13524,7 +14492,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="16" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A16" s="19" t="s">
         <v>212</v>
       </c>
@@ -13636,7 +14604,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="17" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:36" x14ac:dyDescent="0.35">
       <c r="A17" s="45" t="s">
         <v>215</v>
       </c>
@@ -13744,7 +14712,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="19" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:36" x14ac:dyDescent="0.35">
       <c r="AH19" s="11" t="s">
         <v>274</v>
       </c>
@@ -13757,7 +14725,7 @@
         <v>31.5</v>
       </c>
     </row>
-    <row r="20" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:36" x14ac:dyDescent="0.35">
       <c r="AH20" s="11" t="s">
         <v>275</v>
       </c>
@@ -13770,7 +14738,7 @@
         <v>1.5566235649883124</v>
       </c>
     </row>
-    <row r="21" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:36" x14ac:dyDescent="0.35">
       <c r="AH21" s="11" t="s">
         <v>276</v>
       </c>
@@ -13783,7 +14751,7 @@
         <v>31.5</v>
       </c>
     </row>
-    <row r="22" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:36" x14ac:dyDescent="0.35">
       <c r="AH22" s="11" t="s">
         <v>277</v>
       </c>
@@ -13796,7 +14764,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="23" spans="1:36" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:36" x14ac:dyDescent="0.35">
       <c r="AH23" s="11" t="s">
         <v>278</v>
       </c>
@@ -13821,24 +14789,24 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A1:AR24"/>
-  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="8.7265625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="21.28515625" style="19" customWidth="1"/>
-    <col min="2" max="8" width="14.140625" customWidth="1"/>
-    <col min="9" max="9" width="14.140625" style="17" customWidth="1"/>
-    <col min="10" max="19" width="14.140625" customWidth="1"/>
-    <col min="20" max="20" width="14.140625" style="17" customWidth="1"/>
-    <col min="21" max="25" width="14.140625" customWidth="1"/>
-    <col min="26" max="26" width="14.140625" style="17" customWidth="1"/>
-    <col min="27" max="34" width="14.140625" customWidth="1"/>
-    <col min="35" max="35" width="14.140625" style="17" customWidth="1"/>
-    <col min="36" max="37" width="14.140625" customWidth="1"/>
-    <col min="38" max="38" width="14.140625" style="17" customWidth="1"/>
-    <col min="39" max="43" width="14.140625" customWidth="1"/>
-    <col min="44" max="51" width="15.85546875" customWidth="1"/>
+    <col min="1" max="1" width="21.26953125" style="19" customWidth="1"/>
+    <col min="2" max="8" width="14.1796875" customWidth="1"/>
+    <col min="9" max="9" width="14.1796875" style="17" customWidth="1"/>
+    <col min="10" max="19" width="14.1796875" customWidth="1"/>
+    <col min="20" max="20" width="14.1796875" style="17" customWidth="1"/>
+    <col min="21" max="25" width="14.1796875" customWidth="1"/>
+    <col min="26" max="26" width="14.1796875" style="17" customWidth="1"/>
+    <col min="27" max="34" width="14.1796875" customWidth="1"/>
+    <col min="35" max="35" width="14.1796875" style="17" customWidth="1"/>
+    <col min="36" max="37" width="14.1796875" customWidth="1"/>
+    <col min="38" max="38" width="14.1796875" style="17" customWidth="1"/>
+    <col min="39" max="43" width="14.1796875" customWidth="1"/>
+    <col min="44" max="51" width="15.81640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:44" s="13" customFormat="1" ht="180" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:44" s="13" customFormat="1" ht="180" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="18" t="s">
         <v>279</v>
       </c>
@@ -13972,7 +14940,7 @@
         <v>322</v>
       </c>
     </row>
-    <row r="2" spans="1:44" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:44" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>323</v>
       </c>
@@ -14112,7 +15080,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:44" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:44" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>324</v>
       </c>
@@ -14252,7 +15220,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="4" spans="1:44" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:44" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>325</v>
       </c>
@@ -14392,7 +15360,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="5" spans="1:44" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:44" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>326</v>
       </c>
@@ -14532,7 +15500,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="6" spans="1:44" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:44" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>327</v>
       </c>
@@ -14672,7 +15640,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="7" spans="1:44" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:44" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>328</v>
       </c>
@@ -14812,7 +15780,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="8" spans="1:44" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:44" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>329</v>
       </c>
@@ -14952,7 +15920,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="9" spans="1:44" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:44" x14ac:dyDescent="0.35">
       <c r="A9" s="19" t="s">
         <v>330</v>
       </c>
@@ -15092,7 +16060,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="10" spans="1:44" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:44" x14ac:dyDescent="0.35">
       <c r="A10" s="19" t="s">
         <v>331</v>
       </c>
@@ -15232,7 +16200,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="11" spans="1:44" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:44" x14ac:dyDescent="0.35">
       <c r="A11" s="19" t="s">
         <v>332</v>
       </c>
@@ -15372,7 +16340,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="12" spans="1:44" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:44" x14ac:dyDescent="0.35">
       <c r="A12" s="19" t="s">
         <v>333</v>
       </c>
@@ -15512,7 +16480,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="13" spans="1:44" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:44" x14ac:dyDescent="0.35">
       <c r="A13" s="19" t="s">
         <v>334</v>
       </c>
@@ -15652,7 +16620,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="14" spans="1:44" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:44" x14ac:dyDescent="0.35">
       <c r="A14" s="19" t="s">
         <v>335</v>
       </c>
@@ -15792,7 +16760,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="15" spans="1:44" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:44" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>336</v>
       </c>
@@ -15929,7 +16897,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="16" spans="1:44" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:44" x14ac:dyDescent="0.35">
       <c r="A16" s="1" t="s">
         <v>337</v>
       </c>
@@ -16069,7 +17037,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="17" spans="1:44" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:44" x14ac:dyDescent="0.35">
       <c r="I17" s="49"/>
       <c r="T17" s="49"/>
       <c r="Z17" s="49"/>
@@ -16077,7 +17045,7 @@
       <c r="AL17" s="49"/>
       <c r="AR17" s="49"/>
     </row>
-    <row r="18" spans="1:44" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:44" x14ac:dyDescent="0.35">
       <c r="I18" s="51"/>
       <c r="T18" s="51"/>
       <c r="Z18" s="51"/>
@@ -16085,7 +17053,7 @@
       <c r="AL18" s="51"/>
       <c r="AR18" s="51"/>
     </row>
-    <row r="19" spans="1:44" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:44" x14ac:dyDescent="0.35">
       <c r="A19" s="19" t="s">
         <v>338</v>
       </c>
@@ -16262,7 +17230,7 @@
         <v>47.666666666666664</v>
       </c>
     </row>
-    <row r="20" spans="1:44" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:44" x14ac:dyDescent="0.35">
       <c r="A20" s="19" t="s">
         <v>339</v>
       </c>
@@ -16439,7 +17407,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="21" spans="1:44" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:44" x14ac:dyDescent="0.35">
       <c r="A21" s="19" t="s">
         <v>340</v>
       </c>
@@ -16598,7 +17566,7 @@
       </c>
       <c r="AR21" s="51"/>
     </row>
-    <row r="22" spans="1:44" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:44" x14ac:dyDescent="0.35">
       <c r="A22" s="19" t="s">
         <v>275</v>
       </c>
@@ -16775,7 +17743,7 @@
         <v>20.254335220838414</v>
       </c>
     </row>
-    <row r="23" spans="1:44" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:44" x14ac:dyDescent="0.35">
       <c r="A23" s="19" t="s">
         <v>341</v>
       </c>
@@ -16952,7 +17920,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="24" spans="1:44" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:44" x14ac:dyDescent="0.35">
       <c r="A24" s="19" t="s">
         <v>278</v>
       </c>
@@ -17142,14 +18110,14 @@
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
   <dimension ref="A1:AG80"/>
-  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="8.7265625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="10" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="9.453125" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="10" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:33" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -17250,13 +18218,13 @@
         <v>372</v>
       </c>
     </row>
-    <row r="2" spans="1:33" hidden="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:33" hidden="1" x14ac:dyDescent="0.35">
       <c r="A2" s="11" t="s">
         <v>34</v>
       </c>
       <c r="B2" s="11"/>
     </row>
-    <row r="3" spans="1:33" hidden="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:33" hidden="1" x14ac:dyDescent="0.35">
       <c r="A3" s="26" t="s">
         <v>40</v>
       </c>
@@ -17264,7 +18232,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="4" spans="1:33" hidden="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:33" hidden="1" x14ac:dyDescent="0.35">
       <c r="A4" s="26" t="s">
         <v>47</v>
       </c>
@@ -17272,7 +18240,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="5" spans="1:33" hidden="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:33" hidden="1" x14ac:dyDescent="0.35">
       <c r="A5" s="26" t="s">
         <v>49</v>
       </c>
@@ -17280,7 +18248,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="6" spans="1:33" hidden="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:33" hidden="1" x14ac:dyDescent="0.35">
       <c r="A6" s="26" t="s">
         <v>51</v>
       </c>
@@ -17288,7 +18256,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="7" spans="1:33" hidden="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:33" hidden="1" x14ac:dyDescent="0.35">
       <c r="A7" s="26" t="s">
         <v>53</v>
       </c>
@@ -17296,7 +18264,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="8" spans="1:33" hidden="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:33" hidden="1" x14ac:dyDescent="0.35">
       <c r="A8" s="26" t="s">
         <v>55</v>
       </c>
@@ -17304,7 +18272,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="9" spans="1:33" hidden="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:33" hidden="1" x14ac:dyDescent="0.35">
       <c r="A9" s="27" t="s">
         <v>58</v>
       </c>
@@ -17312,7 +18280,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="10" spans="1:33" hidden="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:33" hidden="1" x14ac:dyDescent="0.35">
       <c r="A10" s="26" t="s">
         <v>59</v>
       </c>
@@ -17320,7 +18288,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="11" spans="1:33" hidden="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:33" hidden="1" x14ac:dyDescent="0.35">
       <c r="A11" s="27" t="s">
         <v>62</v>
       </c>
@@ -17328,7 +18296,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="12" spans="1:33" hidden="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:33" hidden="1" x14ac:dyDescent="0.35">
       <c r="A12" s="27" t="s">
         <v>64</v>
       </c>
@@ -17336,7 +18304,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="13" spans="1:33" hidden="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:33" hidden="1" x14ac:dyDescent="0.35">
       <c r="A13" s="26" t="s">
         <v>65</v>
       </c>
@@ -17344,7 +18312,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="14" spans="1:33" hidden="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:33" hidden="1" x14ac:dyDescent="0.35">
       <c r="A14" s="26" t="s">
         <v>67</v>
       </c>
@@ -17352,7 +18320,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="15" spans="1:33" hidden="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:33" hidden="1" x14ac:dyDescent="0.35">
       <c r="A15" s="26" t="s">
         <v>69</v>
       </c>
@@ -17360,7 +18328,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="16" spans="1:33" hidden="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:33" hidden="1" x14ac:dyDescent="0.35">
       <c r="A16" s="27" t="s">
         <v>71</v>
       </c>
@@ -17368,7 +18336,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="17" spans="1:2" hidden="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A17" s="26" t="s">
         <v>73</v>
       </c>
@@ -17376,7 +18344,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="18" spans="1:2" hidden="1" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A18" s="26" t="s">
         <v>75</v>
       </c>
@@ -17384,7 +18352,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="19" spans="1:2" hidden="1" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A19" s="26" t="s">
         <v>78</v>
       </c>
@@ -17392,7 +18360,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="20" spans="1:2" hidden="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A20" s="40" t="s">
         <v>81</v>
       </c>
@@ -17400,7 +18368,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="21" spans="1:2" hidden="1" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A21" s="31" t="s">
         <v>85</v>
       </c>
@@ -17408,7 +18376,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="22" spans="1:2" hidden="1" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A22" s="31" t="s">
         <v>87</v>
       </c>
@@ -17416,7 +18384,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="23" spans="1:2" hidden="1" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A23" s="41" t="s">
         <v>89</v>
       </c>
@@ -17424,7 +18392,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="24" spans="1:2" hidden="1" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A24" s="31" t="s">
         <v>91</v>
       </c>
@@ -17432,7 +18400,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="25" spans="1:2" hidden="1" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A25" s="31" t="s">
         <v>94</v>
       </c>
@@ -17440,7 +18408,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="26" spans="1:2" hidden="1" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A26" s="31" t="s">
         <v>96</v>
       </c>
@@ -17448,7 +18416,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="27" spans="1:2" hidden="1" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A27" s="39" t="s">
         <v>98</v>
       </c>
@@ -17456,7 +18424,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="28" spans="1:2" hidden="1" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A28" s="31" t="s">
         <v>100</v>
       </c>
@@ -17464,7 +18432,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="29" spans="1:2" hidden="1" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A29" s="31" t="s">
         <v>102</v>
       </c>
@@ -17472,7 +18440,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="30" spans="1:2" hidden="1" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A30" s="31" t="s">
         <v>104</v>
       </c>
@@ -17480,7 +18448,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="31" spans="1:2" hidden="1" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A31" s="31" t="s">
         <v>107</v>
       </c>
@@ -17488,7 +18456,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="32" spans="1:2" hidden="1" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A32" s="32" t="s">
         <v>109</v>
       </c>
@@ -17496,7 +18464,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="33" spans="1:2" hidden="1" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A33" s="31" t="s">
         <v>112</v>
       </c>
@@ -17504,7 +18472,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="34" spans="1:2" hidden="1" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A34" s="31" t="s">
         <v>116</v>
       </c>
@@ -17512,7 +18480,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="35" spans="1:2" hidden="1" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A35" s="31" t="s">
         <v>119</v>
       </c>
@@ -17520,7 +18488,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="36" spans="1:2" hidden="1" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A36" s="31" t="s">
         <v>122</v>
       </c>
@@ -17528,7 +18496,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="37" spans="1:2" hidden="1" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A37" s="31" t="s">
         <v>125</v>
       </c>
@@ -17536,7 +18504,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="38" spans="1:2" hidden="1" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A38" s="31" t="s">
         <v>127</v>
       </c>
@@ -17544,7 +18512,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="39" spans="1:2" hidden="1" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A39" s="31" t="s">
         <v>129</v>
       </c>
@@ -17552,7 +18520,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="40" spans="1:2" hidden="1" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A40" s="31" t="s">
         <v>131</v>
       </c>
@@ -17560,7 +18528,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="41" spans="1:2" hidden="1" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A41" s="31" t="s">
         <v>134</v>
       </c>
@@ -17568,7 +18536,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="42" spans="1:2" hidden="1" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A42" s="32" t="s">
         <v>136</v>
       </c>
@@ -17576,7 +18544,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="43" spans="1:2" hidden="1" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A43" s="31" t="s">
         <v>137</v>
       </c>
@@ -17584,7 +18552,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="44" spans="1:2" hidden="1" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A44" s="31" t="s">
         <v>140</v>
       </c>
@@ -17592,7 +18560,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="45" spans="1:2" hidden="1" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A45" s="31" t="s">
         <v>143</v>
       </c>
@@ -17600,7 +18568,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="46" spans="1:2" hidden="1" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A46" s="31" t="s">
         <v>145</v>
       </c>
@@ -17608,7 +18576,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="47" spans="1:2" hidden="1" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A47" s="31" t="s">
         <v>147</v>
       </c>
@@ -17616,7 +18584,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="48" spans="1:2" hidden="1" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A48" s="31" t="s">
         <v>150</v>
       </c>
@@ -17624,7 +18592,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="49" spans="1:33" hidden="1" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:33" hidden="1" x14ac:dyDescent="0.35">
       <c r="A49" s="31" t="s">
         <v>152</v>
       </c>
@@ -17632,7 +18600,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="50" spans="1:33" hidden="1" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:33" hidden="1" x14ac:dyDescent="0.35">
       <c r="A50" s="31" t="s">
         <v>153</v>
       </c>
@@ -17640,7 +18608,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="51" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:33" x14ac:dyDescent="0.35">
       <c r="A51" s="26" t="s">
         <v>156</v>
       </c>
@@ -17738,7 +18706,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="52" spans="1:33" hidden="1" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:33" hidden="1" x14ac:dyDescent="0.35">
       <c r="A52" s="31" t="s">
         <v>159</v>
       </c>
@@ -17746,7 +18714,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="53" spans="1:33" hidden="1" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:33" hidden="1" x14ac:dyDescent="0.35">
       <c r="A53" s="31" t="s">
         <v>160</v>
       </c>
@@ -17754,7 +18722,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="54" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:33" x14ac:dyDescent="0.35">
       <c r="A54" s="26" t="s">
         <v>162</v>
       </c>
@@ -17852,7 +18820,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="55" spans="1:33" hidden="1" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:33" hidden="1" x14ac:dyDescent="0.35">
       <c r="A55" s="31" t="s">
         <v>165</v>
       </c>
@@ -17860,7 +18828,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="56" spans="1:33" hidden="1" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:33" hidden="1" x14ac:dyDescent="0.35">
       <c r="A56" s="31" t="s">
         <v>168</v>
       </c>
@@ -17952,7 +18920,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="57" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:33" x14ac:dyDescent="0.35">
       <c r="A57" s="26" t="s">
         <v>169</v>
       </c>
@@ -18050,7 +19018,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="58" spans="1:33" hidden="1" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:33" hidden="1" x14ac:dyDescent="0.35">
       <c r="A58" s="31" t="s">
         <v>172</v>
       </c>
@@ -18058,7 +19026,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="59" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:33" x14ac:dyDescent="0.35">
       <c r="A59" s="47" t="s">
         <v>174</v>
       </c>
@@ -18156,7 +19124,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="60" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:33" x14ac:dyDescent="0.35">
       <c r="A60" s="26" t="s">
         <v>177</v>
       </c>
@@ -18254,7 +19222,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="61" spans="1:33" hidden="1" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:33" hidden="1" x14ac:dyDescent="0.35">
       <c r="A61" s="31" t="s">
         <v>180</v>
       </c>
@@ -18352,7 +19320,7 @@
         <v>0.5</v>
       </c>
     </row>
-    <row r="62" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:33" x14ac:dyDescent="0.35">
       <c r="A62" s="47" t="s">
         <v>181</v>
       </c>
@@ -18450,7 +19418,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="63" spans="1:33" hidden="1" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:33" hidden="1" x14ac:dyDescent="0.35">
       <c r="A63" s="31" t="s">
         <v>184</v>
       </c>
@@ -18458,7 +19426,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="64" spans="1:33" hidden="1" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:33" hidden="1" x14ac:dyDescent="0.35">
       <c r="A64" s="32" t="s">
         <v>185</v>
       </c>
@@ -18466,7 +19434,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="65" spans="1:33" hidden="1" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:33" hidden="1" x14ac:dyDescent="0.35">
       <c r="A65" s="31" t="s">
         <v>186</v>
       </c>
@@ -18474,7 +19442,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="66" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:33" x14ac:dyDescent="0.35">
       <c r="A66" s="26" t="s">
         <v>187</v>
       </c>
@@ -18572,7 +19540,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="67" spans="1:33" hidden="1" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:33" hidden="1" x14ac:dyDescent="0.35">
       <c r="A67" s="31" t="s">
         <v>190</v>
       </c>
@@ -18580,7 +19548,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="68" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:33" x14ac:dyDescent="0.35">
       <c r="A68" s="26" t="s">
         <v>194</v>
       </c>
@@ -18678,7 +19646,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="69" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:33" x14ac:dyDescent="0.35">
       <c r="A69" s="47" t="s">
         <v>197</v>
       </c>
@@ -18776,7 +19744,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="70" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:33" x14ac:dyDescent="0.35">
       <c r="A70" s="26" t="s">
         <v>200</v>
       </c>
@@ -18874,7 +19842,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="71" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:33" x14ac:dyDescent="0.35">
       <c r="A71" s="26" t="s">
         <v>204</v>
       </c>
@@ -18972,7 +19940,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="72" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:33" x14ac:dyDescent="0.35">
       <c r="A72" s="26" t="s">
         <v>206</v>
       </c>
@@ -19070,7 +20038,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="73" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:33" x14ac:dyDescent="0.35">
       <c r="A73" s="26" t="s">
         <v>209</v>
       </c>
@@ -19168,7 +20136,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="74" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:33" x14ac:dyDescent="0.35">
       <c r="A74" s="26" t="s">
         <v>212</v>
       </c>
@@ -19266,7 +20234,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="75" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:33" x14ac:dyDescent="0.35">
       <c r="A75" s="47" t="s">
         <v>215</v>
       </c>
@@ -19361,7 +20329,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="77" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:33" x14ac:dyDescent="0.35">
       <c r="A77" t="s">
         <v>274</v>
       </c>
@@ -19487,7 +20455,7 @@
         <v>0.36666666666666664</v>
       </c>
     </row>
-    <row r="78" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:33" x14ac:dyDescent="0.35">
       <c r="A78" t="s">
         <v>373</v>
       </c>
@@ -19613,7 +20581,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="79" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:33" x14ac:dyDescent="0.35">
       <c r="A79" t="s">
         <v>278</v>
       </c>
@@ -19634,7 +20602,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="80" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:33" x14ac:dyDescent="0.35">
       <c r="A80" t="s">
         <v>374</v>
       </c>

</xml_diff>